<commit_message>
Update jobs directory data (auto-push)
</commit_message>
<xml_diff>
--- a/src/jobs/jobs.xlsx
+++ b/src/jobs/jobs.xlsx
@@ -641,19 +641,36 @@
           <t>Implement Climate Change Risk Management Policy and develop frameworks that align with organizational goals and objectives.
 Identification of climate risk at portfolio level/account level, and to identify and prioritize customer/sector segments for assessing climate related risks.
 Conduct comprehensive assessment of the Banks exposure to climate change-related financial risks (Physical &amp; Transition), including potential impacts on assets, operations and supply chain.
-Calculation of carbon footpr</t>
+Calculation of carbon footprint in lending portfolio at portfolio level/account level and monitor periodical emissions data, reporting.
+To prepare data inputs and execute various climate scenarios and stress testing cases. Integrate Climate Stress Testing with Credit and market risk stress testing.
+Required to conduct primary and secondary research on Regulatory (RBI, SEBI, BASEL etc.) guidelines or globally accepted standards (such as TCFD, GRI, SBTi etc.) on Net zero strategy, Climate Change Risk Management and to prepare Climate-related disclosures etc.
+Ensure compliance with regulatory requirements related to Climate change risks, including disclosures and reporting requirements.
+To provide climate change risk related training/ workshops</t>
         </is>
       </c>
       <c r="P2" s="6" t="inlineStr">
         <is>
           <t>Work Experience in Risk Management Cycle - with expertise in Climate Change Risk Management.
 Identification/Assessment/Measurement/Metrics and Disclosures and Risk Mitigation Strategies, Stress Testing - creation, execution and analysis of stress testing outcome.
-Experience in Climate Change Risk As</t>
+Experience in Climate Change Risk Assessment &amp; measurement, Sustainability strategy, Climate Finance, Green finance, clean energy and ESG related areas.
+Working Knowledge on Climate Risk Models, like Integrated Assessment Models (IAMs) or Climate physical and transition risk assessment tools by various service providers, such as Global Change Assessment Model (GCAM) and Paris Agreement Capital Transition Assessment (PACTA) etc.
+Expertise in Model development/ validation/ audit/ review experience for financial and non-financial risks.
+Experience of working on Stress test models (ex- for Transition and Physical Risk, Integration of credit risk in climate scenario etc.) etc.
+Having hands on knowledge on NGFS (Network for Greening the Financial System) and other climate scenarios.
+Proficiency in Climate Scenario Analysis and Stress testing.
+Hands on experience in calculating financed emissions and reporting
+Having working knowledge on frameworks such as SBTi, PCAF, GRI, BRSR etc.
+Effective written and verbal communication skills
+Excellent Communication Skills
+Problem Solving Attitude
+Analytical Thinking
+Excellent data analytical skills and comfortable working with large datasets
+Excellent skills in MS office, especially in MS Excel and PowerPoint etc</t>
         </is>
       </c>
       <c r="Q2" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate change risk management, climate risk assessment, climate finance, and green finance, which are all related to climate risk. The job requires experience in climate change risk management and knowledge of climate risk models, which further supports t</t>
+          <t>The job description mentions climate change risk management, climate risk assessment, climate finance, and green finance, which are all related to climate risk. The job requires experience in climate change risk management and knowledge of climate risk models, which further supports the classification as climate_risk.</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr"/>
@@ -736,7 +753,7 @@
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Climate Risk Assessment: Conduct physical risk assessments, transition risk assessments, and climate-related opportunities assessments for clients across various sectors. Develop models to compute financial impacts of climate related risks and opportunities Climate scenario analysis using IPCC, IEA, and NGFS scenarios to inform client strategies. Provide recommendations on climate risk management and resilience strategies. Nature and Biodiversity Risk Assessment: Conduct nature and biodiversity </t>
+          <t>Climate Risk Assessment: Conduct physical risk assessments, transition risk assessments, and climate-related opportunities assessments for clients across various sectors. Develop models to compute financial impacts of climate related risks and opportunities Climate scenario analysis using IPCC, IEA, and NGFS scenarios to inform client strategies. Provide recommendations on climate risk management and resilience strategies. Nature and Biodiversity Risk Assessment: Conduct nature and biodiversity risk assessments for clients, identifying potential impacts on their operations and supply chains. Develop strategies to mitigate nature and biodiversity risks and capitalize on opportunities. Climate Transition Planning: Develop climate transition plans, aligning with global climate goals and standards. Provide recommendations on climate policy, regulation, and market trends. Climate Resilience Strategy Development: Support clients in developing climate resilience strategies, including climate adaptation and disaster risk reduction measures. Conduct vulnerability assessments and provide recommendations for climate-resilient infrastructure and operations. Climate Finance: Advise clients on climate finance opportunities, including green bonds, climate-themed funds, and impact investing. Develop business cases and models to support climate-related investments. Reporting and Disclosure: Support clients in preparing reports aligned with TCFD, IFRS S1, IFRS S2, TNFD, ESRS etc.</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -746,7 +763,7 @@
       </c>
       <c r="Q3" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate risk assessment, physical risk assessments, transition risk assessments, climate scenario analysis, and climate resilience strategy development, which are all key aspects of climate risk management.</t>
+          <t>The job description mentions climate risk assessment, physical risk assessments, transition risk assessments, climate scenario analysis, and climate resilience strategy development, which are all key aspects of climate risk management.</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -829,17 +846,17 @@
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Work as part of a multidisciplinary team across a range of industries, assisting organisations on how they manage and report on a broad range of sustainability and climate-related risks and impacts. Delivery of assurance of non-financial reporting, including sustainability metrics, emissions and energy reporting across a range of industry sectors. Advise clients on the development of their strategies and delivery of non-financial reporting, including sustainability metrics, emissions and energy </t>
+          <t>Work as part of a multidisciplinary team across a range of industries, assisting organisations on how they manage and report on a broad range of sustainability and climate-related risks and impacts. Delivery of assurance of non-financial reporting, including sustainability metrics, emissions and energy reporting across a range of industry sectors. Advise clients on the development of their strategies and delivery of non-financial reporting, including sustainability metrics, emissions and energy reporting across a range of industry sectors. Contribute to strategy, solutions, methodologies, analytical frameworks and tools to help clients succeed and navigate complex regulatory environments and manage stakeholder expectations. Assist clients to develop and implement sustainability strategies, develop targets, and implement plans to enhance sustainability value for a broad range of sustainability topics, including diversity, waste, modern slavery and environmental impacts. Assist in climate scenario analysis including understanding climate risks and opportunities, in order to formulate short- and long-term management objectives.</t>
         </is>
       </c>
       <c r="P4" s="6" t="inlineStr">
         <is>
-          <t>Climate and nature disclosure experience, including knowledge of the Taskforce on Climate-related Financial Disclosure (TCFD) and Taskforce on Nature-related Financial Disclosure (TNFD) Frameworks. Knowledge of, and experience in decarbonisation approaches, climate risk and climate strategy. Agility</t>
+          <t>Climate and nature disclosure experience, including knowledge of the Taskforce on Climate-related Financial Disclosure (TCFD) and Taskforce on Nature-related Financial Disclosure (TNFD) Frameworks. Knowledge of, and experience in decarbonisation approaches, climate risk and climate strategy. Agility to learn and adapt on the job, ask the right questions and strive for the best solutions for clients.</t>
         </is>
       </c>
       <c r="Q4" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate change, climate risk, decarbonisation, GHG accounting, and climate scenario analysis, which are all relevant to the climate risk profile.</t>
+          <t>The job description mentions climate change, climate risk, decarbonisation, GHG accounting, and climate scenario analysis, which are all relevant to the climate risk profile.</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -926,17 +943,17 @@
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>Work as part of a multidisciplinary team across a range of industries, assisting organisations on how they manage and report on a broad range of sustainability and climate-related risks and impacts. Manage engagement teams and provide coaching and development advice to staff members. Coordinate project activities and build strong lines of communication with clients, engagement teams and senior leaders to ensure engagements are managed to clearly defined timelines while delivering high quality wo</t>
+          <t>Work as part of a multidisciplinary team across a range of industries, assisting organisations on how they manage and report on a broad range of sustainability and climate-related risks and impacts. Manage engagement teams and provide coaching and development advice to staff members. Coordinate project activities and build strong lines of communication with clients, engagement teams and senior leaders to ensure engagements are managed to clearly defined timelines while delivering high quality work products. Delivery of assurance of non-financial reporting, including sustainability metrics, emissions and energy reporting across a range of industry sectors. Advise clients on the development of their strategies and delivery of non-financial reporting, including sustainability metrics, emissions and energy reporting across a range of industry sectors. Contribute to strategy, solutions, methodologies, analytical frameworks and tools to help clients succeed and navigate complex regulatory environments and manage stakeholder expectations. Assist clients to develop and implement sustainability strategies, develop targets, and implement plans to enhance sustainability value for a broad range of sustainability topics, including diversity, waste, modern slavery and environmental impacts. Assist in climate scenario analysis including understanding climate risks and opportunities, in order to formulate short- and long-term management objectives.</t>
         </is>
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Professional services/consulting experience, Tertiary qualification in a quantitative subject, Experience in climate change services, Experience in GHG accounting, Demonstrable experience in reporting and/or assurance of greenhouse gas emissions, Working knowledge of the climate reporting regime in </t>
+          <t>Professional services/consulting experience, Tertiary qualification in a quantitative subject, Experience in climate change services, Experience in GHG accounting, Demonstrable experience in reporting and/or assurance of greenhouse gas emissions, Working knowledge of the climate reporting regime in New Zealand, Awareness of the Australian Accounting Standard Board S2 standard requirements, Experience leading teams and coaching and developing team members, Climate and nature disclosure experience, Knowledge of, and experience in decarbonisation approaches, climate risk and climate strategy</t>
         </is>
       </c>
       <c r="Q5" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate change services, GHG accounting, climate risk, decarbonisation approaches, and climate strategy, which are all relevant to the climate risk profile.</t>
+          <t>The job description mentions climate change services, GHG accounting, climate risk, decarbonisation approaches, and climate strategy, which are all relevant to the climate risk profile.</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -1015,7 +1032,7 @@
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
-          <t>Develop financing strategies for renewable energy, carbon reduction, and other climate-focused initiatives. Advise on ESG investment opportunities and impact funding. Secure funding through green bonds, sustainability-linked loans, carbon credit financing, and other instruments. Engage with banks, financial institutions, impact investors, and government agencies to unlock climate finance. Structure innovative financing models such as blended finance, PPPs (Public-Private Partnerships), and risk-</t>
+          <t>Develop financing strategies for renewable energy, carbon reduction, and other climate-focused initiatives. Advise on ESG investment opportunities and impact funding. Secure funding through green bonds, sustainability-linked loans, carbon credit financing, and other instruments. Engage with banks, financial institutions, impact investors, and government agencies to unlock climate finance. Structure innovative financing models such as blended finance, PPPs (Public-Private Partnerships), and risk-sharing mechanisms. Support fundraising through equity, debt, grants, and concessional finance. Ensure projects align with national and international climate policies, including Indias green finance framework. Stay updated on regulatory changes, carbon market trends, and sustainable investment guidelines. Conduct financial modeling, risk assessments, and return-on-investment analysis for sustainable projects. Evaluate the financial viability of Net Zero Indias sustainability initiatives. Collaborate with government bodies, financial institutions, corporate partners, and NGOs for sustainable funding solutions. Conduct workshops, training, and awareness programs on green finance opportunities.</t>
         </is>
       </c>
       <c r="P6" s="6" t="inlineStr">
@@ -1025,7 +1042,7 @@
       </c>
       <c r="Q6" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions sustainable finance, ESG investments, green bonds, and climate-focused fundraising, which are all key aspects of sustainable finance.</t>
+          <t>The job description mentions sustainable finance, ESG investments, green bonds, and climate-focused fundraising, which are all key aspects of sustainable finance.</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr"/>
@@ -1108,17 +1125,17 @@
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
-          <t>Lead end-to-end digital transformation and PMO for large capital projects in metals &amp; mining covering planning, execution, governance, and benefits realization. You will drive adoption of digital/AI solutions to deliver measurable improvements in time, cost, quality, and safety. Establish and run the PMO, build/maintain Integrated Master Schedule, implement Cost Controls, drive Risk &amp; Safety Management, oversee Quality Management, own procurement management, run performance reviews for contracto</t>
+          <t>Lead end-to-end digital transformation and PMO for large capital projects in metals &amp; mining covering planning, execution, governance, and benefits realization. You will drive adoption of digital/AI solutions to deliver measurable improvements in time, cost, quality, and safety. Establish and run the PMO, build/maintain Integrated Master Schedule, implement Cost Controls, drive Risk &amp; Safety Management, oversee Quality Management, own procurement management, run performance reviews for contractors and material vendors, implement Digital Storage &amp; Logistics Management, define the digital roadmap and success metrics, orchestrate adoption of digital solutions, ensure cybersecurity and data governance, act as client-facing lead for multi billion dollar programs, lead multi-disciplinary teams, manage benefits realization, and track KPIs tied to business case.</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>Program governance, PMO operations, EVM, schedule &amp; cost assurance, risk management, digital solutioning &amp; change management, stakeholder management, excellent communication, executive reporting, proposal support/pre sales, Digital-led Transformation &amp; Capital Project Management, Metals &amp; Mining, Ac</t>
+          <t>Program governance, PMO operations, EVM, schedule &amp; cost assurance, risk management, digital solutioning &amp; change management, stakeholder management, excellent communication, executive reporting, proposal support/pre sales, Digital-led Transformation &amp; Capital Project Management, Metals &amp; Mining, Accepting Feedback, Active Listening, Analytical Thinking, Carbon Accounting, Climate Change Adaptation Program Design, Climate Change Impacts and Risks, Climate Finance, Energy Efficiency, Energy Policy and Regulation, Energy Transition.</t>
         </is>
       </c>
       <c r="Q7" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions climate change mitigation and adaptation, energy efficiency, and renewable energy solutions, which are related to environmental sustainability and clean energy. Although it does not directly fit into the other categories, it is adjacent to clean e</t>
+          <t>The job description mentions climate change mitigation and adaptation, energy efficiency, and renewable energy solutions, which are related to environmental sustainability and clean energy. Although it does not directly fit into the other categories, it is adjacent to clean energy and has some relevance to environmental sustainability.</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -1201,17 +1218,17 @@
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Work as part of a multidisciplinary team across a range of industries, assisting organisations on how they manage and report on a broad range of sustainability and climate related risks and impacts. Assurance of non-financial reporting, including sustainability metrics, emissions and energy reporting across a range of industry sectors. Contribute to strategy, solutions, methodologies, analytical frameworks and tools to help clients succeed and navigate complex regulatory environments and manage </t>
+          <t>Work as part of a multidisciplinary team across a range of industries, assisting organisations on how they manage and report on a broad range of sustainability and climate related risks and impacts. Assurance of non-financial reporting, including sustainability metrics, emissions and energy reporting across a range of industry sectors. Contribute to strategy, solutions, methodologies, analytical frameworks and tools to help clients succeed and navigate complex regulatory environments and manage stakeholder expectations. Assist clients to develop and implement sustainability strategies, develop targets, and implement plans to enhance sustainability value for a broad range of sustainability topics, including diversity, waste, modern slavery and environmental impacts. Analyse effects of water, air quality and climate change towards organisations and communities, including ensuring integrity of environmental data as well as understanding climate risks and opportunities, in order to formulate short- and long-term management objectives</t>
         </is>
       </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>Professional services/consulting experience. Knowledge of relevant legislation, regulations and codes of practice as well as a good understanding of the climate-related issues. Practical experience with energy and emissions reporting schemes including National Greenhouse Emissions Reporting (NGER) s</t>
+          <t>Professional services/consulting experience. Knowledge of relevant legislation, regulations and codes of practice as well as a good understanding of the climate-related issues. Practical experience with energy and emissions reporting schemes including National Greenhouse Emissions Reporting (NGER) scheme, the Safeguard Mechanism and the Australian Carbon Credit Unit (ACCU) Scheme. Climate risk assessment and disclosure experience, including knowledge of the Taskforce on Climate-related Financial Disclosure (TCFD) Framework. Knowledge of key assurance standards including General Audit and Assurance Procedures (GAAP), International Sustainability Standards Board (ISSB) and the associated Australian Sustainability Reporting Standards (ASRS). Knowledge of, and experience in decarbonisation approaches, climate risk and climate strategy</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate change, climate risk, decarbonisation, and greenhouse gas emissions, which are all relevant to the climate risk profile. The role also involves working with clients to develop and implement sustainability strategies, and assisting them in navigatin</t>
+          <t>The job description mentions climate change, climate risk, decarbonisation, and greenhouse gas emissions, which are all relevant to the climate risk profile. The role also involves working with clients to develop and implement sustainability strategies, and assisting them in navigating complex regulatory environments, which further supports the climate risk profile classification</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -1294,17 +1311,17 @@
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
-          <t>Supporting the Manager/ SM in day-to-day delivery of ESG engagements and associated activities, while ensuring that the engagements are delivered in a manner that complies with internal and regulatory procedures, Being responsible for the quality of deliverables produced, including qualitative and quantitative analysis, Contributing to thought leadership and developing market intelligence to support ESG practice development, Proven abilities to establish and sustain sound relationships with clie</t>
+          <t>Supporting the Manager/ SM in day-to-day delivery of ESG engagements and associated activities, while ensuring that the engagements are delivered in a manner that complies with internal and regulatory procedures, Being responsible for the quality of deliverables produced, including qualitative and quantitative analysis, Contributing to thought leadership and developing market intelligence to support ESG practice development, Proven abilities to establish and sustain sound relationships with clients and other stakeholders, Demonstrated experience in engaging with new clients and managing client expectations, Highly experienced in managing, mentoring and guiding teams</t>
         </is>
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>Prior experience of undertaking ESG Gap Assessment and providing logical and impactful recommendations, Strong understanding of ESG processes and systems, Experience conducting climate risk assessment online with TCFD guidelines, Proven experience of undertaking a detailed Peer Review &amp; Benchmarking</t>
+          <t>Prior experience of undertaking ESG Gap Assessment and providing logical and impactful recommendations, Strong understanding of ESG processes and systems, Experience conducting climate risk assessment online with TCFD guidelines, Proven experience of undertaking a detailed Peer Review &amp; Benchmarking, Strong knowledge and experience in the field of Sustainability, Knowledge about Greenhouse Gas Accounting &amp; Inventorization (Scope-1,2,3), Familiar with Science based targets and decarbonization initiatives, Highly experienced in data governance – people, process, controls and technology aspects, Strong written and verbal communication skills</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[general_esg] The job description mentions ESG (Environmental, Social &amp; Governance) and sustainability, which are key aspects of general ESG profile. The job also involves climate risk assessment, greenhouse gas accounting, and decarbonization initiatives, which are all relevant to ESG strategy and </t>
+          <t>The job description mentions ESG (Environmental, Social &amp; Governance) and sustainability, which are key aspects of general ESG profile. The job also involves climate risk assessment, greenhouse gas accounting, and decarbonization initiatives, which are all relevant to ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -1387,7 +1404,7 @@
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
-          <t>Manage the implementation of advisory mandates, bespoke data and report deliveries of ISS ESG Climate Solutions. Conduct climate impact analysis on investment portfolios across all asset classes. Provide support and input for Client Calls based on deliverables requirements and effectively address client queries. Co-ordinate with required stakeholders to ensure timely delivery of high quality of data to the clients. Contribute to standardization and automation effort of bespoke analysis. Bring on</t>
+          <t>Manage the implementation of advisory mandates, bespoke data and report deliveries of ISS ESG Climate Solutions. Conduct climate impact analysis on investment portfolios across all asset classes. Provide support and input for Client Calls based on deliverables requirements and effectively address client queries. Co-ordinate with required stakeholders to ensure timely delivery of high quality of data to the clients. Contribute to standardization and automation effort of bespoke analysis. Bring on board ideas and implementation techniques to improve and streamline analysis and delivery of products especially for alternative asset classes.</t>
         </is>
       </c>
       <c r="P10" s="6" t="inlineStr">
@@ -1397,7 +1414,7 @@
       </c>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate-related risks, GHG emissions, and climate impact analysis, which are all relevant to the climate risk profile.</t>
+          <t>The job description mentions climate-related risks, GHG emissions, and climate impact analysis, which are all relevant to the climate risk profile.</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
@@ -1484,17 +1501,17 @@
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">In this crucial role, you’ll support the development of NatWest Markets’ sustainable finance and ESG risk capabilities across European capital markets. We’ll look to you to support senior originators in front‑line origination, risk engagement and client delivery by translating sustainability, climate and broader ESG themes into tangible financing, investment and risk outcomes. As a Financing &amp; Risk Solutions Associate, you will be supporting the effective management of transactions to make sure </t>
+          <t>In this crucial role, you’ll support the development of NatWest Markets’ sustainable finance and ESG risk capabilities across European capital markets. We’ll look to you to support senior originators in front‑line origination, risk engagement and client delivery by translating sustainability, climate and broader ESG themes into tangible financing, investment and risk outcomes. As a Financing &amp; Risk Solutions Associate, you will be supporting the effective management of transactions to make sure that all activities are in line with the bank’s policies covering conduct, operational, credit, and regulatory risks. You’ll contribute to the development of high‑quality sustainability‑linked client materials and regulatory‑aligned ESG assessments. You’ll also be assisting with client deep dives, navigating the sales coverage teams and gathering feedback from internal client touchpoints. Preparing pitch‑books, investor presentations, analysing market dynamics, identifying market trends, other marketing materials focusing on sustainability‑related analys. Producing client materials with focus on climate, ESG and regulatory developments shaping European capital markets. Tracking markets dynamics, including sustainable finance trends, evolving supervisory expectations and ESG‑related investor demand. Updating and maintaining internal databases and writing weekly market commentary for circulation to clients, including insights on transition and physical risk, regulatory disclosure regimes and ESG‑linked issuance activity. Supporting portfolio‑level ESG materiality and risk assessments in line with ECB and global supervisory expectations, contributing to audit‑ready, front‑line risk ownership</t>
         </is>
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>Comfort operating in evolving and complex sustainability‑related regulatory environments. Knowledge of investment banking and credit related products. Advanced power point and excel skills and experience with Pivots, vlookup, hlookup, index match and other advance excel formulas. Strong communicatio</t>
+          <t>Comfort operating in evolving and complex sustainability‑related regulatory environments. Knowledge of investment banking and credit related products. Advanced power point and excel skills and experience with Pivots, vlookup, hlookup, index match and other advance excel formulas. Strong communication and interpersonal skills with the ability to build relationship with key stakeholders including working with Risk, Compliance, Sustainability, SFA and Coverage teams. Excellent analytical and commercial awareness skills with high attention to detail, strong problem solving and logical thinking skills</t>
         </is>
       </c>
       <c r="Q11" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions sustainable finance, ESG risk, climate risk, and regulatory frameworks such as EU Taxonomy and CSRD, indicating a strong focus on sustainable finance and ESG topics.</t>
+          <t>The job description mentions sustainable finance, ESG risk, climate risk, and regulatory frameworks such as EU Taxonomy and CSRD, indicating a strong focus on sustainable finance and ESG topics.</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
@@ -1573,17 +1590,17 @@
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
-          <t>Work with global teams and clients to analyze sustainability data, delivering key insights that empower investors and decision-makers. Lead initiatives to elevate Apex Group s sustainability performance, supporting clients on their sustainability journey while enhancing the ESG reporting, analysis, and due diligence processes. Leverage extensive ESG expertise to provide high-quality advisory services in ESG policy and regulatory reporting, strategy, and risk management. Act as a key expert on on</t>
+          <t>Work with global teams and clients to analyze sustainability data, delivering key insights that empower investors and decision-makers. Lead initiatives to elevate Apex Group s sustainability performance, supporting clients on their sustainability journey while enhancing the ESG reporting, analysis, and due diligence processes. Leverage extensive ESG expertise to provide high-quality advisory services in ESG policy and regulatory reporting, strategy, and risk management. Act as a key expert on one or more of the following regulatory areas, interpreting complex regulations and integrating them into client value creation processes: Corporate Sustainability Due Diligence Directive (CSDDD); Corporate Sustainability Reporting Directive (CSRD); EU Deforestation Regulation (EUDR); EU Taxonomy; Minimum Safeguards; Sustainable Finance Disclosures Regulation (SFDR); and Taskforce on Nature-related Financial Disclosures (TNFD). Evaluate the material impact of biodiversity and ecosystems on businesses to identify associated risks and opportunities, helping clients manage their environmental impacts. Contribute to the continuous improvement of existing ESG products and the development of innovative solutions that meet client needs and regulatory demands.</t>
         </is>
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>Proficiency in quantitative and qualitative data collection, analysis, and reporting. Exceptional organizational competency with strong attention to detail. Excellent interpersonal skills with the ability to communicate and influence internal and external stakeholders, including proficiency in video</t>
+          <t>Proficiency in quantitative and qualitative data collection, analysis, and reporting. Exceptional organizational competency with strong attention to detail. Excellent interpersonal skills with the ability to communicate and influence internal and external stakeholders, including proficiency in video conferencing, written communication, and presentation. Proficiency in MS Office is needed, while knowledge of programming languages is a plus.</t>
         </is>
       </c>
       <c r="Q12" s="6" t="inlineStr">
         <is>
-          <t>[eu_taxonomy_sfdr] The job description mentions specific EU regulations such as EU Taxonomy, CSRD, and SFDR, which are key components of the EU Taxonomy and SFDR profile. The role also involves ESG reporting, analysis, and due diligence, which are closely related to the EU Taxonomy and SFDR regulati</t>
+          <t>The job description mentions specific EU regulations such as EU Taxonomy, CSRD, and SFDR, which are key components of the EU Taxonomy and SFDR profile. The role also involves ESG reporting, analysis, and due diligence, which are closely related to the EU Taxonomy and SFDR regulations.</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr"/>
@@ -1650,7 +1667,7 @@
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
-          <t>Develop and implement machine learning and deep learning models for satellite and geospatial data analysis. Integrate and process multimodal datasets. Build and automate scalable data processing pipelines using Python and cloud-based solutions. Collaborate with interdisciplinary teams and international partners to deliver customer-facing projects. Support the development of recommended practices and standards for EO data analytics. Present findings and recommendations to customers, supporting th</t>
+          <t>Develop and implement machine learning and deep learning models for satellite and geospatial data analysis. Integrate and process multimodal datasets. Build and automate scalable data processing pipelines using Python and cloud-based solutions. Collaborate with interdisciplinary teams and international partners to deliver customer-facing projects. Support the development of recommended practices and standards for EO data analytics. Present findings and recommendations to customers, supporting their digital transformation and compliance journeys. Contribute to proposal writing, research activities, and the expansion of DNV’s EO service portfolio.</t>
         </is>
       </c>
       <c r="P13" s="6" t="inlineStr">
@@ -1660,7 +1677,7 @@
       </c>
       <c r="Q13" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions working on sustainability, energy transition, and environmental challenges, which aligns with the clean energy adjacent profile. The role involves developing data-driven solutions for complex challenges in safety, sustainability, and energy transi</t>
+          <t>The job description mentions working on sustainability, energy transition, and environmental challenges, which aligns with the clean energy adjacent profile. The role involves developing data-driven solutions for complex challenges in safety, sustainability, and energy transition, and the company is involved in navigating the transition to a decarbonized and more sustainable energy future.</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr"/>
@@ -1744,12 +1761,12 @@
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>Civil &amp; Geological Engineering, Soil Mechanics or similar, Civil &amp; Geotechnical Engineering, MSc Soil Mechanics, Hydrogeology, Hydrogeologist, Civil Engineering in Environmental Science and MSc in Earth Science, Acoustics Engineering, Music Technology or Sound Engineering or other, Environmental and</t>
+          <t>Civil &amp; Geological Engineering, Soil Mechanics or similar, Civil &amp; Geotechnical Engineering, MSc Soil Mechanics, Hydrogeology, Hydrogeologist, Civil Engineering in Environmental Science and MSc in Earth Science, Acoustics Engineering, Music Technology or Sound Engineering or other, Environmental and Sustainability Engineering, Energy Engineering, Environmental Studies and similar</t>
         </is>
       </c>
       <c r="Q14" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions various environmental and sustainability-related roles such as Rock Engineering, Geotechnical Engineering, Hydrogeology, Contaminated Areas, Acoustics, and Environmental Management - Sustainability &amp; Climate Change, which are all related to enviro</t>
+          <t>The job description mentions various environmental and sustainability-related roles such as Rock Engineering, Geotechnical Engineering, Hydrogeology, Contaminated Areas, Acoustics, and Environmental Management - Sustainability &amp; Climate Change, which are all related to environmental science, conservation, and sustainability, making it a good fit for the clean_energy_adjacent profile</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
@@ -1836,17 +1853,17 @@
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>Disclosure requirements Interpretation and Integration: Act as the subject matter expert, interpret mandatory disclosure requirements under global ESG/ sustainability related standards. Develop a comprehensive Materiality Assessment Framework: Design and architect a robust Materiality Assessment framework that aligns seamlessly with the requirements of the amended ESRS. Maintain the DR Inventory: Define, update, and manage the disclosure requirement (DR) inventory, including ownership of each DR</t>
+          <t>Disclosure requirements Interpretation and Integration: Act as the subject matter expert, interpret mandatory disclosure requirements under global ESG/ sustainability related standards. Develop a comprehensive Materiality Assessment Framework: Design and architect a robust Materiality Assessment framework that aligns seamlessly with the requirements of the amended ESRS. Maintain the DR Inventory: Define, update, and manage the disclosure requirement (DR) inventory, including ownership of each DR and data point. Assess DR Applicability: Review and confirm the applicability of DRs for the current reporting year, including application of omission methodologies. Develop and Refine Reporting Processes: Develop and maintain efficient ESG reporting templates and processes. Prepare Report Drafts: Create preliminary report drafts and update with inputs from Information Providers and prepare for final submission. Continuous Monitoring: Establish mechanisms for ongoing monitoring of compliance effectiveness and identify potential new gaps arising from future regulatory updates or evolving business practices. Assurance Readiness: Prepare documentation and evidence to support internal and external audits and assurance activities related to sustainability related compliance and gap remediation. Benchmarking: Research and analyze best practices in sustainability related disclosures, gap remediation, and so on. Collaborate with Leads on Key Activities: Support leads in the following: Ensuring timely and accurate reporting of ESG disclosures through standardized and controlled processes. Developing and implementing disclosure controls and procedures for ESG disclosures. Managing the collection of attestations. Enhancing report design, branding, and visual elements (e.g., infographics). Engaging with and coordinating external assurance providers. Coordinating internal audits and external reviews. Preparing final reports for approval by relevant governance bodies. Contributing to other essential tasks as needed.</t>
         </is>
       </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>Proven ability to design, implement, and optimize financial controls; define and execute robust financial reporting; and an eye digitization/automation of manual processes to enhance controls and compliance drive efficiency through automation and digitization initiatives. Good understanding of ESG r</t>
+          <t>Proven ability to design, implement, and optimize financial controls; define and execute robust financial reporting; and an eye digitization/automation of manual processes to enhance controls and compliance drive efficiency through automation and digitization initiatives. Good understanding of ESG regulatory requirements, and global sustainability standards. Strong understanding of Banking/ FIs relevant reporting requirements. Assurance/ Audit experience preferred. Demonstrated analytical and critical thinking skills to dissect complex regulatory language and identify practical implications. Strong problem-solving abilities and a proactive approach to identifying and addressing compliance challenges. Demonstrated project management skills with the ability to lead cross-functional initiatives. High attention to detail and accuracy, ensuring meticulous gap identification and remediation. Superior written and verbal communication skills, capable of explaining complex regulatory concepts to diverse audiences. Ability to influence stakeholders and drive consensus on remediation strategies. Proficiency in using data analysis tools (e.g., Excel) and familiarity with ESG reporting software. Self-motivated, adaptable, and able to thrive in a fast-paced, evolving regulatory environment.</t>
         </is>
       </c>
       <c r="Q15" s="6" t="inlineStr">
         <is>
-          <t>[eu_taxonomy_sfdr] The job description mentions EU Corporate Sustainability Reporting Directive (CSRD), EU Taxonomy, and other ESG-related regulations, indicating a strong focus on EU Taxonomy and SFDR compliance.</t>
+          <t>The job description mentions EU Corporate Sustainability Reporting Directive (CSRD), EU Taxonomy, and other ESG-related regulations, indicating a strong focus on EU Taxonomy and SFDR compliance.</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
@@ -1929,7 +1946,7 @@
       </c>
       <c r="O16" s="6" t="inlineStr">
         <is>
-          <t>Working on sustainability in deals at PwC, you will focus on providing consulting services related to integrating sustainability principles into mergers and acquisitions and private equity transactions (debt and equity) and corporate strategies. You will analyse environmental and social risk, assess client needs based on global frameworks, conduct impact assessments and develop comprehensive sustainability strategies for value creation, and offer guidance and support to help clients transition t</t>
+          <t>Working on sustainability in deals at PwC, you will focus on providing consulting services related to integrating sustainability principles into mergers and acquisitions and private equity transactions (debt and equity) and corporate strategies. You will analyse environmental and social risk, assess client needs based on global frameworks, conduct impact assessments and develop comprehensive sustainability strategies for value creation, and offer guidance and support to help clients transition to sustainable and purpose-led business models.</t>
         </is>
       </c>
       <c r="P16" s="6" t="inlineStr">
@@ -1939,7 +1956,7 @@
       </c>
       <c r="Q16" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions integrating sustainability principles into mergers and acquisitions, private equity transactions, and corporate strategies, which is related to sustainable finance. It also mentions ESG ratings methodology, ESG policies, and ESG due diligences, whic</t>
+          <t>The job description mentions integrating sustainability principles into mergers and acquisitions, private equity transactions, and corporate strategies, which is related to sustainable finance. It also mentions ESG ratings methodology, ESG policies, and ESG due diligences, which are key aspects of sustainable finance.</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
@@ -2041,7 +2058,7 @@
       </c>
       <c r="Q17" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description explicitly mentions climate risk, climate-related risks, climate strategy development, and climate disclosure frameworks, which are all key aspects of climate risk assessment and management.</t>
+          <t>The job description explicitly mentions climate risk, climate-related risks, climate strategy development, and climate disclosure frameworks, which are all key aspects of climate risk assessment and management.</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -2128,7 +2145,9 @@
 * Support to senior team members on GHG inventories for corporates, cities, and sectors following IPCC Guidelines and GHG Protocol.
 * Develop and implement GHG calculation tools for baseline emissions and forecasting.
 * Use LCA tools to evaluate embodied carbon in infrastructure and master planning.
-* Support senior team member/lead on design and execution of decarbonization roadmaps with clear targets and timelines in line with SBTi and national climate goals</t>
+* Support senior team member/lead on design and execution of decarbonization roadmaps with clear targets and timelines in line with SBTi and national climate goals.
+* Apply PCAF guidelines for assessing financed, facilitated, or insurance-associated emissions (desirable).
+Climate Risk Modeling and Assessment</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2138,7 +2157,7 @@
       </c>
       <c r="Q18" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions GHG accounting, decarbonization, climate risk modeling, and assessment, which are all related to climate risk. The job also mentions following IPCC Guidelines and GHG Protocol, and applying PCAF guidelines, which are all relevant to climate risk management</t>
+          <t>The job description mentions GHG accounting, decarbonization, climate risk modeling, and assessment, which are all related to climate risk. The job also mentions following IPCC Guidelines and GHG Protocol, and applying PCAF guidelines, which are all relevant to climate risk management.</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
@@ -2227,7 +2246,7 @@
       </c>
       <c r="Q19" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate risk, GHG emissions, and Net Zero reports, which are key indicators of a climate risk profile.</t>
+          <t>The job description mentions climate risk, GHG emissions, and Net Zero reports, which are key indicators of a climate risk profile.</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr"/>
@@ -2383,17 +2402,17 @@
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
-          <t>Lead and manage all operational aspects of the Projects business, by setting up and overseeing key internal support functions (HR, IT, finance, and Business Services). Develop and implement fit-for-purpose systems, tools, and processes that enable the Projects team to operate with autonomy and efficiency, while maintaining alignment with corporate standards. Support the design and implementation of a capital investment framework to guide decision-making and capital allocation. Ensure alignment b</t>
+          <t>Lead and manage all operational aspects of the Projects business, by setting up and overseeing key internal support functions (HR, IT, finance, and Business Services). Develop and implement fit-for-purpose systems, tools, and processes that enable the Projects team to operate with autonomy and efficiency, while maintaining alignment with corporate standards. Support the design and implementation of a capital investment framework to guide decision-making and capital allocation. Ensure alignment between Projects team operations and broader corporate frameworks and standards. Prepare high-quality materials for Board and committee reporting, ensuring clarity, accuracy and timeliness. Lead and coordinate project development workstreams, ensuring clear ownership, timelines and accountability across internal teams and external partners. Establish and manage project governance cadence, including setting agendas, facilitating meetings, tracking actions and driving timely decision-making. Maintain integrated project plans, monitoring progress against milestones, budgets and risks, and escalating issues as required. Oversee governance processes to support disciplined project progression and investment approvals. Partner with Corporate Finance on budgeting, forecasting and resource planning. Develop and track KPIs, identifying performance trends and driving continuous improvement. Work closely with the executive team to align operational delivery with business priorities. Ensure compliance with legal, regulatory and internal standards. Identify and manage operational risks across the project lifecycle. Manage key vendor and service provider relationships, including contract negotiation and performance oversight. Foster a high-performance, accountable and collaborative team environment. Support capability development within the Projects team and broader organisation.</t>
         </is>
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>Proficiency with CRMs, MS Office, and advanced Excel skills. Experience managing virtual data rooms. Strong financial acumen and experience with budgeting and forecasting. Excellent leadership, communication, and interpersonal skills. Strong analytical and problem-solving skills. Pragmatic, solution</t>
+          <t>Proficiency with CRMs, MS Office, and advanced Excel skills. Experience managing virtual data rooms. Strong financial acumen and experience with budgeting and forecasting. Excellent leadership, communication, and interpersonal skills. Strong analytical and problem-solving skills. Pragmatic, solutions-oriented, and comfortable operating in ambiguity. Effective communication and stakeholder engagement. Ability to manage multiple projects simultaneously.</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions experience in renewable energy, decarbonisation, infrastructure or nature-based projects as highly desirable, and the company is a specialist climate change investment and advisory firm, indicating a strong focus on environmental sustainability an</t>
+          <t>The job description mentions experience in renewable energy, decarbonisation, infrastructure or nature-based projects as highly desirable, and the company is a specialist climate change investment and advisory firm, indicating a strong focus on environmental sustainability and clean energy.</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
@@ -2476,17 +2495,17 @@
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop relationships with corporate buyers, airlines, traders, intermediaries and financial institutions active in carbon markets. Manage the full commercial lifecycle, from lead generation and client engagement through to transaction execution. Originate and execute transactions across voluntary carbon markets, CORSIA-eligible credits and emerging compliance-linked carbon markets. Identify new commercial opportunities and areas of the market where CFP Energy should focus its efforts, based on </t>
+          <t>Develop relationships with corporate buyers, airlines, traders, intermediaries and financial institutions active in carbon markets. Manage the full commercial lifecycle, from lead generation and client engagement through to transaction execution. Originate and execute transactions across voluntary carbon markets, CORSIA-eligible credits and emerging compliance-linked carbon markets. Identify new commercial opportunities and areas of the market where CFP Energy should focus its efforts, based on evolving regulation and market demand. Support the structuring and negotiation of commercial transactions, including carbon credit offtake agreements, forward purchases and other structured environmental market products. Work closely with internal trading teams to develop pricing strategies and execute transactions. Track market developments, pricing dynamics and supply-demand trends to support commercial strategy and client discussions. Build relationships with project developers, carbon funds and intermediaries to source high-quality carbon credit supply. Evaluate projects across different methodologies, standards and geographies. Support commercial due diligence and maintain awareness of project pipelines.</t>
         </is>
       </c>
       <c r="P22" s="6" t="inlineStr">
         <is>
-          <t>Strong market instincts, entrepreneurial mindset, confidence to build and leverage relationships, ability to structure and execute carbon credit transactions, experience with commercial negotiation, origination or structured transactions, strong understanding of carbon credit project structures, met</t>
+          <t>Strong market instincts, entrepreneurial mindset, confidence to build and leverage relationships, ability to structure and execute carbon credit transactions, experience with commercial negotiation, origination or structured transactions, strong understanding of carbon credit project structures, methodologies and market dynamics</t>
         </is>
       </c>
       <c r="Q22" s="6" t="inlineStr">
         <is>
-          <t>[carbon_markets] The job description mentions voluntary carbon markets, carbon credits, CORSIA, and compliance-linked carbon markets, which are all related to carbon markets. The role involves originating and executing transactions across voluntary carbon markets, and the ideal candidate should have</t>
+          <t>The job description mentions voluntary carbon markets, carbon credits, CORSIA, and compliance-linked carbon markets, which are all related to carbon markets. The role involves originating and executing transactions across voluntary carbon markets, and the ideal candidate should have experience in carbon markets, environmental commodities, energy trading, or a related field.</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
@@ -2569,7 +2588,7 @@
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
-          <t>The PhD candidate tasks will include: organizing logistics for regular river sampling by local teams: shipment of materials and samples, establish new collaborations with other partners in the Congo Basin. organizing and conducting new sampling campaigns in collaboration with local partners in the Congo Basin field measurements of river discharge, physico-chemical parameters and greenhouse gas concentrations and fluxes field sampling for a wide range of biogeochemical proxies, sample preservatio</t>
+          <t>The PhD candidate tasks will include: organizing logistics for regular river sampling by local teams: shipment of materials and samples, establish new collaborations with other partners in the Congo Basin. organizing and conducting new sampling campaigns in collaboration with local partners in the Congo Basin field measurements of river discharge, physico-chemical parameters and greenhouse gas concentrations and fluxes field sampling for a wide range of biogeochemical proxies, sample preservation for analyses in Belgium. laboratory analysis of samples (quantification and stable isotope analyses of diffferent carbon pools, nutrient analyses and greenhouse gas analysis, …) dissemination of results at scientific conferences and in interational, peer-reviewed journals. you will be expected to contribute to educational tasks depending on opportunities and your own interests, and assist in coaching MSc thesis students. opportunitities exist to make your own contribution to the research objectives depending on personal interests and in collaboration with other research teams.</t>
         </is>
       </c>
       <c r="P23" s="6" t="inlineStr">
@@ -2579,7 +2598,7 @@
       </c>
       <c r="Q23" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions research on riverine carbon dynamics and fluxes in the Congo Basin, which is related to environmental science and the management of natural resources, fitting the clean_energy_adjacent profile.</t>
+          <t>The job description mentions research on riverine carbon dynamics and fluxes in the Congo Basin, which is related to environmental science and the management of natural resources, fitting the clean_energy_adjacent profile.</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
@@ -2663,12 +2682,12 @@
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>Excellent communication skills, with the ability to articulate complex issues clearly and persuasively in both written and spoken English. A wellestablished professional network in EU affairs and climaterelated policy fields. Demonstrated ability to design and deliver complex strategies that mobilis</t>
+          <t>Excellent communication skills, with the ability to articulate complex issues clearly and persuasively in both written and spoken English. A wellestablished professional network in EU affairs and climaterelated policy fields. Demonstrated ability to design and deliver complex strategies that mobilise diverse actors toward shared outcomes.</t>
         </is>
       </c>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate change, netzero economy, greenhouse gas emissions reductions, and climate policy, which are all relevant to climate risk.</t>
+          <t>The job description mentions climate change, netzero economy, greenhouse gas emissions reductions, and climate policy, which are all relevant to climate risk.</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr"/>
@@ -2748,7 +2767,9 @@
 Advise and collaborate across businesses and global functions to drive common objectives
 Follow human rights developments, societal trends and best practices, and translate them into actionable improvements
 Strengthen risk management, social performance and value creation through robust social responsibility work
-Ensure the continuous development, motivation and professiona</t>
+Ensure the continuous development, motivation and professional competence of the Social Responsibility team
+Represent UPM in company-level CSR initiatives and collaboration with key stakeholders
+Contribute to wider Group-level activities such as responsible sourcing, HR, investment management, compliance and internal audit</t>
         </is>
       </c>
       <c r="P25" s="6" t="inlineStr">
@@ -2762,7 +2783,7 @@
       </c>
       <c r="Q25" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions social responsibility, sustainability, human rights, and responsible sourcing, which are all relevant to ESG strategy and corporate sustainability.</t>
+          <t>The job description mentions social responsibility, sustainability, human rights, and responsible sourcing, which are all relevant to ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr"/>
@@ -2841,7 +2862,7 @@
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
-          <t>The first project will focus on a VM0047 afforestation project, but the role will extend to supporting additional projects across Arbonics portfolio. This is a hybrid role combining technical carbon project development and stakeholder collaboration. In addition to leading the research and preparation of PDD documentation, you will support commercial teams in evaluating and acquiring new commercial opportunities. You will become the technical expert representing Arbonics in discussions with lando</t>
+          <t>The first project will focus on a VM0047 afforestation project, but the role will extend to supporting additional projects across Arbonics portfolio. This is a hybrid role combining technical carbon project development and stakeholder collaboration. In addition to leading the research and preparation of PDD documentation, you will support commercial teams in evaluating and acquiring new commercial opportunities. You will become the technical expert representing Arbonics in discussions with landowners, partners, and project stakeholders, helping answer detailed questions about project eligibility, methodology requirements, and carbon accounting. Key Responsibilities: Carbon project development, Technical expertise in project development, Stakeholder engagement</t>
         </is>
       </c>
       <c r="P26" s="6" t="inlineStr">
@@ -2851,7 +2872,7 @@
       </c>
       <c r="Q26" s="6" t="inlineStr">
         <is>
-          <t>[carbon_markets] The job description mentions carbon project development, Verra VCS methodologies, and carbon credits, which are all related to carbon markets.</t>
+          <t>The job description mentions carbon project development, Verra VCS methodologies, and carbon credits, which are all related to carbon markets.</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
@@ -2934,7 +2955,7 @@
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">We are looking for a Customer Solutions Engineer to take ownership of the technical success of our enterprise banking clients. This is a high-impact, remote consultancy engagement within Europe, requiring availability within ±1 hour CET. In this role, you will work closely with the CPTO and the Customer team, acting as the primary technical counterpart for global banks operating in highly regulated environments. You will stand at the intersection of product, engineering, and enterprise clients, </t>
+          <t>We are looking for a Customer Solutions Engineer to take ownership of the technical success of our enterprise banking clients. This is a high-impact, remote consultancy engagement within Europe, requiring availability within ±1 hour CET. In this role, you will work closely with the CPTO and the Customer team, acting as the primary technical counterpart for global banks operating in highly regulated environments. You will stand at the intersection of product, engineering, and enterprise clients, shaping how our platform scales, integrates, and delivers long-term value.</t>
         </is>
       </c>
       <c r="P27" s="6" t="inlineStr">
@@ -2944,7 +2965,7 @@
       </c>
       <c r="Q27" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'impact technology', 'driving global climate action', 'ESG experts', and 'sustainability' in the context of financial products, indicating a strong focus on sustainable finance and ESG investing.</t>
+          <t>The job description mentions 'impact technology', 'driving global climate action', 'ESG experts', and 'sustainability' in the context of financial products, indicating a strong focus on sustainable finance and ESG investing.</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
@@ -3037,7 +3058,7 @@
       </c>
       <c r="Q28" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions ESG, sustainability, climate change risk assessments, and social and human rights impact assessments, which are all related to environmental, social, and governance topics.</t>
+          <t>The job description mentions ESG, sustainability, climate change risk assessments, and social and human rights impact assessments, which are all related to environmental, social, and governance topics.</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
@@ -3116,17 +3137,17 @@
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
-          <t>support the development of NatWest Markets sustainable finance and ESG risk capabilities across European capital markets, support senior originators in frontline origination, risk engagement and client delivery, contribute to the development of high-quality sustainability-linked client materials and regulatory-aligned ESG assessments, assist with client deep dives, navigate the sales coverage teams and gather feedback from internal client touchpoints, prepare pitch-books, investor presentations,</t>
+          <t>support the development of NatWest Markets sustainable finance and ESG risk capabilities across European capital markets, support senior originators in frontline origination, risk engagement and client delivery, contribute to the development of high-quality sustainability-linked client materials and regulatory-aligned ESG assessments, assist with client deep dives, navigate the sales coverage teams and gather feedback from internal client touchpoints, prepare pitch-books, investor presentations, analyze market dynamics, identify market trends, produce client materials with focus on climate, ESG and regulatory developments, track markets dynamics, update and maintain internal databases, write weekly market commentary, support portfolio-level ESG materiality and risk assessments</t>
         </is>
       </c>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>sustainability and ESG risk, knowledge of various debt products and markets, comfort operating in evolving and complex sustainability-related regulatory environments, knowledge of investment banking and credit related products, advanced power point and excel skills, strong communication and interper</t>
+          <t>sustainability and ESG risk, knowledge of various debt products and markets, comfort operating in evolving and complex sustainability-related regulatory environments, knowledge of investment banking and credit related products, advanced power point and excel skills, strong communication and interpersonal skills, excellent analytical and commercial awareness skills</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions sustainable finance, ESG risk, climate-related financial risk, and European sustainability regulatory frameworks, indicating a strong focus on sustainable finance and ESG topics.</t>
+          <t>The job description mentions sustainable finance, ESG risk, climate-related financial risk, and European sustainability regulatory frameworks, indicating a strong focus on sustainable finance and ESG topics.</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr"/>
@@ -3270,7 +3291,7 @@
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deloitte Audit &amp; Assurance - Talent Program Revisore Junior (0 - 1 anno di Esperienza). Le nostre altre attività di supporto sono: revisione di bilanci IAS/IFRS OIC e di reporting package, progetti di First Time Adoption (FTA) ovvero transizione dai principi contabili nazionali a principi contabili internazionali, verifica delle dichiarazioni (ad esempio 770), attestazioni delle ricerche e sviluppo. In quanto Analyst avrai la possibilità di imparare da colleghe e colleghi più Senior (attraverso </t>
+          <t>Deloitte Audit &amp; Assurance - Talent Program Revisore Junior (0 - 1 anno di Esperienza). Le nostre altre attività di supporto sono: revisione di bilanci IAS/IFRS OIC e di reporting package, progetti di First Time Adoption (FTA) ovvero transizione dai principi contabili nazionali a principi contabili internazionali, verifica delle dichiarazioni (ad esempio 770), attestazioni delle ricerche e sviluppo. In quanto Analyst avrai la possibilità di imparare da colleghe e colleghi più Senior (attraverso il learning on the job) e sviluppare competenze tecniche e relazionali.</t>
         </is>
       </c>
       <c r="P31" s="6" t="inlineStr">
@@ -3280,7 +3301,7 @@
       </c>
       <c r="Q31" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] La menzione di strategie di Corporate Sustainability, ESG e sostenibilità ambientale, sociale e di governance all'interno della descrizione dell'azienda e del ruolo</t>
+          <t>La menzione di strategie di Corporate Sustainability, ESG e sostenibilità ambientale, sociale e di governance all'interno della descrizione dell'azienda e del ruolo</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr"/>
@@ -3357,7 +3378,7 @@
       </c>
       <c r="Q32" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions working with renewable energy sources (solar, hydro, and wind), low carbon energies, and contributing to the objective of Carbon Neutrality by 2050, which are all related to environmental sustainability and the clean energy sector.</t>
+          <t>The job description mentions working with renewable energy sources (solar, hydro, and wind), low carbon energies, and contributing to the objective of Carbon Neutrality by 2050, which are all related to environmental sustainability and the clean energy sector.</t>
         </is>
       </c>
       <c r="R32" s="2" t="inlineStr"/>
@@ -3436,7 +3457,7 @@
       </c>
       <c r="O33" s="6" t="inlineStr">
         <is>
-          <t>Deliver mandatory sustainability reporting services, including process development and audit readiness across carbon footprint measurement, climate risk assessments, scenario analysis, and preparation of sustainability disclosures. Provide tailored advice on sustainability and climate-related financial reporting across sectors, aligned with evolving standards and frameworks. Deliver expert advice on IFRS, AASB, and Australian Sustainability Reporting Standards. Support the CFO Advisory team with</t>
+          <t>Deliver mandatory sustainability reporting services, including process development and audit readiness across carbon footprint measurement, climate risk assessments, scenario analysis, and preparation of sustainability disclosures. Provide tailored advice on sustainability and climate-related financial reporting across sectors, aligned with evolving standards and frameworks. Deliver expert advice on IFRS, AASB, and Australian Sustainability Reporting Standards. Support the CFO Advisory team with technical accounting aspects of projects. Support and mentor junior team members. Contribute to proposal development, training, and coaching.</t>
         </is>
       </c>
       <c r="P33" s="6" t="inlineStr">
@@ -3446,7 +3467,7 @@
       </c>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate risk assessments, scenario analysis, and sustainability reporting, which are key aspects of climate risk management. The role also involves providing advice on sustainability and climate-related financial reporting, which is a critical component of</t>
+          <t>The job description mentions climate risk assessments, scenario analysis, and sustainability reporting, which are key aspects of climate risk management. The role also involves providing advice on sustainability and climate-related financial reporting, which is a critical component of climate risk management.</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr">
@@ -3525,7 +3546,7 @@
       </c>
       <c r="O34" s="6" t="inlineStr">
         <is>
-          <t>Serve as an ESG data expert for a broad universe of global companies, understand and further their expertise on Morningstar indexes’ sustainability product offerings, including methodology criteria and data needs, work closely with multiple global teams across various functions to ensure that indexes team gets the required data in time to support the product roadmap, stay up to date with developments in sustainable, environmental, and social activities, including current and emerging trends, dri</t>
+          <t>Serve as an ESG data expert for a broad universe of global companies, understand and further their expertise on Morningstar indexes’ sustainability product offerings, including methodology criteria and data needs, work closely with multiple global teams across various functions to ensure that indexes team gets the required data in time to support the product roadmap, stay up to date with developments in sustainable, environmental, and social activities, including current and emerging trends, drivers, key players, best practices, the regulatory landscape, etc., ensure appropriate methods and techniques to improve and maintain the highest quality standards in the data collected/ingested by the team, develop indexes ESG dashboards and metrics, provides coaching and training to junior team members as appropriate and according to the specific needs of the person and the group, provide floor support by answering questions, solving issues that come up throughout the day, work with technology teams in the role of UAT/Business Owner to complete the design of ESG data ingestion processes and tools.</t>
         </is>
       </c>
       <c r="P34" s="6" t="inlineStr">
@@ -3535,7 +3556,7 @@
       </c>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>[esg] The job description mentions ESG data expertise, EU taxonomy, climate risk, and sustainable investing, which are all relevant to the ESG profile.</t>
+          <t>The job description mentions ESG data expertise, EU taxonomy, climate risk, and sustainable investing, which are all relevant to the ESG profile.</t>
         </is>
       </c>
       <c r="R34" s="2" t="inlineStr">
@@ -3614,7 +3635,7 @@
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
-          <t>Process and analyze geospatial data to contribute to the development of Swiss Re products and solutions, Develop and maintain scripts and pipelines to automate data processing and standardize workflows, Work closely with diverse teams across Swiss Re, providing geo-domain expertise, technical guidance, and support, Drive small projects independently, Coordinate and communicate effectively with other teams and stakeholders, provide regular project status updates, and ensure comprehensive and up-t</t>
+          <t>Process and analyze geospatial data to contribute to the development of Swiss Re products and solutions, Develop and maintain scripts and pipelines to automate data processing and standardize workflows, Work closely with diverse teams across Swiss Re, providing geo-domain expertise, technical guidance, and support, Drive small projects independently, Coordinate and communicate effectively with other teams and stakeholders, provide regular project status updates, and ensure comprehensive and up-to-date project documentation, Proactively identify, report, and resolve any issues or conflicts that may arise within the team or project, Foster a collaborative and positive team environment, Scout for new ideas and development for positive outcomes</t>
         </is>
       </c>
       <c r="P35" s="6" t="inlineStr">
@@ -3624,7 +3645,7 @@
       </c>
       <c r="Q35" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions natural catastrophes, climate change, and geospatial risk assessment, which are all relevant to climate risk, The company is also working to make the world more resilient, which implies a focus on managing and mitigating climate-related risks</t>
+          <t>The job description mentions natural catastrophes, climate change, and geospatial risk assessment, which are all relevant to climate risk, The company is also working to make the world more resilient, which implies a focus on managing and mitigating climate-related risks</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr"/>
@@ -3691,7 +3712,7 @@
       </c>
       <c r="O36" s="6" t="inlineStr">
         <is>
-          <t>The E T Consultant’s will support implementation of GPNBS programming. Tasks include coordinating and leading operational expert support on NBS to Task Teams and clients under the Operations pillar of the Program (advice on technical studies for project design and implementation, joining field missions and virtual meetings with client governments). The E T consultant will also be expected to contribute or lead knowledge products related to climate risk and NBS and support the other Pillars of th</t>
+          <t>The E T Consultant’s will support implementation of GPNBS programming. Tasks include coordinating and leading operational expert support on NBS to Task Teams and clients under the Operations pillar of the Program (advice on technical studies for project design and implementation, joining field missions and virtual meetings with client governments). The E T consultant will also be expected to contribute or lead knowledge products related to climate risk and NBS and support the other Pillars of the program where relevant. The E T Consultant will work closely with the Task Team Leaders and core staff of the Global Program, under managerial supervision of the Practice Manager of IDURM. Specific responsibilities and duties will include (but not be limited to) the following: Take a leading role in the delivery of geospatial and analytical assessments to Task Teams and Governments, including the NBSOS. Provide direct support to clients and Task Teams globally in the identification, assessment, implementation and monitoring of NBS, by conducting and supervising technical studies, providing input to project documents, training and capacity building, developing result indicators, participating in virtual and in-person meetings and missions, and related activities. Cultivate and advance partnerships with firms, consultants, external institutions, and internal World Bank teams for the co-development of new products, support to operational Task Teams, and advancement of the field of NBS. Lead and/or contribute to knowledge products related to NBS analytics developed under the Knowledge pillar of the Program. Illustrate Program advancements and contributions in the form of blogs, peer-reviewed papers, conference contributions, etc. Contribute to programmatic outputs including results monitoring, reporting, budgeting, and branding Deliver presentations and workshops at a variety of settings, including with Task Teams, government counterparts and at internal and external events.</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -3701,7 +3722,7 @@
       </c>
       <c r="Q36" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate risk, climate resilience, and climate change, indicating a strong focus on climate-related issues. The role involves working on Nature-Based Solutions for Climate Resilience, which is a key area of focus for climate risk management.</t>
+          <t>The job description mentions climate risk, climate resilience, and climate change, indicating a strong focus on climate-related issues. The role involves working on Nature-Based Solutions for Climate Resilience, which is a key area of focus for climate risk management.</t>
         </is>
       </c>
       <c r="R36" s="2" t="inlineStr"/>
@@ -3780,17 +3801,17 @@
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
-          <t>The General Counsel (GC) will serve as the chief legal advisor to the organisation, overseeing all legal, regulatory, governance, and compliance matters for a rapidly growing renewable energy business. The GC will lead the legal function, support strategic decision-making, manage external counsel, and ensure the organisation’s interests are protected across all jurisdictions in which it operates. Key Responsibilities include Strategic Legal Leadership, Project Development &amp; Renewable Energy Tran</t>
+          <t>The General Counsel (GC) will serve as the chief legal advisor to the organisation, overseeing all legal, regulatory, governance, and compliance matters for a rapidly growing renewable energy business. The GC will lead the legal function, support strategic decision-making, manage external counsel, and ensure the organisation’s interests are protected across all jurisdictions in which it operates. Key Responsibilities include Strategic Legal Leadership, Project Development &amp; Renewable Energy Transactions, Mergers &amp; Acquisitions, Power Purchase Agreements (PPAs) &amp; Revenue Contracts, Investment, Divestment &amp; Capital Markets, Corporate Governance &amp; Compliance, and External Counsel &amp; Stakeholder Management.</t>
         </is>
       </c>
       <c r="P37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Essential skills include drafting, negotiation, and commercial advisory skills. Desirable skills include international renewable energy experience, prior leadership of a legal function or high-performing legal team, experience in ESG, sustainability regulations, and climate-related disclosures, and </t>
+          <t>Essential skills include drafting, negotiation, and commercial advisory skills. Desirable skills include international renewable energy experience, prior leadership of a legal function or high-performing legal team, experience in ESG, sustainability regulations, and climate-related disclosures, and familiarity with corporate governance in high-growth or investor-backed companies.</t>
         </is>
       </c>
       <c r="Q37" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description is focused on renewable energy projects, utility-scale solar, wind, battery storage, and hybrid energy projects, which are all related to clean energy and environmental science.</t>
+          <t>The job description is focused on renewable energy projects, utility-scale solar, wind, battery storage, and hybrid energy projects, which are all related to clean energy and environmental science.</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
@@ -3877,17 +3898,17 @@
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
-          <t>The TNC-GCF Climate Finance Specialist provides sophisticated business, financial and economic expertise to address conservation challenges. The TNC-GCF Climate Finance Specialist will support a key strategic initiative within The Nature Conservancy by sourcing, developing, and guiding the structuring of non-grant instruments financed by the Green Climate Fund in support of some of our most ambitious climate and conservation efforts. The Specialist is primarily responsible for developing the non</t>
+          <t>The TNC-GCF Climate Finance Specialist provides sophisticated business, financial and economic expertise to address conservation challenges. The TNC-GCF Climate Finance Specialist will support a key strategic initiative within The Nature Conservancy by sourcing, developing, and guiding the structuring of non-grant instruments financed by the Green Climate Fund in support of some of our most ambitious climate and conservation efforts. The Specialist is primarily responsible for developing the non-grant instrument (NGI) components of GCF project proposals, creating the enabling conditions to successfully deliver GCF projects with NGIs.</t>
         </is>
       </c>
       <c r="P38" s="6" t="inlineStr">
         <is>
-          <t>Deep knowledge of financial institutions, including community, commercial, development, sovereign or investment banks and their approaches to loan origination, underwriting, on-lending and risk assessment. Knowledge of environmental and social management systems within financial institutions. Experi</t>
+          <t>Deep knowledge of financial institutions, including community, commercial, development, sovereign or investment banks and their approaches to loan origination, underwriting, on-lending and risk assessment. Knowledge of environmental and social management systems within financial institutions. Experience negotiating complex agreements and working with teams across the organization as well as externally. Experience with current and evolving sustainable finance and ESG trends.</t>
         </is>
       </c>
       <c r="Q38" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions experience with sustainable finance and ESG trends, and the role involves working with non-grant instruments financed by the Green Climate Fund, which is related to sustainable finance and impact investing.</t>
+          <t>The job description mentions experience with sustainable finance and ESG trends, and the role involves working with non-grant instruments financed by the Green Climate Fund, which is related to sustainable finance and impact investing.</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -3980,7 +4001,7 @@
       </c>
       <c r="Q39" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions working on environmental projects, including renewable energy, and conducting ecological field surveys, which aligns with the clean energy adjacent profile.</t>
+          <t>The job description mentions working on environmental projects, including renewable energy, and conducting ecological field surveys, which aligns with the clean energy adjacent profile.</t>
         </is>
       </c>
       <c r="R39" s="2" t="inlineStr">
@@ -4067,17 +4088,17 @@
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
-          <t>Lead ESG advisory projects from inception to delivery, including strategic direction and team coordination. Collaborate with project managers to plan and execute projects, ensuring client satisfaction and successful outcomes. Develop and present comprehensive analyses, conclusions, and deliverables, including written reports, metrics, and insights. Execute multi-disciplinary projects across various aspects of sustainability platforms in a collaborative manner. Ensure quality deliverables aligned</t>
+          <t>Lead ESG advisory projects from inception to delivery, including strategic direction and team coordination. Collaborate with project managers to plan and execute projects, ensuring client satisfaction and successful outcomes. Develop and present comprehensive analyses, conclusions, and deliverables, including written reports, metrics, and insights. Execute multi-disciplinary projects across various aspects of sustainability platforms in a collaborative manner. Ensure quality deliverables aligned with client objectives and maintain high levels of client satisfaction through effective communication and engagement. Stay updated on ESG concepts, methodologies, and best practices, and share insights with the team to foster continuous improvement.</t>
         </is>
       </c>
       <c r="P40" s="6" t="inlineStr">
         <is>
-          <t>Strong knowledge of ESG reporting frameworks, including GRI, SASB, DJSI/S&amp;P, CDP, BRSR, TCFD, and UNPRI. Advanced proficiency in MS Excel; data science skills are a plus. Strong written and verbal communication skills in English, with excellent presentation skills. Capable of working under pressure,</t>
+          <t>Strong knowledge of ESG reporting frameworks, including GRI, SASB, DJSI/S&amp;P, CDP, BRSR, TCFD, and UNPRI. Advanced proficiency in MS Excel; data science skills are a plus. Strong written and verbal communication skills in English, with excellent presentation skills. Capable of working under pressure, maintaining flexibility in work hours. Working independently with minimal supervision.</t>
         </is>
       </c>
       <c r="Q40" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions ESG reporting, climate risk analysis, corporate ESG disclosures, and decarbonization strategies, which are all relevant to environmental, social, and governance topics, indicating a strong fit for the general_esg profile.</t>
+          <t>The job description mentions ESG reporting, climate risk analysis, corporate ESG disclosures, and decarbonization strategies, which are all relevant to environmental, social, and governance topics, indicating a strong fit for the general_esg profile.</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4164,17 +4185,17 @@
       </c>
       <c r="O41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Execute consulting projects for different clients related to ESG/ Sustainability Advisory across areas such as ESG Strategic Direction covering stakeholder engagement and materiality assessment, ESG Policy and Governance Framework, Sustainability Reporting &amp; Disclosures based on different frameworks, GHG Accounting, Decarbonization Roadmap using SBTi guidelines, Sustainable Financing, Supply chain, etc. Undertake activities required for execution such as research on companies and ESG practices, </t>
+          <t>Execute consulting projects for different clients related to ESG/ Sustainability Advisory across areas such as ESG Strategic Direction covering stakeholder engagement and materiality assessment, ESG Policy and Governance Framework, Sustainability Reporting &amp; Disclosures based on different frameworks, GHG Accounting, Decarbonization Roadmap using SBTi guidelines, Sustainable Financing, Supply chain, etc. Undertake activities required for execution such as research on companies and ESG practices, peer benchmarking, developing data collection templates and writing of ESG/ Sustainability reports. Ensure timely delivery of all project deliverables as per agreed timelines and client satisfaction. Travel to client location as may be required from time to time for the project activities. Work in tandem with the other team members and any other internal and external stakeholders such as design team, subject matter experts, etc. Assist the practice lead/ manager in practice development activities such as preparing pre-sales pitches, approach papers, point of views, articles, newsletter, etc. Keeping abreast of ESG trends and regulatory requirements in focus geographies Any other support that may be required from time to time for the development and growth of the practice.</t>
         </is>
       </c>
       <c r="P41" s="6" t="inlineStr">
         <is>
-          <t>Hands-on experience, knowledge and understanding of ESG/ sustainability concepts and frameworks like GRI, SASB, TCFD, etc. Proficient in MS Word, PowerPoint and Excel. Good writing and analytical skills Comfortable to engage in multiple projects simultaneously Highly flexible and quick learner to ad</t>
+          <t>Hands-on experience, knowledge and understanding of ESG/ sustainability concepts and frameworks like GRI, SASB, TCFD, etc. Proficient in MS Word, PowerPoint and Excel. Good writing and analytical skills Comfortable to engage in multiple projects simultaneously Highly flexible and quick learner to adopt and apply new methodology/ approach Open to travel for project execution Excellent communicator and good team player</t>
         </is>
       </c>
       <c r="Q41" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions ESG Advisory, Sustainability Reporting, GHG Accounting, Decarbonization Roadmap, and Sustainable Financing, which are all related to environmental, social, and governance topics, indicating a strong fit with the general ESG profile.</t>
+          <t>The job description mentions ESG Advisory, Sustainability Reporting, GHG Accounting, Decarbonization Roadmap, and Sustainable Financing, which are all related to environmental, social, and governance topics, indicating a strong fit with the general ESG profile.</t>
         </is>
       </c>
       <c r="R41" s="2" t="inlineStr">
@@ -4250,12 +4271,12 @@
       </c>
       <c r="P42" s="6" t="inlineStr">
         <is>
-          <t>Conoscenza dei principali software office quali MS Excel, Word, Power Point; Conoscenza di dei software di analisi dati e di mercato (R/Phyton, SAS, Qlik, SQL, PowerBi); Conoscenza dei framework di sostenibilità (es. SFDR, Taxonomy Regulation, ECB aspettative, CSR, DNF, PRI ecc.); Conoscenza di indi</t>
+          <t>Conoscenza dei principali software office quali MS Excel, Word, Power Point; Conoscenza di dei software di analisi dati e di mercato (R/Phyton, SAS, Qlik, SQL, PowerBi); Conoscenza dei framework di sostenibilità (es. SFDR, Taxonomy Regulation, ECB aspettative, CSR, DNF, PRI ecc.); Conoscenza di indici internazionali di sostenibilità come TCFD, GRI, CDP, SBTi e ESG</t>
         </is>
       </c>
       <c r="Q42" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions sustainability, climate change, and ESG frameworks, indicating a focus on environmental, social, and governance topics.</t>
+          <t>The job description mentions sustainability, climate change, and ESG frameworks, indicating a focus on environmental, social, and governance topics.</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr"/>
@@ -4334,7 +4355,7 @@
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assist in preparation of regular and ad-hoc risk reports, Review limits and guidelines of pension funds, compliance limit check of portfolio and target investments according to investment policy and imposed limits, Perform daily pension fund limit monitoring, Conduct investment risk analysis, quantitative and qualitative research, Perform analysis of the ESG risks applicable to pension funds and target investments, Maintain and improve supportive tools for analysis, measurement and reporting of </t>
+          <t>Assist in preparation of regular and ad-hoc risk reports, Review limits and guidelines of pension funds, compliance limit check of portfolio and target investments according to investment policy and imposed limits, Perform daily pension fund limit monitoring, Conduct investment risk analysis, quantitative and qualitative research, Perform analysis of the ESG risks applicable to pension funds and target investments, Maintain and improve supportive tools for analysis, measurement and reporting of investment and ESG metrics of pension funds and target investments, Deliver and follow-up on personal tasks timely and according to the set quality standards, Take responsibility in professional self-development and contribute to own and team performance improvement by constructive feedback and relevant suggestions</t>
         </is>
       </c>
       <c r="P43" s="6" t="inlineStr">
@@ -4344,7 +4365,7 @@
       </c>
       <c r="Q43" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'sustainable finance', 'ESG risks', and 'investment risk analysis', which are key terms related to sustainable finance and ESG investing.</t>
+          <t>The job description mentions 'sustainable finance', 'ESG risks', and 'investment risk analysis', which are key terms related to sustainable finance and ESG investing.</t>
         </is>
       </c>
       <c r="R43" s="2" t="inlineStr">
@@ -4432,12 +4453,12 @@
       </c>
       <c r="P44" s="6" t="inlineStr">
         <is>
-          <t>Proven experience with: Valorisation of research and technology, including optimal IP valorisation, Scaling and de-risking innovations towards industry, Public-private partnerships, Ability to connect complex ecosystems and align stakeholders around a shared ambition, Fluent in English and Dutch; ot</t>
+          <t>Proven experience with: Valorisation of research and technology, including optimal IP valorisation, Scaling and de-risking innovations towards industry, Public-private partnerships, Ability to connect complex ecosystems and align stakeholders around a shared ambition, Fluent in English and Dutch; other languages are a plus</t>
         </is>
       </c>
       <c r="Q44" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions cleantech, circularity, materials, chemistry, and industrial transition, which are all related to environmental science and sustainability, and specifically mentions the development of low-CO₂ construction materials, plastics recycling, and bio-ec</t>
+          <t>The job description mentions cleantech, circularity, materials, chemistry, and industrial transition, which are all related to environmental science and sustainability, and specifically mentions the development of low-CO₂ construction materials, plastics recycling, and bio-economy, which are all relevant to the clean energy and environmental science fields</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
@@ -4520,7 +4541,7 @@
       </c>
       <c r="O45" s="6" t="inlineStr">
         <is>
-          <t>The intern will support ISO with analytical and preparatory work that helps identify behavioural barriers, motivational drivers, and communication opportunities linked to four priority areas identified through the Green Pulse Survey conducted in 2025. The role is primarily analytical and strategic, with communications and graphic design skills considered an asset to support knowledge translation and internal engagement. The intern will be responsible for the following general/specific tasks: Beh</t>
+          <t>The intern will support ISO with analytical and preparatory work that helps identify behavioural barriers, motivational drivers, and communication opportunities linked to four priority areas identified through the Green Pulse Survey conducted in 2025. The role is primarily analytical and strategic, with communications and graphic design skills considered an asset to support knowledge translation and internal engagement. The intern will be responsible for the following general/specific tasks: Behavioural Insights Review &amp; Evidence Synthesis, Behavioural Diagnostics &amp; Prioritization, Strategy Development Support, Coordination &amp; Consultation Support, Knowledge Management &amp; Documentation.</t>
         </is>
       </c>
       <c r="P45" s="6" t="inlineStr">
@@ -4530,7 +4551,7 @@
       </c>
       <c r="Q45" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions sustainability, social and behaviour change, and environmental footprint, which are all related to ESG strategy and corporate sustainability.</t>
+          <t>The job description mentions sustainability, social and behaviour change, and environmental footprint, which are all related to ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
@@ -4601,17 +4622,17 @@
       </c>
       <c r="O46" s="6" t="inlineStr">
         <is>
-          <t>Corporate and Project Financing: In collaboration with the Corporate Finance Manager, you will ensure suitable and competitive financing of the group’s financial needs. You propose and design the most appropriate type of debt taking into account the group strategy &amp; policies. You go to the capital market and lead financing projects, negotiate the best financing conditions and finalise the transactions. You evaluate the interest of sustainable finance &amp; ESG instruments, propose the most appropria</t>
+          <t>Corporate and Project Financing: In collaboration with the Corporate Finance Manager, you will ensure suitable and competitive financing of the group’s financial needs. You propose and design the most appropriate type of debt taking into account the group strategy &amp; policies. You go to the capital market and lead financing projects, negotiate the best financing conditions and finalise the transactions. You evaluate the interest of sustainable finance &amp; ESG instruments, propose the most appropriate options for Fluxys activities. Hedging &amp; risks: Together with the back-office team, you will monitor and report on interest rates, exchange rates and liquidity risks. You propose appropriate hedging transactions and negotiate best foreign exchange and hedging conditions. Group treasury management: You carry out daily treasury activities and maximise the return on financial investments and optimise cash management by monitoring short-term deposits and financing. Stakeholder management: You will work with and maintain an active network of relationships with banks, institutional investors and other financial market players. You monitor markets conditions and develop market intelligence and provide financing advisory services to a wide range of internal stakeholders (M&amp;A, business development, subsidiaries). You contribute to financial due diligence exercises by providing accurate and timely information.</t>
         </is>
       </c>
       <c r="P46" s="6" t="inlineStr">
         <is>
-          <t>Strong analytical skills, in-depth understanding of financial markets, comprehensive knowledge of various debt instruments, proficiency in daily treasury activities, cash management, and optimizing financial investments, experience in people management, natural communicator, high-impact professional</t>
+          <t>Strong analytical skills, in-depth understanding of financial markets, comprehensive knowledge of various debt instruments, proficiency in daily treasury activities, cash management, and optimizing financial investments, experience in people management, natural communicator, high-impact professional, strong strategic mindset, results-oriented and resilient.</t>
         </is>
       </c>
       <c r="Q46" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'sustainable finance &amp; ESG instruments' and the company is committed to fast-tracking the shift to a carbon neutral world, indicating a focus on sustainable finance and ESG concepts.</t>
+          <t>The job description mentions 'sustainable finance &amp; ESG instruments' and the company is committed to fast-tracking the shift to a carbon neutral world, indicating a focus on sustainable finance and ESG concepts.</t>
         </is>
       </c>
       <c r="R46" s="2" t="inlineStr"/>
@@ -4696,7 +4717,7 @@
       </c>
       <c r="Q47" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions ESG factors, sustainable finance, green finance, and sustainable investment initiatives, which are all relevant to the sustainable finance profile.</t>
+          <t>The job description mentions ESG factors, sustainable finance, green finance, and sustainable investment initiatives, which are all relevant to the sustainable finance profile.</t>
         </is>
       </c>
       <c r="R47" s="2" t="inlineStr"/>
@@ -4763,7 +4784,7 @@
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
-          <t>You will have the opportunity to gain insight into the forest management and natural capital sector and be involved in everything from asset management to deal sourcing and execution, providing an ideal opportunity to develop your skills and learn about the day-to-day work in natural capital investments. As an Investment Intern, you will participate in various activities related to forestry and natural capital investments, including: Doing market research and analysing market trends, Creating fu</t>
+          <t>You will have the opportunity to gain insight into the forest management and natural capital sector and be involved in everything from asset management to deal sourcing and execution, providing an ideal opportunity to develop your skills and learn about the day-to-day work in natural capital investments. As an Investment Intern, you will participate in various activities related to forestry and natural capital investments, including: Doing market research and analysing market trends, Creating fund marketing materials and other internal or external presentations, Assisting in the analysis of new investment opportunities and preparation of investment presentations, Assisting in financial modelling and valuation as part of the screening process of new investment opportunities, Participating in due diligence processes for new acquisitions, according to possibilities, Supporting in the value creation of existing portfolio companies by participating in day-to-day asset management, according to possibilities, Collaborating on exciting business development projects to further CapMan Natural Capital’s impact</t>
         </is>
       </c>
       <c r="P48" s="6" t="inlineStr">
@@ -4773,7 +4794,7 @@
       </c>
       <c r="Q48" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions natural capital investments, forestry, and sustainable forestry investments, which are related to environmental science and conservation, fitting the clean_energy_adjacent profile.</t>
+          <t>The job description mentions natural capital investments, forestry, and sustainable forestry investments, which are related to environmental science and conservation, fitting the clean_energy_adjacent profile.</t>
         </is>
       </c>
       <c r="R48" s="2" t="inlineStr"/>
@@ -4852,7 +4873,7 @@
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perform in-depth financial modelling and analysis related to capital structure, funding strategy, acquisition and debt capacity, and credit ratings. Integrate sustainability considerations into financial analysis, including impacts on availability, pricing and structure of capital. Prepare clear, well-structured and robust materials for senior internal stakeholders and client presentations. Take an active role in client projects, with increasing exposure to senior decision-makers. Contribute to </t>
+          <t>Perform in-depth financial modelling and analysis related to capital structure, funding strategy, acquisition and debt capacity, and credit ratings. Integrate sustainability considerations into financial analysis, including impacts on availability, pricing and structure of capital. Prepare clear, well-structured and robust materials for senior internal stakeholders and client presentations. Take an active role in client projects, with increasing exposure to senior decision-makers. Contribute to the continuous development of analytical tools, methodologies and advisory processes.</t>
         </is>
       </c>
       <c r="P49" s="6" t="inlineStr">
@@ -4862,7 +4883,7 @@
       </c>
       <c r="Q49" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions integrating sustainability considerations into financial analysis, and the role is part of the Corporate &amp; Sustainability Advisory team, indicating a focus on sustainable finance.</t>
+          <t>The job description mentions integrating sustainability considerations into financial analysis, and the role is part of the Corporate &amp; Sustainability Advisory team, indicating a focus on sustainable finance.</t>
         </is>
       </c>
       <c r="R49" s="2" t="inlineStr">
@@ -4954,12 +4975,12 @@
       </c>
       <c r="P50" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCA Tools like SimaPro, guideline documents and operational system of a GHG reduction scheme, project cycle and Regulatory requirements, auditing principles, procedures and techniques, risk assessment techniques, data and information sampling techniques, materiality and level of assurance concepts, </t>
+          <t>LCA Tools like SimaPro, guideline documents and operational system of a GHG reduction scheme, project cycle and Regulatory requirements, auditing principles, procedures and techniques, risk assessment techniques, data and information sampling techniques, materiality and level of assurance concepts, MS Office, verbal &amp; written expression, fluent in spoken English, par-excellence writing skills, deadline oriented</t>
         </is>
       </c>
       <c r="Q50" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions GHG Footprint, LCA, ESG, BRSR Reporting, and GHG reduction schemes, which are directly related to climate risk and transition risk.</t>
+          <t>The job description mentions GHG Footprint, LCA, ESG, BRSR Reporting, and GHG reduction schemes, which are directly related to climate risk and transition risk.</t>
         </is>
       </c>
       <c r="R50" s="2" t="inlineStr">
@@ -5107,7 +5128,7 @@
       </c>
       <c r="O52" s="6" t="inlineStr">
         <is>
-          <t>The HR Project &amp; Transformation Lead will partner across the HR functions and Business Groups to deliver value-added services to management and employees. Lead and drive projects that enhance networking opportunities and foster HR collaboration across Sectors and Business Units within the Region, including cross-regional collaboration among RHQ HR teams. Assume responsibility as Project Lead and Project Manager in relation to collaboration activities across Groups. Expand engagement with other G</t>
+          <t>The HR Project &amp; Transformation Lead will partner across the HR functions and Business Groups to deliver value-added services to management and employees. Lead and drive projects that enhance networking opportunities and foster HR collaboration across Sectors and Business Units within the Region, including cross-regional collaboration among RHQ HR teams. Assume responsibility as Project Lead and Project Manager in relation to collaboration activities across Groups. Expand engagement with other Groups around internal mobility to attract and retain employees across the Region. Work as the HR lead on projects as required. Work closely with management and stakeholders to further enhance work relationships and collaboration across Groups in EMEA. Promote the Hitachi Brand in EMEA, to attract and onboard top talent. Provide regional enablement for legislative changes such as the EU Pay Directive. Support education of Managers and employees around new landscape for Diversity. Drive a ‘growth mindset’ culture within the Regional HQ and beyond. Support line managers across the Region in leading and delivering change including restructuring, reorganization, integration, consultation, TUPE, redundancy, job redesign and redeployments. Manage and resolve complex employee relations issues as needed</t>
         </is>
       </c>
       <c r="P52" s="6" t="inlineStr">
@@ -5117,7 +5138,7 @@
       </c>
       <c r="Q52" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions integrating sustainability considerations into financial analysis, and the role is part of the Corporate &amp; Sustainability Advisory team, indicating a focus on sustainable finance.</t>
+          <t>The job description does not explicitly mention ESG, sustainability, or climate-related responsibilities, requirements, or skills, despite the company being involved in climate change innovation and green energy. The role is focused on HR project and transformation leadership, which does not fit into any of the specified ESG/sustainability profiles.</t>
         </is>
       </c>
       <c r="R52" s="2" t="inlineStr"/>
@@ -5184,17 +5205,17 @@
       </c>
       <c r="O53" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Head of Finance and Accounting is a highly visible leadership position responsible for managing the organization’s financial control environment and ensuring compliance with IFRS, Group Financial Guidelines and local Statutory Accounting and regulatory requirements across the Europe, Middle East and Africa region. This role oversees end-to-end accounting operations, including monthly, quarterly, and annual closings, and holds accountability for working capital and balance sheet forecasting, </t>
+          <t>The Head of Finance and Accounting is a highly visible leadership position responsible for managing the organization’s financial control environment and ensuring compliance with IFRS, Group Financial Guidelines and local Statutory Accounting and regulatory requirements across the Europe, Middle East and Africa region. This role oversees end-to-end accounting operations, including monthly, quarterly, and annual closings, and holds accountability for working capital and balance sheet forecasting, Balance Sheet and treasury management, and intercompany processes to maintain financial integrity. Key Responsibilities: Financial Governance &amp; Compliance, Process Improvement &amp; Standardization, Stakeholder Collaboration, Team Leadership &amp; Transformation, Safety First</t>
         </is>
       </c>
       <c r="P53" s="6" t="inlineStr">
         <is>
-          <t>Technical expertise in finance and accounting, leadership capabilities, strong communication and collaboration skills, ability to build and develop a high-performing accounting organization, experience with SAP ERP systems, knowledge of IFRS, statutory reporting, internal controls, audit management,</t>
+          <t>Technical expertise in finance and accounting, leadership capabilities, strong communication and collaboration skills, ability to build and develop a high-performing accounting organization, experience with SAP ERP systems, knowledge of IFRS, statutory reporting, internal controls, audit management, treasury operations, FX risk management, and working capital optimization</t>
         </is>
       </c>
       <c r="Q53" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions GHG Footprint, LCA, ESG, BRSR Reporting, and GHG reduction schemes, which are directly related to climate risk and transition risk.</t>
+          <t>The job description does not explicitly mention ESG, sustainability, or environmental topics in the context of the role's responsibilities, requirements, or skills, except for a general mention of 'sustainable' in the company description which is not directly related to the job's responsibilities</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr"/>
@@ -5261,17 +5282,17 @@
       </c>
       <c r="O54" s="6" t="inlineStr">
         <is>
-          <t>With an exclusive focus on the Nespresso business, you will work within the core Finance team, supporting the design of financial, fiscal, and accounting flows across various business processes while building and enhancing the technology platforms that support the business. As a Senior Finance IT Business Analyst, you will coordinate and guide a team of IT Business Analysts and Product Experts responsible for understanding end-to-end business flows. You will analyze and define business and funct</t>
+          <t>With an exclusive focus on the Nespresso business, you will work within the core Finance team, supporting the design of financial, fiscal, and accounting flows across various business processes while building and enhancing the technology platforms that support the business. As a Senior Finance IT Business Analyst, you will coordinate and guide a team of IT Business Analysts and Product Experts responsible for understanding end-to-end business flows. You will analyze and define business and functional requirements, collaborating with team members to translate these requirements into the product backlog.</t>
         </is>
       </c>
       <c r="P54" s="6" t="inlineStr">
         <is>
-          <t>Experience working on Finance/Fiscal legislation initiatives related to retail business flows running on ERP systems, POS systems and e-Commerce. Experience working in a global environment and with virtual teams. Strong analytical thinking and business analysis skills. Effective communication, inter</t>
-        </is>
-      </c>
-      <c r="Q54" s="2" t="inlineStr">
-        <is>
-          <t>This role contributes to the sustainable development goals of Nestlé by supporting the financial and technological aspects of Nespresso's operations.</t>
+          <t>Experience working on Finance/Fiscal legislation initiatives related to retail business flows running on ERP systems, POS systems and e-Commerce. Experience working in a global environment and with virtual teams. Strong analytical thinking and business analysis skills. Effective communication, interpersonal, and stakeholder management abilities.</t>
+        </is>
+      </c>
+      <c r="Q54" s="6" t="inlineStr">
+        <is>
+          <t>The job description does not mention any specific ESG, sustainability, or climate-related responsibilities, requirements, or skills that would fit into one of the provided profiles.</t>
         </is>
       </c>
       <c r="R54" s="2" t="inlineStr"/>
@@ -5346,17 +5367,17 @@
       </c>
       <c r="O55" s="6" t="inlineStr">
         <is>
-          <t>Lead and Deliver Strategic Mining Advisory Projects, Manage and execute environmental and social performance input into feasibility studies, due diligence assignments, ITRs/ITERs, and operational improvement programs. Deliver clear, innovative, and commercially relevant insights aligned with client needs and project scope. Provide Senior Technical Expertise, Participate in Multi-Disciplinary Project Teams, Engage Senior and Executive-Level Stakeholders, Drive Business Development and Industry Pr</t>
+          <t>Lead and Deliver Strategic Mining Advisory Projects, Manage and execute environmental and social performance input into feasibility studies, due diligence assignments, ITRs/ITERs, and operational improvement programs. Deliver clear, innovative, and commercially relevant insights aligned with client needs and project scope. Provide Senior Technical Expertise, Participate in Multi-Disciplinary Project Teams, Engage Senior and Executive-Level Stakeholders, Drive Business Development and Industry Presence, Support Team Culture, Collaboration &amp; Wellbeing</t>
         </is>
       </c>
       <c r="P55" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Technical Skills &amp; Experience, Environmental and social impact assessment, environmental and social due diligence, environmental and social management systems, lenders environmental and social performance requirements, including but not limited to Equator Principles and IFC Environmental and Social </t>
+          <t>Technical Skills &amp; Experience, Environmental and social impact assessment, environmental and social due diligence, environmental and social management systems, lenders environmental and social performance requirements, including but not limited to Equator Principles and IFC Environmental and Social Performance Standards</t>
         </is>
       </c>
       <c r="Q55" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions environmental and social performance management, impact assessment, and due diligence, which are all relevant to ESG strategy and corporate sustainability. The role also involves providing advice on environmental and social performance to mining clients, wh</t>
+          <t>The job description mentions environmental and social performance management, impact assessment, and due diligence, which are all relevant to ESG strategy and corporate sustainability. The role also involves providing advice on environmental and social performance to mining clients, which aligns with the general ESG profile.</t>
         </is>
       </c>
       <c r="R55" s="2" t="inlineStr">
@@ -5439,17 +5460,17 @@
       </c>
       <c r="O56" s="6" t="inlineStr">
         <is>
-          <t>Develop and execute a comprehensive sales strategy for Neural Alpha’s SaaS platform, targeting financial institutions, asset managers, corporates and NGOs. Own the full sales cycle from prospecting and lead qualification through to negotiation, close and handover to Customer Success. Build and manage a robust sales pipeline using CRM tools, ensuring accurate forecasting and reporting to senior leadership. Establish and lead the creation of a scalable sales function, defining processes, playbooks</t>
+          <t>Develop and execute a comprehensive sales strategy for Neural Alpha’s SaaS platform, targeting financial institutions, asset managers, corporates and NGOs. Own the full sales cycle from prospecting and lead qualification through to negotiation, close and handover to Customer Success. Build and manage a robust sales pipeline using CRM tools, ensuring accurate forecasting and reporting to senior leadership. Establish and lead the creation of a scalable sales function, defining processes, playbooks, methodologies and best practices. Lead client-facing engagements including discovery calls, platform demonstrations, proof of concept discussions and commercial negotiations. Represent Neural Alpha at industry conferences, webinars, roundtables, working groups and networking events, building the company’s profile and generating new business opportunities.</t>
         </is>
       </c>
       <c r="P56" s="6" t="inlineStr">
         <is>
-          <t>Proficiency with CRM platforms (e.g. HubSpot, Salesforce) and modern sales enablement tools. Comfortable embracing and leveraging AI tools and technology to enhance personal productivity and sales effectiveness. Knowledge of ESG, sustainable finance, or regulatory frameworks such as ISSB, CSRD, EU T</t>
+          <t>Proficiency with CRM platforms (e.g. HubSpot, Salesforce) and modern sales enablement tools. Comfortable embracing and leveraging AI tools and technology to enhance personal productivity and sales effectiveness. Knowledge of ESG, sustainable finance, or regulatory frameworks such as ISSB, CSRD, EU Taxonomy, SFDR and TNFD.</t>
         </is>
       </c>
       <c r="Q56" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions experience selling into financial institutions, asset managers or large corporates, and knowledge of ESG, sustainable finance, or regulatory frameworks such as ISSB, CSRD, EU Taxonomy, SFDR and TNFD, indicating a strong connection to sustainable fin</t>
+          <t>The job description mentions experience selling into financial institutions, asset managers or large corporates, and knowledge of ESG, sustainable finance, or regulatory frameworks such as ISSB, CSRD, EU Taxonomy, SFDR and TNFD, indicating a strong connection to sustainable finance.</t>
         </is>
       </c>
       <c r="R56" s="2" t="inlineStr">
@@ -5532,7 +5553,7 @@
       </c>
       <c r="O57" s="6" t="inlineStr">
         <is>
-          <t>The incumbent will be responsible for product strategy and coordination, product delivery, capacity building and deployment, quality assurance, stakeholder engagement, and knowledge management. Specific duties include: Liaise with CAFI PES technical team and implementation partners to capture functional requirements, Translate operational needs into clear technical specifications for developers, Monitor and report on project progress, Drive the functional vision and evolution of the products, En</t>
+          <t>The incumbent will be responsible for product strategy and coordination, product delivery, capacity building and deployment, quality assurance, stakeholder engagement, and knowledge management. Specific duties include: Liaise with CAFI PES technical team and implementation partners to capture functional requirements, Translate operational needs into clear technical specifications for developers, Monitor and report on project progress, Drive the functional vision and evolution of the products, Ensure integration with other digital tools used by CAFI, Develop the work plan for the developers, Review prototypes, Coordinate user acceptance testing and validation of system features, Facilitate/Coordinate training of CAFI colleagues, implementation partners and partner governments on system use, Develop user guides and SOPs for PES digital workflows, Ensure data integrity, traceability, and compliance with CAFI’s monitoring &amp; evaluation and data protection policies, Ensure the overall cyber security and integrity of the system, Facilitate integration of independent verification processes into the system, Maintain regular communication between CAFI Secretariat, IT teams, and field partners, Document lessons learned and contribute to system improvement roadmap, Facilitate knowledge-sharing and capacity-building activities for project partners and stakeholders, Identify opportunities for PES systems through collaboration with other technical teams and experts, Plan and lead in-person workshops and side events, Contribute to global Digital Public Infrastructure discussions, briefing notes, and concepts related to the PES systems, Plan, design, and coordinate a Community of Practice.</t>
         </is>
       </c>
       <c r="P57" s="6" t="inlineStr">
@@ -5542,7 +5563,7 @@
       </c>
       <c r="Q57" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description is related to the conservation of forests, reduction of deforestation, and promotion of sustainable development, which are all relevant to the clean energy and environmental conservation sector.</t>
+          <t>The job description is related to the conservation of forests, reduction of deforestation, and promotion of sustainable development, which are all relevant to the clean energy and environmental conservation sector.</t>
         </is>
       </c>
       <c r="R57" s="2" t="inlineStr">
@@ -5625,7 +5646,7 @@
       </c>
       <c r="O58" s="6" t="inlineStr">
         <is>
-          <t>You will contribute to financial audit engagements and, in parallel, support the Data Audit Team by delivering analytics that strengthen audit quality, consistency, and documentation. Collect, structure and process large financial and operational datasets for audit purposes. Perform data analyses to support risk assessments and audit procedures. Build audit-ready outputs and visualizations using Excel and Power BI where relevant. Automate and continuously improve data-driven audit analyses and t</t>
+          <t>You will contribute to financial audit engagements and, in parallel, support the Data Audit Team by delivering analytics that strengthen audit quality, consistency, and documentation. Collect, structure and process large financial and operational datasets for audit purposes. Perform data analyses to support risk assessments and audit procedures. Build audit-ready outputs and visualizations using Excel and Power BI where relevant. Automate and continuously improve data-driven audit analyses and techniques. Ensure data integrity by validating the completeness and reliability of client data and documenting key checks and transformations in line with audit quality standards. Collaborate with audit teams to enable strong, meaningful audit conclusions by designing fit-for-purpose analytics. Act as a key point of contact with client finance stakeholders and internal data owners to collect the right data, on time, and clarify extraction requirements. Actively contribute to innovation and continuous improvement within the audit data team.</t>
         </is>
       </c>
       <c r="P58" s="6" t="inlineStr">
@@ -5633,9 +5654,9 @@
           <t>Data analytics, data engineering, Excel, Power BI, SQL, Python, business economics, finance, audit fundamentals</t>
         </is>
       </c>
-      <c r="Q58" s="2" t="inlineStr">
-        <is>
-          <t>This role is within the finance industry, focusing on auditing and data analytics for financial reporting and risk assessment.</t>
+      <c r="Q58" s="6" t="inlineStr">
+        <is>
+          <t>The job description does not explicitly mention ESG, sustainability, or environmental topics in the context of the role's responsibilities, requirements, or skills, other than the company's general sustainability policy which is not directly related to the job.</t>
         </is>
       </c>
       <c r="R58" s="2" t="inlineStr">
@@ -5718,7 +5739,7 @@
       </c>
       <c r="O59" s="6" t="inlineStr">
         <is>
-          <t>The role will include the following objectives: Provide technical expertise and operational support to GFDRR’s Disaster-FCV Nexus program, focusing on FCV-sensitive disaster risk management and climate resilience. Strengthen GFDRR’s analytical, advisory, and partnership work on the disaster-FCV nexus, including knowledge generation, policy dialogue, and capacity building. Facilitate collaboration and knowledge exchange with EU institutions, regional bodies, and other stakeholders in Brussels and</t>
+          <t>The role will include the following objectives: Provide technical expertise and operational support to GFDRR’s Disaster-FCV Nexus program, focusing on FCV-sensitive disaster risk management and climate resilience. Strengthen GFDRR’s analytical, advisory, and partnership work on the disaster-FCV nexus, including knowledge generation, policy dialogue, and capacity building. Facilitate collaboration and knowledge exchange with EU institutions, regional bodies, and other stakeholders in Brussels and beyond.</t>
         </is>
       </c>
       <c r="P59" s="6" t="inlineStr">
@@ -5728,7 +5749,7 @@
       </c>
       <c r="Q59" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[climate_risk] The job description mentions climate change, disaster risk management, and climate resilience, which are all related to climate risk. The role also involves working with the Global Facility for Disaster Reduction and Recovery (GFDRR), which is a global partnership that helps low- and </t>
+          <t>The job description mentions climate change, disaster risk management, and climate resilience, which are all related to climate risk. The role also involves working with the Global Facility for Disaster Reduction and Recovery (GFDRR), which is a global partnership that helps low- and middle-income countries better understand and reduce their vulnerability to natural hazards and climate change.</t>
         </is>
       </c>
       <c r="R59" s="2" t="inlineStr">
@@ -5811,17 +5832,17 @@
       </c>
       <c r="O60" s="6" t="inlineStr">
         <is>
-          <t>We are looking for a skilled quantitative professional, who may combine working on Belgian and European financial institutions. The ability to drive work forward to a conclusion, to find pragmatic solutions to complex problems and to explain and document them convincingly, are key factors in order to be successful in this role. Typical projects you will be involved in: Participate in, and lead Risk engagements, with the focus credit risk modeling, including the link with accounting (e.g. IFRS 9)</t>
+          <t>We are looking for a skilled quantitative professional, who may combine working on Belgian and European financial institutions. The ability to drive work forward to a conclusion, to find pragmatic solutions to complex problems and to explain and document them convincingly, are key factors in order to be successful in this role. Typical projects you will be involved in: Participate in, and lead Risk engagements, with the focus credit risk modeling, including the link with accounting (e.g. IFRS 9) You participate in engagements in the Risk practice, in the quantitative space, both from an advisory and an assurance perspective Support banks in preparing for regulatory reviews, or help them mitigate model weaknesses Assist banks in any stage of the model life cycle (developing new models, backtesting, independent validation of credit models, …) In the context of market risk and (derivative) valuation models typical tasks are: Develop and apply EY tools &amp; models Participate to model development and model validation exercises Identify new areas for further development of EY tools &amp; models, including the innovative application of machine learning in this application domain Assess the impact of climate risk and ESG considerations in general on market risk and (derivative) valuation model Explore and exploit the potential of alternative data and machine learning techniques to help financial institutions bring their credit modelling to the next level Investigate the impact of climate risk and ESG aspects in general on credit risk Contribute to the standardization and automation of the model development and model validation process Understand our full range of service offerings and actively identify and develop new opportunities to address emerging client needs You coordinate the workload in various projects, and develop productive working relationships with internal and external clients You prepare concise, complete and convincing reports on the work done, and present it to more senior colleagues and clients You act as a team member, coaching and supervising junior staff, seeking guidance from senior colleagues as needed, and keeping everybody informed on the progress of the assignment.</t>
         </is>
       </c>
       <c r="P60" s="6" t="inlineStr">
         <is>
-          <t>Solid understanding of quantitative modeling techniques and practical experience with valuation of complex instruments (e.g. derivative, illiquid bonds) and/or market risk (e.g. FRTB, IRRBB, VAR models) is mandatory Deep understanding of quantitative modeling techniques, with practical experience in</t>
+          <t>Solid understanding of quantitative modeling techniques and practical experience with valuation of complex instruments (e.g. derivative, illiquid bonds) and/or market risk (e.g. FRTB, IRRBB, VAR models) is mandatory Deep understanding of quantitative modeling techniques, with practical experience in credit risk (IRB, IFRS9) and practical experience with derivative pricing in one or more asset classes (FX, rates, equity, …) Knowledge of some key vendor packages, and some frequently used programming languages (R, Matlab, C++, Python, SAS) in the risk and/or valuation domain is mandatory Strong interest in or some initial experience with machine learning algorithms</t>
         </is>
       </c>
       <c r="Q60" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'sustainable finance workgroup' and 'climate risk modelling for financial institutions', indicating a focus on sustainable finance and ESG considerations in the context of financial risk management.</t>
+          <t>The job description mentions 'sustainable finance workgroup' and 'climate risk modelling for financial institutions', indicating a focus on sustainable finance and ESG considerations in the context of financial risk management.</t>
         </is>
       </c>
       <c r="R60" s="2" t="inlineStr">
@@ -5912,7 +5933,7 @@
       </c>
       <c r="Q61" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions 'atmospheric perils', 'extreme weather events', 'changing climate', and 'climate modelling' which are all related to climate risk.</t>
+          <t>The job description mentions 'atmospheric perils', 'extreme weather events', 'changing climate', and 'climate modelling' which are all related to climate risk.</t>
         </is>
       </c>
       <c r="R61" s="2" t="inlineStr">
@@ -5995,17 +6016,17 @@
       </c>
       <c r="O62" s="6" t="inlineStr">
         <is>
-          <t>The intern will have the opportunity to be involved in the following duties: Supporting different research works conducted by the team; Analyzing policy documents and legal texts, to collect and review data; Assisting with research and fact-checking for International IDEA materials and background information; Assisting in the organization and the follow-up of conferences, events and activities, including assisting with reporting, note-taking and some logistical tasks; Providing desk research and</t>
+          <t>The intern will have the opportunity to be involved in the following duties: Supporting different research works conducted by the team; Analyzing policy documents and legal texts, to collect and review data; Assisting with research and fact-checking for International IDEA materials and background information; Assisting in the organization and the follow-up of conferences, events and activities, including assisting with reporting, note-taking and some logistical tasks; Providing desk research and contributing to the conceptualization of other new and ongoing projects within the teams; Developing outreach, media and communications materials; Actively incorporating a gender and inclusion perspective in all activities; Assisting with Ad-hoc projects and tasks.</t>
         </is>
       </c>
       <c r="P62" s="6" t="inlineStr">
         <is>
-          <t>Strong analytical, drafting, editorial and problem-solving skills. Ability to appreciate diversity and work as part of a team in such an environment. Ability to assess, manage and structure information. Strong interpersonal and communication skills. Good knowledge of Microsoft Office suite. Knowledg</t>
+          <t>Strong analytical, drafting, editorial and problem-solving skills. Ability to appreciate diversity and work as part of a team in such an environment. Ability to assess, manage and structure information. Strong interpersonal and communication skills. Good knowledge of Microsoft Office suite. Knowledge of information management systems is an asset.</t>
         </is>
       </c>
       <c r="Q62" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions 'sustainable democracy', 'climate change and democracy', and 'democracy and inclusion', which are related to environmental, social, and governance topics, but the primary focus is on democratic institutions and processes, making it a better fit for the gene</t>
+          <t>The job description mentions 'sustainable democracy', 'climate change and democracy', and 'democracy and inclusion', which are related to environmental, social, and governance topics, but the primary focus is on democratic institutions and processes, making it a better fit for the general ESG profile.</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr">
@@ -6088,7 +6109,7 @@
       </c>
       <c r="O63" s="6" t="inlineStr">
         <is>
-          <t>Our Sustainability Climate Change and Risk covers several disciplines including; Energy Transition &amp; Markets, Decarbonisation and Physical Risk Strategy. As a Graduate Consultant in our Sustainability, Climate Change &amp; Risk team, team at Aurecon, you’ll: Own your career while growing your skills through workshops and self-paced learning, Apply your analytical and problem-solving skills on live client projects, Work with diverse, multidisciplinary teams across engineering, advisory, and design, L</t>
+          <t>Our Sustainability Climate Change and Risk covers several disciplines including; Energy Transition &amp; Markets, Decarbonisation and Physical Risk Strategy. As a Graduate Consultant in our Sustainability, Climate Change &amp; Risk team, team at Aurecon, you’ll: Own your career while growing your skills through workshops and self-paced learning, Apply your analytical and problem-solving skills on live client projects, Work with diverse, multidisciplinary teams across engineering, advisory, and design, Learn from industry experts and mentors through hands-on guidance, Connect through Limelight, our early careers network</t>
         </is>
       </c>
       <c r="P63" s="6" t="inlineStr">
@@ -6098,7 +6119,7 @@
       </c>
       <c r="Q63" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions 'Sustainability Climate Change and Risk', 'Energy Transition &amp; Markets', 'Decarbonisation and Physical Risk Strategy', which are all related to climate risk and sustainability.</t>
+          <t>The job description mentions 'Sustainability Climate Change and Risk', 'Energy Transition &amp; Markets', 'Decarbonisation and Physical Risk Strategy', which are all related to climate risk and sustainability.</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr">
@@ -6185,7 +6206,7 @@
       </c>
       <c r="O64" s="6" t="inlineStr">
         <is>
-          <t>The Associate Director, Climate Change and Environment supports the growth of Tetra Tech International Development’s climate portfolio across Australia and the Indo‑Pacific through business development, technical advisory and practice support. Key responsibilities include: Lead and support business development for climate change and environment opportunities, including proposals, positioning and client engagement, Design and shape integrated climate resilience solutions across sectors such as su</t>
+          <t>The Associate Director, Climate Change and Environment supports the growth of Tetra Tech International Development’s climate portfolio across Australia and the Indo‑Pacific through business development, technical advisory and practice support. Key responsibilities include: Lead and support business development for climate change and environment opportunities, including proposals, positioning and client engagement, Design and shape integrated climate resilience solutions across sectors such as sustainable infrastructure, agriculture, livelihoods, disaster preparedness and natural resource management, Provide senior technical leadership across investment design, implementation, technical assistance and evaluation, Build and maintain strong relationships with DFAT, regional partners, donors and industry stakeholders, Contribute to the delivery and oversight of complex programs, ensuring quality, compliance and commercial rigour, Support practice growth through people leadership, collaboration, and thought leadership activities</t>
         </is>
       </c>
       <c r="P64" s="6" t="inlineStr">
@@ -6195,7 +6216,7 @@
       </c>
       <c r="Q64" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate change, climate resilience, disaster risk reduction, and climate‑inclusive development, which are all relevant to the climate risk profile</t>
+          <t>The job description mentions climate change, climate resilience, disaster risk reduction, and climate‑inclusive development, which are all relevant to the climate risk profile</t>
         </is>
       </c>
       <c r="R64" s="2" t="inlineStr">
@@ -6282,17 +6303,17 @@
       </c>
       <c r="O65" s="6" t="inlineStr">
         <is>
-          <t>Lead a team of 5-6 Senior consultants, analysts for engagement execution and delivery. Showcase exceptional project management abilities and foster a collaborative environment and accountability among team members on engagements. Demonstrate deep technical expertise and industry knowledge, particularly in financial products with a focus on lending solutions. Design, assessment, and benchmarking of financial risk management policies, frameworks, methodologies covering a range of risk domains such</t>
+          <t>Lead a team of 5-6 Senior consultants, analysts for engagement execution and delivery. Showcase exceptional project management abilities and foster a collaborative environment and accountability among team members on engagements. Demonstrate deep technical expertise and industry knowledge, particularly in financial products with a focus on lending solutions. Design, assessment, and benchmarking of financial risk management policies, frameworks, methodologies covering a range of risk domains such as credit risk, market risk, operational risk, liquidity risk, climate risk, and integrated risk topics viz., capital adequacy and stress testing measurement methodologies in financial institutions (FI). Stay abreast of market trends and challenges in the financial services sector to understand client needs and industry dynamics. Understand EY and its service lines and actively assess what the firm can deliver to serve clients. Monitor project progress, manage risks, and effectively communicate status, issues, and priorities to key stakeholders to ensure successful outcomes. Review, analyze, and validate the work completed by junior team members to ensure accuracy and quality. Adapt to projects involving model audits, validation, and development, demonstrating flexibility and domain knowledge</t>
         </is>
       </c>
       <c r="P65" s="6" t="inlineStr">
         <is>
-          <t>Advanced technical skills, with proficiency in Python, SAS, SQL, R, and Excel. Excellent Oral and written communication and presentation skills. Strong documentation skills, with the ability to quickly grasp complex concepts and present them clearly in documents or presentations. Strong multi-taskin</t>
+          <t>Advanced technical skills, with proficiency in Python, SAS, SQL, R, and Excel. Excellent Oral and written communication and presentation skills. Strong documentation skills, with the ability to quickly grasp complex concepts and present them clearly in documents or presentations. Strong multi-tasking skills with demonstrated ability to manage expectations and deliver high quality results under tight deadlines and minimal supervision. In-depth knowledge of Credit risk model development, validation, audit and/or implementation of the banking book portfolio. Solid understanding of Risk analytics methodologies.</t>
         </is>
       </c>
       <c r="Q65" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions 'climate risk' as one of the risk domains, and also mentions 'experience in climatic risk space preferably in the areas of stress testing /scenario designing', indicating that the role involves working with climate-related risks.</t>
+          <t>The job description mentions 'climate risk' as one of the risk domains, and also mentions 'experience in climatic risk space preferably in the areas of stress testing /scenario designing', indicating that the role involves working with climate-related risks.</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
@@ -6379,17 +6400,17 @@
       </c>
       <c r="O66" s="6" t="inlineStr">
         <is>
-          <t>The Team Leader, Sustainable Finance Operations at Intercontinental Exchange (ICE) plays a critical leadership role in managing and developing a high-performing team of ESG data professionals based in Hyderabad. This position ensures the delivery of accurate, comprehensive, and timely Environmental, Social, and Governance (ESG) data to support ICE Climate products and global ESG reporting standards. * Lead and develop a team of 15+ Associates and Analysts, overseeing resource planning, performan</t>
+          <t>The Team Leader, Sustainable Finance Operations at Intercontinental Exchange (ICE) plays a critical leadership role in managing and developing a high-performing team of ESG data professionals based in Hyderabad. This position ensures the delivery of accurate, comprehensive, and timely Environmental, Social, and Governance (ESG) data to support ICE Climate products and global ESG reporting standards. * Lead and develop a team of 15+ Associates and Analysts, overseeing resource planning, performance management, and professional growth. * Ensure the accuracy, completeness, and timely delivery of ESG data by analyzing and validating information from diverse sources. * Monitor ESG market trends and apply insights to enhance data quality and client deliverables. * Drive workflow efficiencies and implement process improvements to optimize accuracy and productivity. * Collaborate with global teams to standardize processes and maintain consistency in data quality. * Provide expert support to ESG product users and resolve inquiries promptly. * Identify and address data quality issues, recommending corrective actions as needed. * Contribute to strategic and ad hoc projects focused on operational excellence and data enhancement. * Prepare and present progress reports, including data visualizations, for leadership and stakeholders. * Foster a culture aligned with ICE values, with a strong emphasis on driving a high-performance culture. * Continuously identify and implement improvements to team and operational efficiency, supporting ongoing operational excellence. * Proactively seek and implement opportunities to leverage AI and automation to maximize efficiency and achieve more with less. * Design and deploy smart systems and automated workflows to streamline operations and enhance data quality.</t>
         </is>
       </c>
       <c r="P66" s="6" t="inlineStr">
         <is>
-          <t>Proficiency in SQL, Macros, and Advanced Excel; experience with Power BI, Tableau, or similar tools preferred. Strong analytical, problem-solving, and communication skills. Ability to align team objectives with organisational goals and deliver high-quality results. Reliability, flexibility, and atte</t>
+          <t>Proficiency in SQL, Macros, and Advanced Excel; experience with Power BI, Tableau, or similar tools preferred. Strong analytical, problem-solving, and communication skills. Ability to align team objectives with organisational goals and deliver high-quality results. Reliability, flexibility, and attention to detail. Demonstrated experience in leveraging AI and automation to improve operational efficiency. Proven track record in building and deploying smart systems and automated workflows within data operations.</t>
         </is>
       </c>
       <c r="Q66" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions ESG data, ESG reporting standards, and ESG product users, which are all relevant to sustainable finance. The role also involves working with ESG content, regulatory frameworks, and capital markets, which are key aspects of sustainable finance.</t>
+          <t>The job description mentions ESG data, ESG reporting standards, and ESG product users, which are all relevant to sustainable finance. The role also involves working with ESG content, regulatory frameworks, and capital markets, which are key aspects of sustainable finance.</t>
         </is>
       </c>
       <c r="R66" s="2" t="inlineStr">
@@ -6468,17 +6489,17 @@
       </c>
       <c r="O67" s="6" t="inlineStr">
         <is>
-          <t>As a member of the Global Center of excellence the Presales technical lead will help customers to make technology decisions, implement best practices for asset management and overall facilitate transforming buildings into smart connected entities. Develop and implement pre-sales strategies that align with the organization’s business goals &amp; targets. Review opportunity inputs, requirements and specifications; should be able to capture the Digital Solution scope and understand the complete require</t>
+          <t>As a member of the Global Center of excellence the Presales technical lead will help customers to make technology decisions, implement best practices for asset management and overall facilitate transforming buildings into smart connected entities. Develop and implement pre-sales strategies that align with the organization’s business goals &amp; targets. Review opportunity inputs, requirements and specifications; should be able to capture the Digital Solution scope and understand the complete requirements of the customer. Drive RFP/RFI responses, preparing technical solution writeups, compliance matrices, BoQs, Hardware sizing calculations, and architecture diagrams tailored to customer use cases across global markets. Collaborate with cross-functional teams, including sales, marketing, product management, and engineering, to ensure alignment and effective Solution development. Translate customer pain points and site realities into solution architectures, integrating PLC/SCADA systems and BMS Platforms (Metasys, Niagara, DDC, JACE or similar) with analytics platform, digital twins, and enterprise FM platforms to demonstrate clear business outcomes. Design and present tailored solutions that demonstrate the value and benefits of the digital products and services. Conduct requirement workshops, technical discovery sessions, and PoCs, ensuring alignment of customer expectations with solution capabilities, integration pathways, data models, KPIs, and future‑state architecture. Lead and mentor design teams during solution shaping; guiding them on OT and IOT protocols, data ingestion, middleware integration, and standard deployment patterns used during customer demo and Proof of Concepts. Preparation and participation for Gate 0 calls / review meetings with JC Branch sales team for technical queries, scope clarifications, compliance and record minutes of meeting. Understand inter-dependence and lead cross-functional teams towards technical solutions for multi-tiered systems. Clarify, prioritize and drive solution commitments as well as establish and maintain clear chains of accountability. Adherence to proposal &amp; estimation process and guideline to select proper Digital Solution Applications/offering to come up with the technical solution. Preparing technical proposals, cost estimates ensuring it meet the customer requirement and provide competitive advantage to JCI. Develop solutions specific dashboards, reporting frameworks, and data modeling strategies as part of presales demonstrations, highlighting portfolio‑level insights and operational benefits. Provide technical leadership to coordinate, prioritize and deliver proposal, commercials in pre-sales process. Articulate goals, desired outcomes, risks/issues and mitigation plan clearly in pre-sales process. Clearly qualify out of the box solutions and possible customizations needed. Provide feedback to product management and development teams regarding customer needs and market demands</t>
         </is>
       </c>
       <c r="P67" s="6" t="inlineStr">
         <is>
-          <t>Strong technical aptitude and ability to quickly learn new products and technologies. Excellent communication and interpersonal skills. Proficiency in using Integrated software and digital communication tools. Ability to present complex technical information in a clear and concise manner. Strong pro</t>
+          <t>Strong technical aptitude and ability to quickly learn new products and technologies. Excellent communication and interpersonal skills. Proficiency in using Integrated software and digital communication tools. Ability to present complex technical information in a clear and concise manner. Strong problem-solving skills and customer-oriented mindset. Ability to work independently and as part of a team.</t>
         </is>
       </c>
       <c r="Q67" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[clean_energy_adjacent] The job description mentions 'sustainable buildings', 'climate-related innovation', 'net zero carbon emissions', and 'energy management', which are related to environmental sustainability and clean energy. Although the primary focus is on building technologies, the company's </t>
+          <t>The job description mentions 'sustainable buildings', 'climate-related innovation', 'net zero carbon emissions', and 'energy management', which are related to environmental sustainability and clean energy. Although the primary focus is on building technologies, the company's commitment to sustainability and reducing carbon emissions aligns with the clean energy adjacent profile.</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr"/>
@@ -6557,7 +6578,7 @@
       </c>
       <c r="O68" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Develop and manage project finance and cash flow models for renewable energy projects—such as Solar PV, Wind, and BESS—to assess profitability, equity returns, and key risks. Maintain project assumptions documentation, return trackers, and tariff models. Engage cross-functionally with Energy Origination/Markets, Business Development, Project Development, and Operations teams to develop comprehensive business insights and evaluate greenfield renewable energy projects across various technologies. </t>
+          <t>Develop and manage project finance and cash flow models for renewable energy projects—such as Solar PV, Wind, and BESS—to assess profitability, equity returns, and key risks. Maintain project assumptions documentation, return trackers, and tariff models. Engage cross-functionally with Energy Origination/Markets, Business Development, Project Development, and Operations teams to develop comprehensive business insights and evaluate greenfield renewable energy projects across various technologies. Assist in the assessment of Power Purchase Agreement (PPA) structures within utility-scale tender processes and the Commercial and Industrial (C&amp;I) sector. Monitor and interpret trends in the Indian renewable energy market, including regulatory developments and policy frameworks, and assess their implications for project economics. Support fundraising activities by maintaining internal and external data rooms and coordinating responses to investor due diligence requests. Assist with internal and external reporting obligations, including preparing investor presentations, CIMS documentation, and Investment Committee (IC) materials. Exhibit strong interpersonal skills and a collaborative mindset, while also demonstrating the ability to work independently when necessary.</t>
         </is>
       </c>
       <c r="P68" s="6" t="inlineStr">
@@ -6567,7 +6588,7 @@
       </c>
       <c r="Q68" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions renewable energy, solar, wind, and BESS, which are all related to clean energy. The company's focus on transitioning to a carbon-free and sustainable economy also supports this classification.</t>
+          <t>The job description mentions renewable energy, solar, wind, and BESS, which are all related to clean energy. The company's focus on transitioning to a carbon-free and sustainable economy also supports this classification.</t>
         </is>
       </c>
       <c r="R68" s="2" t="inlineStr">
@@ -6646,17 +6667,17 @@
       </c>
       <c r="O69" s="6" t="inlineStr">
         <is>
-          <t>Within the Enterprise Risk Management &amp; Risk Oversight Group in GRC, Enterprise Risk Management &amp; Strategic Initiatives is the independent risk management team that plays a pivotal role in identification, assessment and mitigation of risks affecting the organization. The team’s core responsibility is to design, implement and oversee risk measurement &amp; management frameworks at American Express. Manager – Enterprise Risk Management &amp; Strategic Initiatives will be responsible for providing independ</t>
+          <t>Within the Enterprise Risk Management &amp; Risk Oversight Group in GRC, Enterprise Risk Management &amp; Strategic Initiatives is the independent risk management team that plays a pivotal role in identification, assessment and mitigation of risks affecting the organization. The team’s core responsibility is to design, implement and oversee risk measurement &amp; management frameworks at American Express. Manager – Enterprise Risk Management &amp; Strategic Initiatives will be responsible for providing independent oversight and effective challenge on risk-related matters across the organization. This individual will work closely with senior management and business units to ensure effective identification, assessment and mitigation of risks across the enterprise. The responsibilities include, but not limited to: Assisting in the development of risk management frameworks, policies, and procedures to strengthen enterprise-wide risk practices. Conducting risk assessments on Mergers &amp; Acquisitions (M&amp;A), including due diligence review, integration risk management, and ongoing monitoring. Supporting the development of risk governance framework for Joint Ventures and ensuring controls for heightened risk areas. Performing Climate Risk-related assessments, including end to end measurement of physical and transition risk, scenario analysis, and supporting disclosure requirements. Conducting peer benchmarking and research on industry-wide best practices to recommend enhancements for effective risk management and risk oversight. Supporting a variety of strategic projects within the Enterprise Risk Management team to enhance risk identification and measurement capabilities.</t>
         </is>
       </c>
       <c r="P69" s="6" t="inlineStr">
         <is>
-          <t>Strong understanding of risk management principles, methodologies, frameworks, and regulatory requirements. Strong verbal and written communication skills. Analytical and problem-solving skills, with an ability to analyze data, identify trends, and evaluate risk scenarios effectively. Advanced profi</t>
+          <t>Strong understanding of risk management principles, methodologies, frameworks, and regulatory requirements. Strong verbal and written communication skills. Analytical and problem-solving skills, with an ability to analyze data, identify trends, and evaluate risk scenarios effectively. Advanced proficiency in Excel and PowerPoint. Experience with Python/SAS/R is a plus.</t>
         </is>
       </c>
       <c r="Q69" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions performing Climate Risk-related assessments, including end to end measurement of physical and transition risk, scenario analysis, and supporting disclosure requirements, which directly relates to climate risk management.</t>
+          <t>The job description mentions performing Climate Risk-related assessments, including end to end measurement of physical and transition risk, scenario analysis, and supporting disclosure requirements, which directly relates to climate risk management.</t>
         </is>
       </c>
       <c r="R69" s="2" t="inlineStr">
@@ -6744,12 +6765,12 @@
       </c>
       <c r="P70" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Technical skills: environmental and social impact assessment, environmental and social due diligence, environmental and social management systems. Soft skills: client and commercial capability, proposal development, client negotiation, project scoping, strong track record of repeat business, client </t>
+          <t>Technical skills: environmental and social impact assessment, environmental and social due diligence, environmental and social management systems. Soft skills: client and commercial capability, proposal development, client negotiation, project scoping, strong track record of repeat business, client advocacy, and industry influence.</t>
         </is>
       </c>
       <c r="Q70" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions environmental and social performance management, impact assessment, due diligence, and management systems, which are all relevant to ESG strategy and corporate sustainability.</t>
+          <t>The job description mentions environmental and social performance management, impact assessment, due diligence, and management systems, which are all relevant to ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R70" s="2" t="inlineStr">
@@ -6831,6 +6852,652 @@
         </is>
       </c>
       <c r="O71" s="6" t="inlineStr">
+        <is>
+          <t>* promouvoir et développer les offres ESG (Environnement, Social, Gouvernance)
+* s’assurer de la conformité du Métier aux réglementations en vigueur relatives à la finance durable en Europe
+* Vous serez le spécialiste local de la méthodologie extra-financière (relative aux critères ESG (Environnementaux, Sociaux et de Gouvernance)) couvrant l’ensemble des produits financiers de l’offre de Wealth Management à Luxembourg.
+* Vous contribuerez aux analyses à la structuration des données relatives aux préférences ESG des clients, aux caractéristiques ESG des portefeuilles des clients, afin de communiquer ces analyses aux autres collaborateurs de l’offre, aux conseillers clientèle et au management.
+* Vous contribuerez à la réalisation de reportings commerciaux et réglementaires relatifs à des offres de gestion sous mandat ESG, et interagirez dans ce cadre avec les départements juridique, de conformité, de spécialistes ESG, et de gérants.
+* Vous contribuerez aux groupes de travail de BGL BNP Paribas relatifs à la mise en conformité de la Banque aux réglementations SFDR et MIFID ESG, et aux différents projets liés (développement d’outils, de procédures internes, etc.).
+* Vous contribuerez à d’autres tâches d’analyse de données liées à l’activité globale de l’offre de produits et services, ou à certains types de produits en particulier (private equity, produits structurés, etc).</t>
+        </is>
+      </c>
+      <c r="P71" s="6" t="inlineStr">
+        <is>
+          <t>* Capacité à collaborer / travail d’équipe
+* Rigueur
+* Etre orienté(e) résultats
+* Créativité &amp; Innovation / Capacité à résoudre des problèmes
+* Proactivité
+* Capacité d’analyse
+* Capacité à gérer un projet
+* Capacité à définir des indicateurs de performance pertinents
+* Analyse de données (PowerBI, VBA ou autre)
+* Capacité à communiquer - à l’oral et par écrit (français et anglais)</t>
+        </is>
+      </c>
+      <c r="Q71" s="6" t="inlineStr">
+        <is>
+          <t>The job description mentions ESG (Environnement, Social, Gouvernance), finance durable, SFDR, and MIFID ESG, which are all related to sustainable finance. The job also involves promoting and developing ESG offers, ensuring compliance with regulations, and contributing to the development of sustainable finance within a private bank.</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/bnp-paribas</t>
+        </is>
+      </c>
+      <c r="S71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4387894281</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>sustainable_finance</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>V.I.E. Sustainable Solutions</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Societe Generale Corporate and Investment Banking - SGCIB</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Bank/FI | BFSI</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Stockholm, Stockholm County, Sweden</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>Keyword (6)</t>
+        </is>
+      </c>
+      <c r="O72" s="6" t="inlineStr">
+        <is>
+          <t>Development of the offering of sustainable investment, hedging, and financing solutions for Global Markets Activities. Review and maintain the list of proprietary and external indices embedding ESG criteria; analyze their methodology and create marketing documentation. Monitor and contribute to develop the overall sustainable structured solutions offering. Contribute to assisting the rest of the team in specific quantitative analysis requests. Participate in sustainable finance market studies, monitor the development of the sustainability sector, and monitor regulatory or political developments related to ESG issues. Collaborate with the ESG Advisory team and participate in Societe Generale's cross-functional projects in the field of sustainable finance. Prepare and participate in trainings and committees bringing together the ESG ambassadors within the sales, financial engineering and trading teams of the Global Markets Division. Prepare the newsletters and share with the community any relevant communication related to ESG</t>
+        </is>
+      </c>
+      <c r="P72" s="6" t="inlineStr">
+        <is>
+          <t>Good communication and presentation skills. Management of complex projects. Proficient command of MS Office, notably Excel. Coding in Python is a plus</t>
+        </is>
+      </c>
+      <c r="Q72" s="6" t="inlineStr">
+        <is>
+          <t>The job description mentions sustainable investment, hedging, and financing solutions, ESG criteria, sustainable finance market studies, and ESG advisory team, which are all related to sustainable finance</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/societegenerale-corporate-and-investment-banking</t>
+        </is>
+      </c>
+      <c r="S72" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4388245861</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>carbon_markets</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder (Finance &amp; Investment)</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Asthalaxmi Innovations</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Bank/FI | BFSI</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Guwahati, Assam, India</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>executive</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>5-15 Yrs</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>Keyword (6)</t>
+        </is>
+      </c>
+      <c r="O73" s="6" t="inlineStr">
+        <is>
+          <t>This is a full-time, hybrid (onsite/remote) leadership role in India. You will be the architect of our capital strategy, ensuring that our vision for regenerative agriculture is backed by robust investment. Key Responsibilities: Venture Fundraising: Lead the charge in securing investment from Angel Investors, Venture Capital (VC) firms, and Impact Funds. Project Finance: Secure dedicated funding for large-scale Bamboo agroforestry projects across Northeast India and Bhutan (Green Bonds, Carbon Credit pre-financing). Strategic Leadership: Work alongside the founding team to set objectives, oversee resource allocation, and lead cross-functional teams. Partnership Building: Cultivate high-level relationships with stakeholders, government bodies, and international climate finance institutions. Advocacy: Act as a primary voice for AIPL’s mission, driving both social impact and economic returns.</t>
+        </is>
+      </c>
+      <c r="P73" s="6" t="inlineStr">
+        <is>
+          <t>Fundraising Expertise, Financial &amp; Analytical Rigour, Sales &amp; Marketing Prowess, Climate Intelligence, Leadership, Investment &amp; Finance, Sector Expertise, Regional Insight</t>
+        </is>
+      </c>
+      <c r="Q73" s="6" t="inlineStr">
+        <is>
+          <t>The job description mentions carbon credits, carbon markets, and sustainable development, which are key aspects of the carbon markets profile. The company's focus on generating carbon credits and working on agroforestry projects also aligns with this profile.</t>
+        </is>
+      </c>
+      <c r="R73" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/asthalaxmi</t>
+        </is>
+      </c>
+      <c r="S73" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4387915780</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>carbon_markets</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>VP / Head of Marketing</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Varaha</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Corporate | Environmental</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Gurgaon, Haryana, India</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>executive</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>Keyword (6)</t>
+        </is>
+      </c>
+      <c r="O74" s="6" t="inlineStr">
+        <is>
+          <t>Define and lead Varaha's global brand narrative, position Varaha as a pioneer in climate tech and high integrity carbon markets, build and execute a global PR strategy, develop and execute highly targeted Account Based Marketing (ABM) strategies, oversee the creation of a crisp, scientifically disciplined narrative architecture, develop a strategic conference plan, build and mentor a high performance marketing team, manage agencies, consultants, and creative partners.</t>
+        </is>
+      </c>
+      <c r="P74" s="6" t="inlineStr">
+        <is>
+          <t>Account Based Marketing, field events, PR and communications, partner enablement, storytelling, brand narrative, climate tech, carbon markets, marketing strategy, team leadership, agency management</t>
+        </is>
+      </c>
+      <c r="Q74" s="6" t="inlineStr">
+        <is>
+          <t>The job description mentions carbon removal, carbon markets, climate tech, and high integrity carbon markets, indicating a strong focus on carbon markets and climate-related topics.</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/varaha-carbontech</t>
+        </is>
+      </c>
+      <c r="S74" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4388289654</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>climate_risk</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Atmospheric Scientist/Statistician I</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Verisk</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Corporate | Other</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>mid-senior level</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>Keyword (6)</t>
+        </is>
+      </c>
+      <c r="O75" s="6" t="inlineStr">
+        <is>
+          <t>Improve the accuracy of representing atmospheric perils, contribute to model development, validation, and productization for global clients, support model development using observational and reanalysis products, GCMs, and high-resolution simulations</t>
+        </is>
+      </c>
+      <c r="P75" s="6" t="inlineStr">
+        <is>
+          <t>Spatial statistics, extreme value analysis, atmospheric dynamics, dynamic downscaling methods, Python</t>
+        </is>
+      </c>
+      <c r="Q75" s="6" t="inlineStr">
+        <is>
+          <t>The job description mentions developing catastrophe models for the insurance and reinsurance industries, simulating extreme weather events consistent with a changing climate, and advancing the development of atmospheric peril models, which are all related to climate risk</t>
+        </is>
+      </c>
+      <c r="R75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/verisk-analytics</t>
+        </is>
+      </c>
+      <c r="S75" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4388338436</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>3+ weeks ago</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>eu_taxonomy_sfdr</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>naukri</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>ESG Consultant (Carbon)</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Apex Group</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Asset Manager | BFSI</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>mid-senior level</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>5-15 Yrs</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>Keyword (6)</t>
+        </is>
+      </c>
+      <c r="O76" s="6" t="inlineStr">
+        <is>
+          <t>Conduct comprehensive analyses, including Carbon Emissions Tracking, Carbon Footprint Assessments, Environmental Impact Analyses, Life Cycle Assessments (LCAs), Emissions Reduction Strategies, Climate Policy Development, Advocacy, Climate Modeling, Scenario Planning, and target setting aligned with Science-Based Targets (SBTi). Develop and execute data-driven strategies to assist investment managers and portfolio companies in reducing carbon emissions and setting targets. Lead initiatives to improve the sustainability performance of the Apex Group and promote responsible business practices across the organization. Contribute to the enhancement of existing ESG products and the development of innovative new offerings. Stay informed on global ESG standards and frameworks, ensuring the firm s services meet current and emerging market expectations.</t>
+        </is>
+      </c>
+      <c r="P76" s="6" t="inlineStr">
+        <is>
+          <t>Hands-on experience in carbon footprint analysis, GHG assessment, and climate risk advisory, with strong technical expertise in climate change, SBTi, LCA, ISO 14044/14064, decarbonization strategies, and climate risk modeling. A deep understanding of sustainability challenges across various industry sectors. Proficiency in ESG frameworks, such as SASB, GRI, TCFD, UN PRI, CSRD/NFRD, and SFDR. Strong skills in quantitative and qualitative data collection, analysis, and reporting. Excellent communication and interpersonal skills, with the ability to influence both internal and external stakeholders effectively.</t>
+        </is>
+      </c>
+      <c r="Q76" s="6" t="inlineStr">
+        <is>
+          <t>The job description mentions climate risk, carbon emissions tracking, carbon footprint assessments, GHG assessment, climate risk advisory, and decarbonization strategies, which are all relevant to climate risk. Additionally, the job requires experience in climate change, environmental issues, and sustainability, and proficiency in ESG frameworks such as TCFD, which further supports the classification as climate_risk.</t>
+        </is>
+      </c>
+      <c r="R76" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/adani-electricity</t>
+        </is>
+      </c>
+      <c r="S76" s="3" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-esg-consultant-carbon-apex-fund-services-llp-pune-5-to-15-years-100425504128</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr"/>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>climate_risk</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Senior Specialist Data Management</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Telstra</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Corporate | Other</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>Keyword (5)</t>
+        </is>
+      </c>
+      <c r="O77" s="6" t="inlineStr">
+        <is>
+          <t>Lead and deliver strategic mining advisory projects, provide senior technical expertise, participate in multi-disciplinary project teams, engage senior and executive-level stakeholders, drive business development and industry presence, support team culture, collaboration and wellbeing. Manage and execute environmental and social performance input into feasibility studies, due diligence assignments, ITRs/ITERs, and operational improvement programs.</t>
+        </is>
+      </c>
+      <c r="P77" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Technical skills: environmental and social impact assessment, environmental and social due diligence, environmental and social management systems. Soft skills: client and commercial capability, proposal development, client negotiation, project scoping, strong track record of repeat business, client </t>
+        </is>
+      </c>
+      <c r="Q77" s="6" t="inlineStr">
+        <is>
+          <t>[general_esg] The job description mentions environmental and social performance management, impact assessment, due diligence, and management systems, which are all relevant to ESG strategy and corporate sustainability.</t>
+        </is>
+      </c>
+      <c r="R77" s="2" t="inlineStr"/>
+      <c r="S77" s="3" t="inlineStr">
+        <is>
+          <t>https://au.indeed.com/viewjob?jk=d417c2af5d7b5f69</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr"/>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>climate_risk</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>2027 Graduate Hydrogeologist</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>AECOM</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Consulting | Engineering</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Perth WA</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>Keyword (5)</t>
+        </is>
+      </c>
+      <c r="O78" s="6" t="inlineStr">
         <is>
           <t>* promouvoir et développer les offres ESG (Environnement, Social, Gouvernance)
 * s’assurer de la conformité du Métier aux réglementations en vigueur relatives à la finance durable en Europe
@@ -6838,7 +7505,7 @@
 * Vous contribuerez aux analyses à la structuration des données relatives au</t>
         </is>
       </c>
-      <c r="P71" s="6" t="inlineStr">
+      <c r="P78" s="6" t="inlineStr">
         <is>
           <t>* Capacité à collaborer / travail d’équipe
 * Rigueur
@@ -6851,651 +7518,9 @@
 * Analyse de données (PowerBI,</t>
         </is>
       </c>
-      <c r="Q71" s="6" t="inlineStr">
-        <is>
-          <t>[sustainable_finance] The job description mentions ESG (Environnement, Social, Gouvernance), finance durable, SFDR, and MIFID ESG, which are all related to sustainable finance. The job also involves promoting and developing ESG offers, ensuring compliance with regulations, and contributing to the de</t>
-        </is>
-      </c>
-      <c r="R71" s="2" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/company/bnp-paribas</t>
-        </is>
-      </c>
-      <c r="S71" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4387894281</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>sustainable_finance</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>V.I.E. Sustainable Solutions</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>Societe Generale Corporate and Investment Banking - SGCIB</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>Bank/FI | BFSI</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>Stockholm, Stockholm County, Sweden</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>not applicable</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L72" s="2" t="inlineStr"/>
-      <c r="M72" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N72" s="2" t="inlineStr">
-        <is>
-          <t>Keyword (6)</t>
-        </is>
-      </c>
-      <c r="O72" s="6" t="inlineStr">
-        <is>
-          <t>Development of the offering of sustainable investment, hedging, and financing solutions for Global Markets Activities. Review and maintain the list of proprietary and external indices embedding ESG criteria; analyze their methodology and create marketing documentation. Monitor and contribute to develop the overall sustainable structured solutions offering. Contribute to assisting the rest of the team in specific quantitative analysis requests. Participate in sustainable finance market studies, m</t>
-        </is>
-      </c>
-      <c r="P72" s="6" t="inlineStr">
-        <is>
-          <t>Good communication and presentation skills. Management of complex projects. Proficient command of MS Office, notably Excel. Coding in Python is a plus</t>
-        </is>
-      </c>
-      <c r="Q72" s="6" t="inlineStr">
-        <is>
-          <t>[sustainable_finance] The job description mentions sustainable investment, hedging, and financing solutions, ESG criteria, sustainable finance market studies, and ESG advisory team, which are all related to sustainable finance</t>
-        </is>
-      </c>
-      <c r="R72" s="2" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/company/societegenerale-corporate-and-investment-banking</t>
-        </is>
-      </c>
-      <c r="S72" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4388245861</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>carbon_markets</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>Co-Founder (Finance &amp; Investment)</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>Asthalaxmi Innovations</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr">
-        <is>
-          <t>Bank/FI | BFSI</t>
-        </is>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>Guwahati, Assam, India</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>executive</t>
-        </is>
-      </c>
-      <c r="K73" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="L73" s="2" t="inlineStr">
-        <is>
-          <t>5-15 Yrs</t>
-        </is>
-      </c>
-      <c r="M73" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N73" s="2" t="inlineStr">
-        <is>
-          <t>Keyword (6)</t>
-        </is>
-      </c>
-      <c r="O73" s="6" t="inlineStr">
-        <is>
-          <t>This is a full-time, hybrid (onsite/remote) leadership role in India. You will be the architect of our capital strategy, ensuring that our vision for regenerative agriculture is backed by robust investment. Key Responsibilities: Venture Fundraising: Lead the charge in securing investment from Angel Investors, Venture Capital (VC) firms, and Impact Funds. Project Finance: Secure dedicated funding for large-scale Bamboo agroforestry projects across Northeast India and Bhutan (Green Bonds, Carbon C</t>
-        </is>
-      </c>
-      <c r="P73" s="6" t="inlineStr">
-        <is>
-          <t>Fundraising Expertise, Financial &amp; Analytical Rigour, Sales &amp; Marketing Prowess, Climate Intelligence, Leadership, Investment &amp; Finance, Sector Expertise, Regional Insight</t>
-        </is>
-      </c>
-      <c r="Q73" s="6" t="inlineStr">
-        <is>
-          <t>[carbon_markets] The job description mentions carbon credits, carbon markets, and sustainable development, which are key aspects of the carbon markets profile. The company's focus on generating carbon credits and working on agroforestry projects also aligns with this profile.</t>
-        </is>
-      </c>
-      <c r="R73" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/company/asthalaxmi</t>
-        </is>
-      </c>
-      <c r="S73" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4387915780</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-19</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>carbon_markets</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>VP / Head of Marketing</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>Varaha</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>Corporate | Environmental</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>Gurgaon, Haryana, India</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>internship</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>executive</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L74" s="2" t="inlineStr"/>
-      <c r="M74" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N74" s="2" t="inlineStr">
-        <is>
-          <t>Keyword (6)</t>
-        </is>
-      </c>
-      <c r="O74" s="6" t="inlineStr">
-        <is>
-          <t>Define and lead Varaha's global brand narrative, position Varaha as a pioneer in climate tech and high integrity carbon markets, build and execute a global PR strategy, develop and execute highly targeted Account Based Marketing (ABM) strategies, oversee the creation of a crisp, scientifically disciplined narrative architecture, develop a strategic conference plan, build and mentor a high performance marketing team, manage agencies, consultants, and creative partners.</t>
-        </is>
-      </c>
-      <c r="P74" s="6" t="inlineStr">
-        <is>
-          <t>Account Based Marketing, field events, PR and communications, partner enablement, storytelling, brand narrative, climate tech, carbon markets, marketing strategy, team leadership, agency management</t>
-        </is>
-      </c>
-      <c r="Q74" s="6" t="inlineStr">
-        <is>
-          <t>[carbon_markets] The job description mentions carbon removal, carbon markets, climate tech, and high integrity carbon markets, indicating a strong focus on carbon markets and climate-related topics.</t>
-        </is>
-      </c>
-      <c r="R74" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/company/varaha-carbontech</t>
-        </is>
-      </c>
-      <c r="S74" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4388289654</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>climate_risk</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>Atmospheric Scientist/Statistician I</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>Verisk</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>Corporate | Other</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t>mid-senior level</t>
-        </is>
-      </c>
-      <c r="K75" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L75" s="2" t="inlineStr"/>
-      <c r="M75" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N75" s="2" t="inlineStr">
-        <is>
-          <t>Keyword (6)</t>
-        </is>
-      </c>
-      <c r="O75" s="6" t="inlineStr">
-        <is>
-          <t>Improve the accuracy of representing atmospheric perils, contribute to model development, validation, and productization for global clients, support model development using observational and reanalysis products, GCMs, and high-resolution simulations</t>
-        </is>
-      </c>
-      <c r="P75" s="6" t="inlineStr">
-        <is>
-          <t>Spatial statistics, extreme value analysis, atmospheric dynamics, dynamic downscaling methods, Python</t>
-        </is>
-      </c>
-      <c r="Q75" s="6" t="inlineStr">
-        <is>
-          <t>[climate_risk] The job description mentions developing catastrophe models for the insurance and reinsurance industries, simulating extreme weather events consistent with a changing climate, and advancing the development of atmospheric peril models, which are all related to climate risk</t>
-        </is>
-      </c>
-      <c r="R75" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/verisk-analytics</t>
-        </is>
-      </c>
-      <c r="S75" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4388338436</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>3+ weeks ago</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>eu_taxonomy_sfdr</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>naukri</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>ESG Consultant (Carbon)</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>Apex Group</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>Asset Manager | BFSI</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>Pune</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>mid-senior level</t>
-        </is>
-      </c>
-      <c r="K76" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L76" s="2" t="inlineStr">
-        <is>
-          <t>5-15 Yrs</t>
-        </is>
-      </c>
-      <c r="M76" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N76" s="2" t="inlineStr">
-        <is>
-          <t>Keyword (6)</t>
-        </is>
-      </c>
-      <c r="O76" s="6" t="inlineStr">
-        <is>
-          <t>Conduct comprehensive analyses, including Carbon Emissions Tracking, Carbon Footprint Assessments, Environmental Impact Analyses, Life Cycle Assessments (LCAs), Emissions Reduction Strategies, Climate Policy Development, Advocacy, Climate Modeling, Scenario Planning, and target setting aligned with Science-Based Targets (SBTi). Develop and execute data-driven strategies to assist investment managers and portfolio companies in reducing carbon emissions and setting targets. Lead initiatives to imp</t>
-        </is>
-      </c>
-      <c r="P76" s="6" t="inlineStr">
-        <is>
-          <t>Hands-on experience in carbon footprint analysis, GHG assessment, and climate risk advisory, with strong technical expertise in climate change, SBTi, LCA, ISO 14044/14064, decarbonization strategies, and climate risk modeling. A deep understanding of sustainability challenges across various industry</t>
-        </is>
-      </c>
-      <c r="Q76" s="6" t="inlineStr">
-        <is>
-          <t>[climate_risk] The job description mentions climate risk, carbon emissions tracking, carbon footprint assessments, GHG assessment, climate risk advisory, and decarbonization strategies, which are all relevant to climate risk. Additionally, the job requires experience in climate change, environmental</t>
-        </is>
-      </c>
-      <c r="R76" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/company/adani-electricity</t>
-        </is>
-      </c>
-      <c r="S76" s="3" t="inlineStr">
-        <is>
-          <t>https://www.naukri.com/job-listings-esg-consultant-carbon-apex-fund-services-llp-pune-5-to-15-years-100425504128</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-22</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr"/>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>climate_risk</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>Senior Specialist Data Management</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>Telstra</t>
-        </is>
-      </c>
-      <c r="G77" s="2" t="inlineStr">
-        <is>
-          <t>Corporate | Other</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="I77" s="2" t="inlineStr"/>
-      <c r="J77" s="2" t="inlineStr"/>
-      <c r="K77" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L77" s="2" t="inlineStr"/>
-      <c r="M77" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="N77" s="2" t="inlineStr">
-        <is>
-          <t>Keyword (5)</t>
-        </is>
-      </c>
-      <c r="O77" s="6" t="inlineStr">
-        <is>
-          <t>Lead and deliver strategic mining advisory projects, provide senior technical expertise, participate in multi-disciplinary project teams, engage senior and executive-level stakeholders, drive business development and industry presence, support team culture, collaboration and wellbeing. Manage and execute environmental and social performance input into feasibility studies, due diligence assignments, ITRs/ITERs, and operational improvement programs.</t>
-        </is>
-      </c>
-      <c r="P77" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Technical skills: environmental and social impact assessment, environmental and social due diligence, environmental and social management systems. Soft skills: client and commercial capability, proposal development, client negotiation, project scoping, strong track record of repeat business, client </t>
-        </is>
-      </c>
-      <c r="Q77" s="6" t="inlineStr">
-        <is>
-          <t>[general_esg] The job description mentions environmental and social performance management, impact assessment, due diligence, and management systems, which are all relevant to ESG strategy and corporate sustainability.</t>
-        </is>
-      </c>
-      <c r="R77" s="2" t="inlineStr"/>
-      <c r="S77" s="3" t="inlineStr">
-        <is>
-          <t>https://au.indeed.com/viewjob?jk=d417c2af5d7b5f69</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-22</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr"/>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>climate_risk</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>2027 Graduate Hydrogeologist</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>AECOM</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>Consulting | Engineering</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>Perth WA</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr"/>
-      <c r="J78" s="2" t="inlineStr"/>
-      <c r="K78" s="2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L78" s="2" t="inlineStr"/>
-      <c r="M78" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="N78" s="2" t="inlineStr">
-        <is>
-          <t>Keyword (5)</t>
-        </is>
-      </c>
-      <c r="O78" s="6" t="inlineStr">
-        <is>
-          <t>* promouvoir et développer les offres ESG (Environnement, Social, Gouvernance)
-* s’assurer de la conformité du Métier aux réglementations en vigueur relatives à la finance durable en Europe
-* Vous serez le spécialiste local de la méthodologie extra-financière (relative aux critères ESG (Environnementaux, Sociaux et de Gouvernance)) couvrant l’ensemble des produits financiers de l’offre de Wealth Management à Luxembourg.
-* Vous contribuerez aux analyses à la structuration des données relatives au</t>
-        </is>
-      </c>
-      <c r="P78" s="6" t="inlineStr">
-        <is>
-          <t>* Capacité à collaborer / travail d’équipe
-* Rigueur
-* Etre orienté(e) résultats
-* Créativité &amp; Innovation / Capacité à résoudre des problèmes
-* Proactivité
-* Capacité d’analyse
-* Capacité à gérer un projet
-* Capacité à définir des indicateurs de performance pertinents
-* Analyse de données (PowerBI,</t>
-        </is>
-      </c>
       <c r="Q78" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] Job title contains environmental terminology (Hydrogeologist), indicating relevance to environmental science and water management.</t>
+          <t>Job title contains environmental terminology (Hydrogeologist), indicating relevance to environmental science and water management.</t>
         </is>
       </c>
       <c r="R78" s="2" t="inlineStr"/>
@@ -7562,7 +7587,7 @@
       </c>
       <c r="O79" s="6" t="inlineStr">
         <is>
-          <t>Lead the delivery of SaaS programs focused on mandated regulatory reporting, non-financial disclosures, and sustainability reporting. Ensure alignment across product, engineering, implementation, and client/partner teams while meeting evolving regulatory requirements. Drive end-to-end delivery of regulatory reporting solutions (e.g., compliance, ESG, non-financial reporting) Translate regulatory requirements into actionable program plans and product deliverables Align cross-functional teams (Pro</t>
+          <t>Lead the delivery of SaaS programs focused on mandated regulatory reporting, non-financial disclosures, and sustainability reporting. Ensure alignment across product, engineering, implementation, and client/partner teams while meeting evolving regulatory requirements. Drive end-to-end delivery of regulatory reporting solutions (e.g., compliance, ESG, non-financial reporting) Translate regulatory requirements into actionable program plans and product deliverables Align cross-functional teams (Product, Engineering, Implementation, Data, Partners) Manage timelines, dependencies, risks, and regulatory deadlines Ensure accurate and timely client implementations for mandated reporting Act as the bridge between domain experts, clients, and technical teams Oversee release planning aligned with regulatory changes and updates Monitor data quality, reporting accuracy, and audit readiness Provide stakeholder updates, including leadership and external partners</t>
         </is>
       </c>
       <c r="P79" s="6" t="inlineStr">
@@ -7572,7 +7597,7 @@
       </c>
       <c r="Q79" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions ESG/sustainability reporting solutions, non-financial disclosures, and regulatory reporting, which are all relevant to environmental, social, and governance topics.</t>
+          <t>The job description mentions ESG/sustainability reporting solutions, non-financial disclosures, and regulatory reporting, which are all relevant to environmental, social, and governance topics.</t>
         </is>
       </c>
       <c r="R79" s="2" t="inlineStr"/>
@@ -7639,17 +7664,17 @@
       </c>
       <c r="O80" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nello specifico: si interfaccerà con i focal point all’interno delle società del Gruppo, costruirà modelli per la valutazione di specifici rischi aziendali, ne analizzerà i risultati definendo strategie di mitigazione e azioni correttive dei rischi identificati, e monitorandone il relativo piano di implementazione si interfaccerà con le funzioni Compliance e Internal Audit al fine di mappare, valutare e rappresentare all’Alta Direzione aziendale i rischi rilevanti del Gruppo si occuperà di risk </t>
+          <t>Nello specifico: si interfaccerà con i focal point all’interno delle società del Gruppo, costruirà modelli per la valutazione di specifici rischi aziendali, ne analizzerà i risultati definendo strategie di mitigazione e azioni correttive dei rischi identificati, e monitorandone il relativo piano di implementazione si interfaccerà con le funzioni Compliance e Internal Audit al fine di mappare, valutare e rappresentare all’Alta Direzione aziendale i rischi rilevanti del Gruppo si occuperà di risk assessment integrato (ERM- Enterprise Risk Management) con riferimento a tematiche ESG e climate change, e di progetti di assessment BIA (Business Impact Analysis)</t>
         </is>
       </c>
       <c r="P80" s="6" t="inlineStr">
         <is>
-          <t>modelli di valutazione economica-finanziaria di risk management, metodologie statistiche di analisi dati (modelli probabilistici VaR e PaR), utilizzo di software di analisi quali R Project e Python, conoscenza del software MESA_Procomp, orientamento quantitativo, capacità di sintesi e analisi dei fe</t>
+          <t>modelli di valutazione economica-finanziaria di risk management, metodologie statistiche di analisi dati (modelli probabilistici VaR e PaR), utilizzo di software di analisi quali R Project e Python, conoscenza del software MESA_Procomp, orientamento quantitativo, capacità di sintesi e analisi dei fenomeni, capacità relazionali, conoscenza della lingua inglese (livello B2)</t>
         </is>
       </c>
       <c r="Q80" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions risk assessment integrato (ERM- Enterprise Risk Management) with reference to ESG and climate change, which indicates a focus on climate risk management.</t>
+          <t>The job description mentions risk assessment integrato (ERM- Enterprise Risk Management) with reference to ESG and climate change, which indicates a focus on climate risk management.</t>
         </is>
       </c>
       <c r="R80" s="2" t="inlineStr"/>
@@ -7716,17 +7741,17 @@
       </c>
       <c r="O81" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sarai inserito nel department Risk Management &amp; Policies a riporto del responsabile del team ed avrai un ruolo primario in tutte le attività di analisi e pianificazione in ambito risk management e di progettualità strategiche come la revisione dei processi del credito di Unicredit Leasing SpA. In questo ruolo ti occuperai di svolgere le attività finalizzate a: garantire l’attività di controllo e misurazione dei rischi di credito, dei rischi C&amp;E (Climate &amp; Environmental), dei rischi di liquidità </t>
+          <t>Sarai inserito nel department Risk Management &amp; Policies a riporto del responsabile del team ed avrai un ruolo primario in tutte le attività di analisi e pianificazione in ambito risk management e di progettualità strategiche come la revisione dei processi del credito di Unicredit Leasing SpA. In questo ruolo ti occuperai di svolgere le attività finalizzate a: garantire l’attività di controllo e misurazione dei rischi di credito, dei rischi C&amp;E (Climate &amp; Environmental), dei rischi di liquidità e di mercato e di altre tipologie di rischio rilevanti per il perimetro Leasing, formulando analisi, studi, indagini e simulazioni dettagliate per i principali driver; trasformare ed efficientare i processi aziendali nell’ambito di progetti strategici e per rispondere a richieste di necessità di Business, effettuando test e formulando analisi; assicurare la reportistica e il monitoraggio a presidio del rischio, in continua evoluzione con lo sviluppi strategici di Business, nonché a supporto dei vari Organi Aziendali e alla Capogruppo anche a fronte di specifiche richieste (es. Bankit, ECB,…); effettuando test e formulando analisi provvedere all’elaborazione dei forecast mensili e FY dell’anno in corso sui principali driver di rischio (quali loan loss provisions, dinamiche dei non perfoming, asset quality), gestendo in autonomia il modello previsionale, nonché garantendo il monitoraggio del budget.</t>
         </is>
       </c>
       <c r="P81" s="6" t="inlineStr">
         <is>
-          <t>Forte attitudine analitica, approccio strutturato e orientamento alla risoluzione di problemi complesse Ottime capacità relazionali, comunicative e predisposizione al lavoro in team sia in remoto che in presenza Flessibilità, spirito di iniziativa e desiderio di apprendere in un contesto multidiscip</t>
+          <t>Forte attitudine analitica, approccio strutturato e orientamento alla risoluzione di problemi complesse Ottime capacità relazionali, comunicative e predisposizione al lavoro in team sia in remoto che in presenza Flessibilità, spirito di iniziativa e desiderio di apprendere in un contesto multidisciplinare Ottima conoscenza della lingua italiana e buona padronanza dell’inglese Background scolastico caratterizzato da studi quantitativi Buona conoscenza dei principali tool informatici e familiarità con modelli matematici/statistici applicati alla gestione del rischio</t>
         </is>
       </c>
       <c r="Q81" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions 'rischi C&amp;E (Climate &amp; Environmental)' which indicates that the role involves climate-related risk management, making it a good fit for the climate_risk profile.</t>
+          <t>The job description mentions 'rischi C&amp;E (Climate &amp; Environmental)' which indicates that the role involves climate-related risk management, making it a good fit for the climate_risk profile.</t>
         </is>
       </c>
       <c r="R81" s="2" t="inlineStr"/>
@@ -7798,12 +7823,12 @@
       </c>
       <c r="P82" s="6" t="inlineStr">
         <is>
-          <t>Conoscenza del quadro internazionale di mitigazione e adattamento ai cambiamenti climatici e metodi e strumenti di analisi finanziaria; Conoscenza dei framework di sostenibilità (es. SFDR, Taxonomy Regulation, ECB aspettative, CSR, DNF, PRI ecc.); Competenza tecnica nell'analisi dei dati e dei softw</t>
+          <t>Conoscenza del quadro internazionale di mitigazione e adattamento ai cambiamenti climatici e metodi e strumenti di analisi finanziaria; Conoscenza dei framework di sostenibilità (es. SFDR, Taxonomy Regulation, ECB aspettative, CSR, DNF, PRI ecc.); Competenza tecnica nell'analisi dei dati e dei software di mercato (R/Phyton, SAS, Qlik, SQL, PowerBi); Conoscenza di indici internazionali di sostenibilità come TCFD, GRI, CDP, SBTi e indici ESG</t>
         </is>
       </c>
       <c r="Q82" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[general_esg] The job description mentions working in the Climate &amp; Sustainability team, promoting sustainability, and having knowledge of sustainability frameworks (SFDR, Taxonomy Regulation, CSR, etc.) and international sustainability indices (TCFD, GRI, CDP, SBTi, etc.), which are all related to </t>
+          <t>The job description mentions working in the Climate &amp; Sustainability team, promoting sustainability, and having knowledge of sustainability frameworks (SFDR, Taxonomy Regulation, CSR, etc.) and international sustainability indices (TCFD, GRI, CDP, SBTi, etc.), which are all related to ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R82" s="2" t="inlineStr"/>
@@ -7882,7 +7907,7 @@
       </c>
       <c r="O83" s="6" t="inlineStr">
         <is>
-          <t>Manage the design and delivery of inclusive sport and recreation spaces in Kingston, Help shape sustainable spaces for a growing community, Provide expert leadership and direction across the planning, design and delivery of Council’s active leisure, sport and recreation projects, Oversee a multidisciplinary team to translate Kingston’s strategic targets and community aspirations into inclusive, sustainable and financially responsible infrastructure, Guide projects from concept to completion, ens</t>
+          <t>Manage the design and delivery of inclusive sport and recreation spaces in Kingston, Help shape sustainable spaces for a growing community, Provide expert leadership and direction across the planning, design and delivery of Council’s active leisure, sport and recreation projects, Oversee a multidisciplinary team to translate Kingston’s strategic targets and community aspirations into inclusive, sustainable and financially responsible infrastructure, Guide projects from concept to completion, ensuring each one meets quality, governance, budget and time requirements, Direction and coordination of capital works projects, including sport and recreation facilities, playgrounds and foreshore infrastructure, High quality design outcomes that reflect Council and community priorities, embedding sustainability, accessibility and universal design principles, Asset planning and renewal strategies that support long term community needs and responsible investment, Strong partnerships and open communication with stakeholders, including Councillors, community groups, sporting clubs and government agencies, to deliver shared outcomes, A positive and inclusive team environment that empowers people to perform at their best and celebrate collective success</t>
         </is>
       </c>
       <c r="P83" s="6" t="inlineStr">
@@ -7892,7 +7917,7 @@
       </c>
       <c r="Q83" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions 'sustainable spaces', 'sustainability', and 'environment' in the context of sport and recreation spaces, which aligns with the clean energy adjacent profile, The role also involves managing projects related to sport and recreation facilities, play</t>
+          <t>The job description mentions 'sustainable spaces', 'sustainability', and 'environment' in the context of sport and recreation spaces, which aligns with the clean energy adjacent profile, The role also involves managing projects related to sport and recreation facilities, playgrounds, and foreshore infrastructure, which are related to environmental and conservation topics</t>
         </is>
       </c>
       <c r="R83" s="2" t="inlineStr">
@@ -7981,7 +8006,7 @@
       </c>
       <c r="Q84" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions Renewable Energy/Power-to-X, Life Sciences, and other sectors related to environmental sustainability, which aligns with the clean energy adjacent profile.</t>
+          <t>The job description mentions Renewable Energy/Power-to-X, Life Sciences, and other sectors related to environmental sustainability, which aligns with the clean energy adjacent profile.</t>
         </is>
       </c>
       <c r="R84" s="2" t="inlineStr">
@@ -8064,17 +8089,17 @@
       </c>
       <c r="O85" s="6" t="inlineStr">
         <is>
-          <t>Deliver on the Balance Sheet &amp; Income Statement projections for the Enterprise-wide Stress Testing (EWST) exercises, Carry out the movement analysis &amp; narratives for BS/PnL metrics, Carry out analysis on Capital numbers including CET1, Total capital and compare against Basel and reg requirements, Ensure compliance to EWST procedures, methodologies, and controls, Manage all governance related aspects of the execution of stress testing, Drive process improvements and best practices for more effici</t>
+          <t>Deliver on the Balance Sheet &amp; Income Statement projections for the Enterprise-wide Stress Testing (EWST) exercises, Carry out the movement analysis &amp; narratives for BS/PnL metrics, Carry out analysis on Capital numbers including CET1, Total capital and compare against Basel and reg requirements, Ensure compliance to EWST procedures, methodologies, and controls, Manage all governance related aspects of the execution of stress testing, Drive process improvements and best practices for more efficiency and productivity, Support development and maintenance of underlying models to enhance stress testing methodology, Deliver adequate documentation on stress testing methodology subject to management, model validation, audit &amp; regulatory scrutiny, Deliver on the operational risk framework for the stress test process, Risk Management: Ensure all activity adheres to the Enterprise Risk Management Framework, relevant policies, and standards, Processes: Support the establishment and documentation of all processes and effective controls for the hub team, Governance: Demonstrate an awareness and understanding of the regulatory framework in which SCB operates, and the regulatory requirements and expectations relevant to the role, Regulatory &amp; Business Conduct: Display exemplary conduct and live by the SCB’s Values and Code of Conduct</t>
         </is>
       </c>
       <c r="P85" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exceptional written / verbal communication skills, Flexible and adaptable; able to work in ambiguous situations independently, Display a methodical &amp; meticulous approach to problem solving and root cause analysis, Be a team player and able to work collaboratively with others, Knowledge of Python or </t>
+          <t>Exceptional written / verbal communication skills, Flexible and adaptable; able to work in ambiguous situations independently, Display a methodical &amp; meticulous approach to problem solving and root cause analysis, Be a team player and able to work collaboratively with others, Knowledge of Python or equivalent software packages for data analysis, Knowledge of data visualization tools like Tableau / Power BI, Knowledge of IFRS9 Regulation, Financial Analysis, External Reporting, Effective Communications, Project Management, Process Management</t>
         </is>
       </c>
       <c r="Q85" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions 'Climate Risk Stress Tests: A new area of analysis focussing on the impact of climate change on Banking industry', which indicates that the role is related to climate risk and its impact on the banking industry.</t>
+          <t>The job description mentions 'Climate Risk Stress Tests: A new area of analysis focussing on the impact of climate change on Banking industry', which indicates that the role is related to climate risk and its impact on the banking industry.</t>
         </is>
       </c>
       <c r="R85" s="2" t="inlineStr">
@@ -8163,7 +8188,7 @@
       </c>
       <c r="Q86" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions developing catastrophe models for extreme weather events, simulating the full distribution of possible events consistent with a changing climate, and improving the accuracy of representing atmospheric perils, which are all related to climate risk.</t>
+          <t>The job description mentions developing catastrophe models for extreme weather events, simulating the full distribution of possible events consistent with a changing climate, and improving the accuracy of representing atmospheric perils, which are all related to climate risk.</t>
         </is>
       </c>
       <c r="R86" s="2" t="inlineStr">
@@ -8242,17 +8267,17 @@
       </c>
       <c r="O87" s="6" t="inlineStr">
         <is>
-          <t>Perform independent validation of Advanced IRB / Foundation IRB models including: PD, LGD, EAD, and CCF modelling methodologies, Rating system design and performance, RWA attribution and capital impact assessment, Assess model methodologies and assumptions for diverse wholesale product exposures, Evaluate model conceptual soundness, data representativeness, risk differentiation, and calibration methodology, Review and challenge: Model segmentation, overrides, downturn calibration, and economic c</t>
+          <t>Perform independent validation of Advanced IRB / Foundation IRB models including: PD, LGD, EAD, and CCF modelling methodologies, Rating system design and performance, RWA attribution and capital impact assessment, Assess model methodologies and assumptions for diverse wholesale product exposures, Evaluate model conceptual soundness, data representativeness, risk differentiation, and calibration methodology, Review and challenge: Model segmentation, overrides, downturn calibration, and economic cycle considerations, Treatment of collateral, guarantees, credit mitigants, and default definitions, Regulatory compliance with Basel III/IV IRB requirements and regional supervisory rules, Conduct model performance testing, Prepare high-quality validation documentation, Support regulatory engagements, Partner with Model Development, Credit Policy, Data Governance, and Capital Management teams</t>
         </is>
       </c>
       <c r="P87" s="6" t="inlineStr">
         <is>
-          <t>Experience with Corporate lending, project finance, commercial real estate, private equity exposures, Stress testing frameworks (CCAR/ICAAP) and IRB-to-IFRS 9 model linkages, Regulatory interactions with PRA, ECB, Fed/OCC, OSFI, etc., Ability to articulate quantitative findings to non-technical seni</t>
+          <t>Experience with Corporate lending, project finance, commercial real estate, private equity exposures, Stress testing frameworks (CCAR/ICAAP) and IRB-to-IFRS 9 model linkages, Regulatory interactions with PRA, ECB, Fed/OCC, OSFI, etc., Ability to articulate quantitative findings to non-technical senior stakeholders, Strong technical skills in Python, R, SAS, SQL and knowledge of credit modelling statistics</t>
         </is>
       </c>
       <c r="Q87" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions Climate Risk Modelling experience, which is a key aspect of climate risk management, and the role involves validating IRB models that consider environmental policies, indicating a focus on climate-related risks.</t>
+          <t>The job description mentions Climate Risk Modelling experience, which is a key aspect of climate risk management, and the role involves validating IRB models that consider environmental policies, indicating a focus on climate-related risks.</t>
         </is>
       </c>
       <c r="R87" s="2" t="inlineStr"/>
@@ -8331,7 +8356,7 @@
       </c>
       <c r="O88" s="6" t="inlineStr">
         <is>
-          <t>Your role: We are seeking a Site Construction &amp; EHS Manager for a remediation project in Charleroi. This role combines environmental remediation execution with EHS (Environment, Health &amp; Safety) management on-site. You will be responsible for managing the progress of the site work activities ensuring the safe and compliant execution of remediation activities, coordinating with contractors, and maintaining high standards of environmental and safety performance. Key Responsibilities: Oversee and c</t>
+          <t>Your role: We are seeking a Site Construction &amp; EHS Manager for a remediation project in Charleroi. This role combines environmental remediation execution with EHS (Environment, Health &amp; Safety) management on-site. You will be responsible for managing the progress of the site work activities ensuring the safe and compliant execution of remediation activities, coordinating with contractors, and maintaining high standards of environmental and safety performance. Key Responsibilities: Oversee and coordinate remediation and excavation activities on-site in time and budget, Ensure full compliance with Belgian EHS legislation and internal safety protocols, Conduct EHS training sessions for personnel and contractors, Monitor and report on site progress, safety performance, and environmental impact, Implement and maintain site documentation and control tools, Liaise with project stakeholders, suppliers, and regulatory bodies, Identify risks and propose preventive and corrective actions, Promote a culture of safety and continuous improvement on-site, Support project reporting and documentation for internal and external audits</t>
         </is>
       </c>
       <c r="P88" s="6" t="inlineStr">
@@ -8341,7 +8366,7 @@
       </c>
       <c r="Q88" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions environmental remediation, excavation, waste management, and site remediation, which are related to environmental science and conservation, fitting the clean_energy_adjacent profile.</t>
+          <t>The job description mentions environmental remediation, excavation, waste management, and site remediation, which are related to environmental science and conservation, fitting the clean_energy_adjacent profile.</t>
         </is>
       </c>
       <c r="R88" s="2" t="inlineStr">
@@ -8424,17 +8449,17 @@
       </c>
       <c r="O89" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">As a Senior Specialist, Data Management, you will play a critical role in ensuring Telstra Enterprise and TB-MM have trusted, well-governed customer and identity data that enables digital-first selling, customer self-service, automation and AI at scale. You will lead the definition of data requirements, controls and governance that underpin high-quality customer and identity data across platforms. This includes assessing data readiness and risk early, translating complex data and identity needs </t>
+          <t>As a Senior Specialist, Data Management, you will play a critical role in ensuring Telstra Enterprise and TB-MM have trusted, well-governed customer and identity data that enables digital-first selling, customer self-service, automation and AI at scale. You will lead the definition of data requirements, controls and governance that underpin high-quality customer and identity data across platforms. This includes assessing data readiness and risk early, translating complex data and identity needs into clear, actionable requirements, and embedding preventative controls directly into systems and processes.</t>
         </is>
       </c>
       <c r="P89" s="6" t="inlineStr">
         <is>
-          <t>A practical, outcomes-focused approach, with experience driving exception-only remediation and automation to address root causes and reduce recurring data issues. A strong understanding of enterprise systems and application interconnectedness, including how data flows end-to-end and how changes impa</t>
+          <t>A practical, outcomes-focused approach, with experience driving exception-only remediation and automation to address root causes and reduce recurring data issues. A strong understanding of enterprise systems and application interconnectedness, including how data flows end-to-end and how changes impact customers. A customer-centric mindset, with the ability to use data analysis and insights to improve digital experiences, trust, auditability and operational efficiency.</t>
         </is>
       </c>
       <c r="Q89" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[general_esg] The job description mentions working in the Climate &amp; Sustainability team, promoting sustainability, and having knowledge of sustainability frameworks (SFDR, Taxonomy Regulation, CSR, etc.) and international sustainability indices (TCFD, GRI, CDP, SBTi, etc.), which are all related to </t>
+          <t>The job description does not mention any specific ESG/sustainability topics, such as climate risk, sustainable finance, or carbon markets. The mention of 'sustainability' is in the context of the company's general commitment to sustainability, but it is not directly related to the job role or responsibilities.</t>
         </is>
       </c>
       <c r="R89" s="2" t="inlineStr">
@@ -8517,7 +8542,7 @@
       </c>
       <c r="O90" s="6" t="inlineStr">
         <is>
-          <t>Working as part of our established Geoscience and Remediation Services (GRS) team, you will collaborate with a team of environmental engineers, scientists, hydrogeologists and geologists to provide contaminated land assessment, environmental monitoring, and remediation consulting across a wide range of projects, including those in the oil and gas, mining, Department of Defence, and public sectors. The substantive role involves working on challenging projects across various industries, with a pri</t>
+          <t>Working as part of our established Geoscience and Remediation Services (GRS) team, you will collaborate with a team of environmental engineers, scientists, hydrogeologists and geologists to provide contaminated land assessment, environmental monitoring, and remediation consulting across a wide range of projects, including those in the oil and gas, mining, Department of Defence, and public sectors. The substantive role involves working on challenging projects across various industries, with a primary focus on fieldwork supported by occasional office-based tasks. You will also have the opportunity to work on remote client sites, collaborating with internal teams, subcontractors, and clients. Primarily assist with fieldwork and environmental data collection across a variety of project sites, including short, medium and / or long-term site programs in QLD, and occasionally work interstate to support the national GRS team as opportunities arise. Support surface water and groundwater monitoring programs. Contribute to contamination investigations and remediation projects of varying size and complexity. Collect, handle, and manage environmental samples from a range of media, ensuring safety and sample quality. Support the development of technical environmental reports. Collaborate with offices across Australia and New Zealand, gaining exposure to a wide range of projects and disciplines.</t>
         </is>
       </c>
       <c r="P90" s="6" t="inlineStr">
@@ -8527,7 +8552,7 @@
       </c>
       <c r="Q90" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions environmental science, contaminated land assessment, environmental monitoring, and remediation consulting, which are related to environmental science and conservation, fitting the clean_energy_adjacent profile.</t>
+          <t>The job description mentions environmental science, contaminated land assessment, environmental monitoring, and remediation consulting, which are related to environmental science and conservation, fitting the clean_energy_adjacent profile.</t>
         </is>
       </c>
       <c r="R90" s="2" t="inlineStr">
@@ -8610,7 +8635,7 @@
       </c>
       <c r="O91" s="6" t="inlineStr">
         <is>
-          <t>Working as part of our established Geoscience and Remediation Services (GRS) team, you will collaborate with a team of environmental engineers, scientists, hydrogeologists and geologists to provide contaminated land assessment, environmental monitoring, and remediation consulting across a wide range of projects, including those in the oil and gas, mining, Department of Defence, and public sectors. The substantive role involves working on challenging projects across various industries, with a pri</t>
+          <t>Working as part of our established Geoscience and Remediation Services (GRS) team, you will collaborate with a team of environmental engineers, scientists, hydrogeologists and geologists to provide contaminated land assessment, environmental monitoring, and remediation consulting across a wide range of projects, including those in the oil and gas, mining, Department of Defence, and public sectors. The substantive role involves working on challenging projects across various industries, with a primary focus on fieldwork supported by occasional office-based tasks. You will also have the opportunity to work on remote client sites, collaborating with internal teams, subcontractors, and clients. Primarily assist with fieldwork and environmental data collection across a variety of project sites, including short, medium and / or long-term site programs in QLD, and occasionally work interstate to support the national GRS team as opportunities arise. Support surface water and groundwater monitoring programs. Contribute to contamination investigations and remediation projects of varying size and complexity. Collect, handle, and manage environmental samples from a range of media, ensuring safety and sample quality. Support the development of technical environmental reports. Collaborate with offices across Australia and New Zealand, gaining exposure to a wide range of projects and disciplines.</t>
         </is>
       </c>
       <c r="P91" s="6" t="inlineStr">
@@ -8620,7 +8645,7 @@
       </c>
       <c r="Q91" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions environmental science, contaminated land assessment, environmental monitoring, and remediation consulting, which are related to environmental science and conservation, fitting the clean_energy_adjacent profile.</t>
+          <t>The job description mentions environmental science, contaminated land assessment, environmental monitoring, and remediation consulting, which are related to environmental science and conservation, fitting the clean_energy_adjacent profile.</t>
         </is>
       </c>
       <c r="R91" s="2" t="inlineStr">
@@ -8708,12 +8733,12 @@
       </c>
       <c r="P92" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Excellent quantitative skills, including the ability to identify and interpret data, carry out data analysis, and present findings in a visually compelling way; experience of building and running three-statement financial models; excellent written and presentational skills, including the ability to </t>
+          <t>Excellent quantitative skills, including the ability to identify and interpret data, carry out data analysis, and present findings in a visually compelling way; experience of building and running three-statement financial models; excellent written and presentational skills, including the ability to produce deliverables to a high quality and to present them in a compelling fashion; social and interpersonal skills, with the ability to influence stakeholders and build consensus;</t>
         </is>
       </c>
       <c r="Q92" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions experience in sustainable finance, including climate, development, and/or nature finance, and the company's mission is to address global development challenges through strategic investments that promote sustainable and inclusive economic growth.</t>
+          <t>The job description mentions experience in sustainable finance, including climate, development, and/or nature finance, and the company's mission is to address global development challenges through strategic investments that promote sustainable and inclusive economic growth.</t>
         </is>
       </c>
       <c r="R92" s="2" t="inlineStr">
@@ -8796,7 +8821,7 @@
       </c>
       <c r="O93" s="6" t="inlineStr">
         <is>
-          <t>Assist the EIK team on operational areas, such as: Assisting with the initiation, development, and implementation of Technical Assistance (TA) projects. Supporting contracting processes with TA beneficiaries and consultants, including Know Your Customer (KYC) procedures. Assisting in managing procurements of consultants that execute TA projects and ensuring compliance with procurement procedures. Supporting portfolio and/or program management across different business lines and mandates. Contrib</t>
+          <t>Assist the EIK team on operational areas, such as: Assisting with the initiation, development, and implementation of Technical Assistance (TA) projects. Supporting contracting processes with TA beneficiaries and consultants, including Know Your Customer (KYC) procedures. Assisting in managing procurements of consultants that execute TA projects and ensuring compliance with procurement procedures. Supporting portfolio and/or program management across different business lines and mandates. Contribute to effective communication of impact through: Assisting the development and distribution of newsletters, impact reports, and other communication materials for external stakeholders. Supporting the creation of case studies and impact stories . Coordinating with relevant teams to gather content and updates for communication materials. Support the design and implementation of a data repository for storing and analyzing impact and general data, through: Assisting in data entry, validation, and analysis of impact data. Generating reports and presentations based on collected data for internal and external stakeholders. Communicate key findings and insights from data analysis to support decision-making processes.</t>
         </is>
       </c>
       <c r="P93" s="6" t="inlineStr">
@@ -8806,7 +8831,7 @@
       </c>
       <c r="Q93" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions impact investing, ESG, and sustainable development, which are key concepts in sustainable finance. The company's mission and values also align with sustainable finance principles.</t>
+          <t>The job description mentions impact investing, ESG, and sustainable development, which are key concepts in sustainable finance. The company's mission and values also align with sustainable finance principles.</t>
         </is>
       </c>
       <c r="R93" s="2" t="inlineStr">
@@ -8885,17 +8910,17 @@
       </c>
       <c r="O94" s="6" t="inlineStr">
         <is>
-          <t>As a core function, this team executes sustainable financing solutions aligned with evolving ESG standards and market trends. Execution support - intermediate structuring experience, with a growing level of autonomy. Be responsible of specific tasks for the execution of Sustainable Loan and Bond transactions, under the supervision of a senior team members but with a growing level of autonomy. Advise on transaction execution, by framing, designing and supporting the delivery of sustainable financ</t>
+          <t>As a core function, this team executes sustainable financing solutions aligned with evolving ESG standards and market trends. Execution support - intermediate structuring experience, with a growing level of autonomy. Be responsible of specific tasks for the execution of Sustainable Loan and Bond transactions, under the supervision of a senior team members but with a growing level of autonomy. Advise on transaction execution, by framing, designing and supporting the delivery of sustainable finance mandates. Perform analysis of the ESG profile and strategy of issuers/borrowers and key industry trends, and provide structuring recommendations based on findings. Prepare high-quality presentations to clients. Keep abreast with sustainable finance market developments.</t>
         </is>
       </c>
       <c r="P94" s="6" t="inlineStr">
         <is>
-          <t>Proficient in Office (Excel, PowerPoint). Proficient in Bloomberg. Knowledge in: Financial markets - Structuring; Sustainable Finance &amp; Corporate Social Responsibility - Integration of ESG challenges; Sustainable Finance &amp; Corporate Social Responsibility - Transition towards Low Carbon Economy; Data</t>
+          <t>Proficient in Office (Excel, PowerPoint). Proficient in Bloomberg. Knowledge in: Financial markets - Structuring; Sustainable Finance &amp; Corporate Social Responsibility - Integration of ESG challenges; Sustainable Finance &amp; Corporate Social Responsibility - Transition towards Low Carbon Economy; Data - Business Analytics; Sustainable Finance &amp; Corporate Social Responsibility - Sustainable Savings, investment and Financing; Investment &amp; Wholesale Banking - Debt Capital Market – Bonds; Investment &amp; Wholesale Banking - Debt Capital Market - Loans.</t>
         </is>
       </c>
       <c r="Q94" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'sustainable financing solutions', 'sustainable finance', 'ESG standards', 'sustainable loan and bond transactions', and 'transition to a greener economy', which are all related to sustainable finance and ESG investing.</t>
+          <t>The job description mentions 'sustainable financing solutions', 'sustainable finance', 'ESG standards', 'sustainable loan and bond transactions', and 'transition to a greener economy', which are all related to sustainable finance and ESG investing.</t>
         </is>
       </c>
       <c r="R94" s="2" t="inlineStr">
@@ -8982,7 +9007,7 @@
       </c>
       <c r="O95" s="6" t="inlineStr">
         <is>
-          <t>Execution support, advise on and oversee transaction execution, perform analysis of the ESG profile and strategy of issuers/borrowers, prepare high-quality presentations, keep abreast of key sustainable finance market developments, identify and implement innovative solutions, deepen knowledge on sustainable financing, collect and analyze data, maintain open communication with team members, support junior members, raise awareness on sustainable finance, oversee systematic follow-ups on action poi</t>
+          <t>Execution support, advise on and oversee transaction execution, perform analysis of the ESG profile and strategy of issuers/borrowers, prepare high-quality presentations, keep abreast of key sustainable finance market developments, identify and implement innovative solutions, deepen knowledge on sustainable financing, collect and analyze data, maintain open communication with team members, support junior members, raise awareness on sustainable finance, oversee systematic follow-ups on action points, assist in strengthening the Portugal platform</t>
         </is>
       </c>
       <c r="P95" s="6" t="inlineStr">
@@ -8992,7 +9017,7 @@
       </c>
       <c r="Q95" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions sustainable finance, ESG standards, green economy, and sustainable financing solutions, which are all key aspects of sustainable finance</t>
+          <t>The job description mentions sustainable finance, ESG standards, green economy, and sustainable financing solutions, which are all key aspects of sustainable finance</t>
         </is>
       </c>
       <c r="R95" s="2" t="inlineStr">
@@ -9079,7 +9104,7 @@
       </c>
       <c r="O96" s="6" t="inlineStr">
         <is>
-          <t>Manage and mentor a diverse team of credit risk analytics professionals, fostering a culture of excellence and innovation. Provide direction and oversight across specialized functions including IRB modeling, counterparty credit risk analytics and credit stress testing/provisioning. Develop team members' skills and careers, and promote an inclusive, collaborative environment. Drive the strategic development of the Firms credit risk measurement methodologies. Set the vision for next-generation cre</t>
+          <t>Manage and mentor a diverse team of credit risk analytics professionals, fostering a culture of excellence and innovation. Provide direction and oversight across specialized functions including IRB modeling, counterparty credit risk analytics and credit stress testing/provisioning. Develop team members' skills and careers, and promote an inclusive, collaborative environment. Drive the strategic development of the Firms credit risk measurement methodologies. Set the vision for next-generation credit risk models and analytics tools, ensuring they align with business objectives and emerging risks. Continuously improve model frameworks to enhance risk-adjusted return on capital and support prudent risk taking by the Firm. Lead the Credit Risk Analytics teams response to regulatory initiatives and requirements. Oversee the implementation of frameworks such as Basel III Internal Ratings-Based approaches and stress testing programs. Engage with regulators and internal Model Risk Management on model approvals, validation exercises, and regulatory examinations. Ensure all credit risk models and processes meet the highest standards of compliance and transparency. Work closely with a broad range of stakeholders to integrate credit risk insights into decision-making. Partner with Credit Risk Managers and business units to ensure models adequately capture risks and inform credit decisions and limit setting. Collaborate with Technology teams to drive the development of analytics infrastructure and data capabilities. Provide senior leadership with timely, insightful analysis of credit risk findings and trends. Oversee the end-to-end lifecycle of credit risk models, from design and development through validation, implementation, and ongoing performance monitoring. Chair internal model committees and ensure methodological rigor, robust documentation, and adherence to model risk governance standards. Proactively identify model limitations and guide enhancements or redevelopment as needed. Maintain a strong control environment around model usage and results interpretation. Coordinate with Risk Analytics colleagues and other risk stripes globally to ensure consistency and best practices in risk modeling. Contribute to firm-wide risk initiatives and working groups, sharing expertise in credit risk analytics. Leverage the global footprint of the team by seamlessly integrating efforts between Mumbai, New York, London, and Budapest offices.</t>
         </is>
       </c>
       <c r="P96" s="6" t="inlineStr">
@@ -9089,7 +9114,7 @@
       </c>
       <c r="Q96" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions 'Climate Risk Stress Tests: A new area of analysis focussing on the impact of climate change on Banking industry', which indicates that the role is related to climate risk and its impact on the banking industry.</t>
+          <t>The job description does not explicitly mention ESG, sustainability, climate risk, or other related topics. The focus is on credit risk management and analytics, which is a traditional finance role.</t>
         </is>
       </c>
       <c r="R96" s="2" t="inlineStr">
@@ -9168,17 +9193,17 @@
       </c>
       <c r="O97" s="6" t="inlineStr">
         <is>
-          <t>Lead a team of 5-6 Senior consultants, analysts for engagement execution and delivery. Showcase exceptional project management abilities and foster a collaborative environment and accountability among team members on engagements. Demonstrate deep technical expertise and industry knowledge, particularly in financial products with a focus on lending solutions. Design, assessment, and benchmarking of financial risk management policies, frameworks, methodologies covering a range of risk domains such</t>
+          <t>Lead a team of 5-6 Senior consultants, analysts for engagement execution and delivery. Showcase exceptional project management abilities and foster a collaborative environment and accountability among team members on engagements. Demonstrate deep technical expertise and industry knowledge, particularly in financial products with a focus on lending solutions. Design, assessment, and benchmarking of financial risk management policies, frameworks, methodologies covering a range of risk domains such as credit risk, market risk, operational risk, liquidity risk, climate risk, and integrated risk topics viz., capital adequacy and stress testing measurement methodologies in financial institutions (FI). Stay abreast of market trends and challenges in the financial services sector to understand client needs and industry dynamics. Understand EY and its service lines and actively assess what the firm can deliver to serve clients. Monitor project progress, manage risks, and effectively communicate status, issues, and priorities to key stakeholders to ensure successful outcomes. Review, analyze, and validate the work completed by junior team members to ensure accuracy and quality. Adapt to projects involving model audits, validation, and development, demonstrating flexibility and domain knowledge.</t>
         </is>
       </c>
       <c r="P97" s="6" t="inlineStr">
         <is>
-          <t>Advanced technical skills, with proficiency in Python, SAS, SQL, R, and Excel. Excellent Oral and written communication and presentation skills. Strong documentation skills, with the ability to quickly grasp complex concepts and present them clearly in documents or presentations. Strong multi-taskin</t>
+          <t>Advanced technical skills, with proficiency in Python, SAS, SQL, R, and Excel. Excellent Oral and written communication and presentation skills. Strong documentation skills, with the ability to quickly grasp complex concepts and present them clearly in documents or presentations. Strong multi-tasking skills with demonstrated ability to manage expectations and deliver high quality results under tight deadlines and minimal supervision. Professional certifications such as FRM, CFA, PRM, or SCR. Knowledge of regulatory modeling (BASEL, CCAR, IFRS9) is preferred. Exposure to regulatory stress testing processes around credit risk &amp; ICAAP. Experience in climatic risk space preferably in the areas of stress testing /scenario designing. Exposure to Interest Rate Risk in Banking Book (IRRBB). Experience in data/business intelligence (BI) reporting. Familiarity with machine learning models and their practical applications.</t>
         </is>
       </c>
       <c r="Q97" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate risk, stress testing, and regulatory risk, which are relevant to the climate risk profile. Additionally, the job requires experience in climatic risk space, preferably in the areas of stress testing/scenario designing, which further supports the cl</t>
+          <t>The job description mentions climate risk, stress testing, and regulatory risk, which are relevant to the climate risk profile. Additionally, the job requires experience in climatic risk space, preferably in the areas of stress testing/scenario designing, which further supports the classification as climate_risk.</t>
         </is>
       </c>
       <c r="R97" s="2" t="inlineStr"/>
@@ -9253,7 +9278,7 @@
       </c>
       <c r="O98" s="6" t="inlineStr">
         <is>
-          <t>Team members work on a diverse set of client engagements as part of multi-disciplinary project teams, encompassing subject matter authorities, engagement managers, and others. In this role you will develop and use data and analytical skills to create, review, and deliver analyses to clients, frequently using BlackRock proprietary technology platforms. Candidates must be interested in financial markets and be able to apply creative solutions to solve client objectives and challenges. Team members</t>
+          <t>Team members work on a diverse set of client engagements as part of multi-disciplinary project teams, encompassing subject matter authorities, engagement managers, and others. In this role you will develop and use data and analytical skills to create, review, and deliver analyses to clients, frequently using BlackRock proprietary technology platforms. Candidates must be interested in financial markets and be able to apply creative solutions to solve client objectives and challenges. Team members will gain subject matter expertise about financial institutions and relevant capital markets and sustainability objectives.</t>
         </is>
       </c>
       <c r="P98" s="6" t="inlineStr">
@@ -9263,7 +9288,7 @@
       </c>
       <c r="Q98" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions 'climate risk analytics and advisory' as one of the areas of support, indicating that the role involves working with climate-related risks, which aligns with the climate_risk profile.</t>
+          <t>The job description mentions 'climate risk analytics and advisory' as one of the areas of support, indicating that the role involves working with climate-related risks, which aligns with the climate_risk profile.</t>
         </is>
       </c>
       <c r="R98" s="2" t="inlineStr"/>
@@ -9356,7 +9381,7 @@
       </c>
       <c r="Q99" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions 'climate risks' under the 'Emerging Risks' section, indicating that the role involves identifying, measuring, and monitoring climate-related risks.</t>
+          <t>The job description mentions 'climate risks' under the 'Emerging Risks' section, indicating that the role involves identifying, measuring, and monitoring climate-related risks.</t>
         </is>
       </c>
       <c r="R99" s="2" t="inlineStr">
@@ -9443,17 +9468,17 @@
       </c>
       <c r="O100" s="6" t="inlineStr">
         <is>
-          <t>Lead a team of 5-6 Senior consultants, analysts for engagement execution and delivery. Showcase exceptional project management abilities and foster a collaborative environment and accountability among team members on engagements. Demonstrate deep technical expertise and industry knowledge, particularly in financial products with a focus on lending solutions. Design, assessment, and benchmarking of financial risk management policies, frameworks, methodologies covering a range of risk domains such</t>
+          <t>Lead a team of 5-6 Senior consultants, analysts for engagement execution and delivery. Showcase exceptional project management abilities and foster a collaborative environment and accountability among team members on engagements. Demonstrate deep technical expertise and industry knowledge, particularly in financial products with a focus on lending solutions. Design, assessment, and benchmarking of financial risk management policies, frameworks, methodologies covering a range of risk domains such as credit risk, market risk, operational risk, liquidity risk, climate risk, and integrated risk topics viz., capital adequacy and stress testing measurement methodologies in financial institutions (FI). Stay abreast of market trends and challenges in the financial services sector to understand client needs and industry dynamics. Understand EY and its service lines and actively assess what the firm can deliver to serve clients. Monitor project progress, manage risks, and effectively communicate status, issues, and priorities to key stakeholders to ensure successful outcomes. Review, analyze, and validate the work completed by junior team members to ensure accuracy and quality. Adapt to projects involving model audits, validation, and development, demonstrating flexibility and domain knowledge.</t>
         </is>
       </c>
       <c r="P100" s="6" t="inlineStr">
         <is>
-          <t>Advanced technical skills, with proficiency in Python, SAS, SQL, R, and Excel. Excellent Oral and written communication and presentation skills. Strong documentation skills, with the ability to quickly grasp complex concepts and present them clearly in documents or presentations. Strong multi-taskin</t>
+          <t>Advanced technical skills, with proficiency in Python, SAS, SQL, R, and Excel. Excellent Oral and written communication and presentation skills. Strong documentation skills, with the ability to quickly grasp complex concepts and present them clearly in documents or presentations. Strong multi-tasking skills with demonstrated ability to manage expectations and deliver high quality results under tight deadlines and minimal supervision. Familiarity with machine learning models and their practical applications.</t>
         </is>
       </c>
       <c r="Q100" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate risk, stress testing, and scenario designing, which are relevant to climate risk management. Additionally, the job requires experience in climatic risk space, which further supports the classification as climate_risk.</t>
+          <t>The job description mentions climate risk, stress testing, and scenario designing, which are relevant to climate risk management. Additionally, the job requires experience in climatic risk space, which further supports the classification as climate_risk.</t>
         </is>
       </c>
       <c r="R100" s="2" t="inlineStr">
@@ -9540,17 +9565,17 @@
       </c>
       <c r="O101" s="6" t="inlineStr">
         <is>
-          <t>Collaborate with the global team and clients to analyze ESG data, providing valuable insights to investors and decision-makers. Conduct comprehensive ESG Rating assessments, Gap Analyses, ESG Due Diligence, EU Taxonomy, CSRD assessments, SFDR Compliance, Sustainability-linked loan assessments, and develop Carbon Footprint strategy reports. Utilize deep expertise in ESG and sustainability to deliver high-quality advisory services on ESG reporting, sustainability strategy, and risk management. Sta</t>
+          <t>Collaborate with the global team and clients to analyze ESG data, providing valuable insights to investors and decision-makers. Conduct comprehensive ESG Rating assessments, Gap Analyses, ESG Due Diligence, EU Taxonomy, CSRD assessments, SFDR Compliance, Sustainability-linked loan assessments, and develop Carbon Footprint strategy reports. Utilize deep expertise in ESG and sustainability to deliver high-quality advisory services on ESG reporting, sustainability strategy, and risk management. Stay current with global ESG standards and frameworks, ensuring the firms services meet evolving market expectations. Contribute to the refinement of existing ESG products and the development of new ones. Lead initiatives to enhance the sustainability performance of Apex Group.</t>
         </is>
       </c>
       <c r="P101" s="6" t="inlineStr">
         <is>
-          <t>Proficiency in quantitative and qualitative data collection, analysis, and reporting. Exceptional organizational skills with keen attention to detail. Excellent interpersonal skills with the ability to communicate and influence internal and external stakeholders, including proficiency in video confe</t>
+          <t>Proficiency in quantitative and qualitative data collection, analysis, and reporting. Exceptional organizational skills with keen attention to detail. Excellent interpersonal skills with the ability to communicate and influence internal and external stakeholders, including proficiency in video conferencing, written communication, and presentation. Proficiency in MS Office; knowledge of programming languages is a plus.</t>
         </is>
       </c>
       <c r="Q101" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[general_esg] The job description mentions ESG ratings, ESG reporting, sustainability strategy, and risk management, which are all key aspects of general ESG. Additionally, the job requires expertise in ESG and sustainability, and involves working with ESG data and standards, further supporting the </t>
+          <t>The job description mentions ESG ratings, ESG reporting, sustainability strategy, and risk management, which are all key aspects of general ESG. Additionally, the job requires expertise in ESG and sustainability, and involves working with ESG data and standards, further supporting the classification as general ESG.</t>
         </is>
       </c>
       <c r="R101" s="2" t="inlineStr">
@@ -9621,7 +9646,7 @@
       </c>
       <c r="O102" s="6" t="inlineStr">
         <is>
-          <t>La risorsa Experienced sarà inserita in un team di lavoro, affiancando colleghi senior e occupandosi di: Supporto tecnico-specialistico allo svolgimento delle attività di controllo e verifica relativamente alle operazioni poste in essere in attuazione dei programmi regionali finanziati a livello europeo, aventi l’obiettivo di rafforzare la competitività, l'innovazione, la transizione ecologica e digitale, la mobilità sostenibile, l'istruzione e l'inclusione sociale, riducendo i divari territoria</t>
+          <t>La risorsa Experienced sarà inserita in un team di lavoro, affiancando colleghi senior e occupandosi di: Supporto tecnico-specialistico allo svolgimento delle attività di controllo e verifica relativamente alle operazioni poste in essere in attuazione dei programmi regionali finanziati a livello europeo, aventi l’obiettivo di rafforzare la competitività, l'innovazione, la transizione ecologica e digitale, la mobilità sostenibile, l'istruzione e l'inclusione sociale, riducendo i divari territoriali tramite investimenti in ricerca, imprese, ambiente e infrastrutture. Contribuire alla corretta esecuzione delle attività in cui è coinvolto, apportando le proprie conoscenze tecniche, nel rispetto degli indirizzi e degli obiettivi stabiliti, nonché produrre la documentazione e le analisi a supporto della corretta esecuzione delle attività. Supporto tecnico-specialistico in ambito/materia valutazione ambientale strategica (c.d. VAS) e/o nella verifica del rispetto del principio del DNSH (i.e. non arrecare un danno significativo), nell’ambito dell’attuazione dei programmi regionali</t>
         </is>
       </c>
       <c r="P102" s="6" t="inlineStr">
@@ -9631,7 +9656,7 @@
       </c>
       <c r="Q102" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'Sustainable Finance' team, 'strategie ESG', 'conformità normativa', 'integrazione dei fattori di sostenibilità', and 'evoluzione sostenibile del settore finanziario', which are all related to sustainable finance and ESG investing.</t>
+          <t>The job description mentions 'Sustainable Finance' team, 'strategie ESG', 'conformità normativa', 'integrazione dei fattori di sostenibilità', and 'evoluzione sostenibile del settore finanziario', which are all related to sustainable finance and ESG investing.</t>
         </is>
       </c>
       <c r="R102" s="2" t="inlineStr"/>
@@ -9698,7 +9723,7 @@
       </c>
       <c r="O103" s="6" t="inlineStr">
         <is>
-          <t>Gestirai sfidanti progetti di evoluzione e trasformazione del business dei principali player nei settori Infrastructure, Energy &amp; Utility, Industrial Manufacturing, Pharmaceutical attraverso l’efficientamento e la reingegnerizzazione dei processi interni. Attraverso l'affiancamento a risorse PwC di livello manageriale, la risorsa potrà sviluppare competenze di processo in ambito Risk Management (sia entreprise che per tematiche di business verticali), conoscere l'organizzazione di un progetto st</t>
+          <t>Gestirai sfidanti progetti di evoluzione e trasformazione del business dei principali player nei settori Infrastructure, Energy &amp; Utility, Industrial Manufacturing, Pharmaceutical attraverso l’efficientamento e la reingegnerizzazione dei processi interni. Attraverso l'affiancamento a risorse PwC di livello manageriale, la risorsa potrà sviluppare competenze di processo in ambito Risk Management (sia entreprise che per tematiche di business verticali), conoscere l'organizzazione di un progetto strutturato e collaborare alle attività di project management; conoscere la metodologia internazionale Perform di process &amp; skill improvement. All’interno del gruppo ERM, ti occuperai di: Predisposizione e/o sviluppo di framework ERM (in accordo con le normative ISO 31000, CoSo) e PRM; Identificazione e valutazione, attraverso approcci qualitativi e quantitativi, dei principali rischi ed opportunità aziendali, misurando i potenziali impatti economici-finanziari sul business; Valutazione della flessibilità della strategia di business, contribuendo alle scelte aziendali per la definizione del piano strategico al fine di aumentare la resilienza e garantire nel tempo la generazione del valore; Sviluppo di modelli per l’analisi dei rischi ESG in rispondenza alle principali normative di settore (TCFD, ESRS, EU taxonomy, etc.); Soluzioni di Business Continuity Managament.</t>
         </is>
       </c>
       <c r="P103" s="6" t="inlineStr">
@@ -9708,7 +9733,7 @@
       </c>
       <c r="Q103" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions ESG risk analysis, TCFD, ESRS, and EU taxonomy, which are all related to environmental, social, and governance topics, indicating a relevance to general ESG strategy and corporate sustainability.</t>
+          <t>The job description mentions ESG risk analysis, TCFD, ESRS, and EU taxonomy, which are all related to environmental, social, and governance topics, indicating a relevance to general ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R103" s="2" t="inlineStr"/>
@@ -9775,7 +9800,7 @@
       </c>
       <c r="O104" s="6" t="inlineStr">
         <is>
-          <t>Beleidsontwikkeling en advisering op het gebied van duurzaam beleggen, Monitoring van ESG-dienstverleners en vermogensbeheerders, Monitoring van impactbeleggingsmandaten en vastgoedbeleggingen, Opstellen van klimaatanalyses van vastgoedbedrijven, Begeleiden en coördineren van engagementtrajecten en internationale samenwerkingen, Coördineren van verschillende werk- en stuurgroepen, Organiseren en ondersteunen bij opleidingen en events, Onderzoeken en analyseren van systemische barrières in de int</t>
+          <t>Beleidsontwikkeling en advisering op het gebied van duurzaam beleggen, Monitoring van ESG-dienstverleners en vermogensbeheerders, Monitoring van impactbeleggingsmandaten en vastgoedbeleggingen, Opstellen van klimaatanalyses van vastgoedbedrijven, Begeleiden en coördineren van engagementtrajecten en internationale samenwerkingen, Coördineren van verschillende werk- en stuurgroepen, Organiseren en ondersteunen bij opleidingen en events, Onderzoeken en analyseren van systemische barrières in de internationale vastgoedmarkt</t>
         </is>
       </c>
       <c r="P104" s="6" t="inlineStr">
@@ -9785,7 +9810,7 @@
       </c>
       <c r="Q104" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions ESG, duurzaam beleggen, impactbeleggen, and klimaatanalyses, which are all related to sustainable finance. The company also works with institutionele beleggers and pensioenfondsen to implement ESG in their beleggingsportefeuille.</t>
+          <t>The job description mentions ESG, duurzaam beleggen, impactbeleggen, and klimaatanalyses, which are all related to sustainable finance. The company also works with institutionele beleggers and pensioenfondsen to implement ESG in their beleggingsportefeuille.</t>
         </is>
       </c>
       <c r="R104" s="2" t="inlineStr"/>
@@ -9852,17 +9877,17 @@
       </c>
       <c r="O105" s="6" t="inlineStr">
         <is>
-          <t>Are you ready to lead the charge in groundbreaking clinical studies? As a Global Study Director (GSD), you will play a pivotal role in the Cell Therapy Clinical Operations organization, driving the operational planning and delivery of high-priority and complex clinical studies. Your expertise will ensure the successful execution of clinical trials, managing quality, timelines, budgets, resources, investigational sites, vendors, and key project deliverables. Leading a cross-functional study team,</t>
+          <t>Are you ready to lead the charge in groundbreaking clinical studies? As a Global Study Director (GSD), you will play a pivotal role in the Cell Therapy Clinical Operations organization, driving the operational planning and delivery of high-priority and complex clinical studies. Your expertise will ensure the successful execution of clinical trials, managing quality, timelines, budgets, resources, investigational sites, vendors, and key project deliverables. Leading a cross-functional study team, you will provide direction and guidance to achieve study milestones. Collaborate with internal and external stakeholders to resolve issues and ensure compliance with SOPs, regulatory requirements, and ICH/GCP guidelines. Your leadership will extend to mentoring GSADs and spearheading non-drug programs and improvement projects. Accountabilities Lead and coordinate a cross-functional study team to ensure clinical study progress according to timelines, budget, and quality standards. Contribute to vendor/ESP selection activities and lead operational oversight at the study level. Assist with operational planning for upcoming clinical studies, interfacing with cross-functional partners. Collaborate to establish strategies for increasing efficiency of global study teams. Facilitate communication across functions and provide guidance to study team members. Serve as the primary AZ contact for outsourced studies, ensuring delivery according to agreed standards. Hold accountability for essential study level documents development. Ensure external service providers perform to contracted goals and timelines. Develop and maintain relevant study plans, including risk management planning. Oversee study level performance against plans, milestones, and KPIs. Identify and report quality issues within the study and collaborate to overcome barriers. Ensure Trial Master File completion and compliance with governance controls. Manage study budget through lifecycle and provide progress reports. Ensure studies are inspection-ready at all times. Support professional development of team members. Provide guidance and mentoring to less experienced colleagues. Lead non-drug project work and improvement projects.</t>
         </is>
       </c>
       <c r="P105" s="6" t="inlineStr">
         <is>
-          <t>Essential Skills/Experience University degree or equivalent in medical or biological sciences or discipline associated with clinical research. Proven project management experience and training. At least 7 years of clinical trial experience. At least 3 years of experience in global study leadership a</t>
+          <t>Essential Skills/Experience University degree or equivalent in medical or biological sciences or discipline associated with clinical research. Proven project management experience and training. At least 7 years of clinical trial experience. At least 3 years of experience in global study leadership and team leadership. Demonstrated clinical trial expertise in hematology and/or oncology. Extensive knowledge of ICH-GCP guidelines and clinical research regulatory requirements. Thorough understanding of the cross-functional clinical trial process. Strong strategic and critical thinking abilities. Proven skills in complex problem solving and decision-making. Strong abilities in establishing effective working relationships with senior stakeholders. Demonstrated abilities in mentoring. Excellent communication and interpersonal skills. Ability to manage multiple competing priorities. Experience in external provider oversight and management. Desirable Skills/Experience Advanced degree, masters level education or higher. Project management certification. 5 years of experience in global study leadership and team leadership. Significant hematology/oncology expertise. Expertise in different phases of clinical delivery. Experience with project management software solutions. Cell therapy/CAR-T experience. Global phase 3 study experience.</t>
         </is>
       </c>
       <c r="Q105" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions experience in sustainable finance, including climate, development, and/or nature finance, and the company's mission is to address global development challenges through strategic investments that promote sustainable and inclusive economic growth.</t>
+          <t>Although the company mentions dedication to sustainability, it is in the context of a broader company culture and not directly related to the job responsibilities, requirements, or skills. The job itself is focused on clinical trials and cell therapy, which does not fit into any of the specified ESG/sustainability profiles.</t>
         </is>
       </c>
       <c r="R105" s="2" t="inlineStr"/>
@@ -9934,12 +9959,12 @@
       </c>
       <c r="P106" s="6" t="inlineStr">
         <is>
-          <t>Proven experience in estimating, managing, and controlling personnel cost budgets, as well as in developing financial models and conducting economic evaluations of collective labor agreements. Strong negotiation and conflict management skills. Analytical mindset and practical problem-solving orienta</t>
+          <t>Proven experience in estimating, managing, and controlling personnel cost budgets, as well as in developing financial models and conducting economic evaluations of collective labor agreements. Strong negotiation and conflict management skills. Analytical mindset and practical problem-solving orientation. Excellent communication and influencing skills at all organizational levels.</t>
         </is>
       </c>
       <c r="Q106" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions impact investing, ESG, and sustainable development, which are key concepts in sustainable finance. The company's mission and values also align with sustainable finance principles.</t>
+          <t>The job description does not mention any ESG/sustainability topics, climate change, or environmental issues. The focus is on labor relations, law, and human resources, which does not fit any of the provided profiles.</t>
         </is>
       </c>
       <c r="R106" s="2" t="inlineStr"/>
@@ -10095,17 +10120,17 @@
       </c>
       <c r="O108" s="6" t="inlineStr">
         <is>
-          <t>To support BlackRock’s extensive Australian and global business through the provision of high quality and commercially focused legal advice. To interact with the broader BlackRock global community both in Australia and abroad, reflecting the global interconnectivity of our business. To ensure that BlackRock continues to be regarded by regulators and peers as a company with high compliance standards and strong legal acumen. Provide high quality and commercial legal advice to the Australian busine</t>
+          <t>To support BlackRock’s extensive Australian and global business through the provision of high quality and commercially focused legal advice. To interact with the broader BlackRock global community both in Australia and abroad, reflecting the global interconnectivity of our business. To ensure that BlackRock continues to be regarded by regulators and peers as a company with high compliance standards and strong legal acumen. Provide high quality and commercial legal advice to the Australian business on all aspects of asset management and investments. Act as a primary stakeholder in the product development process, fund registration, exchange admission processes, disclosure, distribution, and marketing. Engage with government, regulators, industry groups, and external counsel. Draft and negotiate contracts, including investment management agreements, investment platform agreements, distribution agreements, custody and administration agreements, and services agreements. Draft papers and present advice to internal stakeholders and committees.</t>
         </is>
       </c>
       <c r="P108" s="6" t="inlineStr">
         <is>
-          <t>Strong technical skills, including statutory and contractual interpretation, research and drafting. Proven ability to deliver high quality legal advice. Excellent verbal and written communication skills, including to confidently present to an audience. Ability to work autonomously and operate in a f</t>
+          <t>Strong technical skills, including statutory and contractual interpretation, research and drafting. Proven ability to deliver high quality legal advice. Excellent verbal and written communication skills, including to confidently present to an audience. Ability to work autonomously and operate in a fast-paced global environment with flexibility to adapt to change. An analytical mindset and ability to innovate and generate new ideas to solve complex problems. High levels of attention to detail and document management skills. Relationship management skills to effectively influence stakeholders and to manage competing stakeholder relationships and priorities.</t>
         </is>
       </c>
       <c r="Q108" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'sustainable finance practices' as one of the current and emerging trends and regulatory priorities, indicating a connection to ESG investing and sustainable finance.</t>
+          <t>The job description mentions 'sustainable finance practices' as one of the current and emerging trends and regulatory priorities, indicating a connection to ESG investing and sustainable finance.</t>
         </is>
       </c>
       <c r="R108" s="2" t="inlineStr">
@@ -10188,17 +10213,17 @@
       </c>
       <c r="O109" s="6" t="inlineStr">
         <is>
-          <t>Prioritize internal and external feedback to build clear and cohesive development roadmaps. Translate desired features into precise specifications for developers using documentation, mock-ups, or visual tools. Follow up on newly released features to ensure they work effectively in real operational settings. Strengthen customer communication around product updates, new features, and enhancements. Support digital product operations and internal improvement initiatives. Establish and improve workfl</t>
+          <t>Prioritize internal and external feedback to build clear and cohesive development roadmaps. Translate desired features into precise specifications for developers using documentation, mock-ups, or visual tools. Follow up on newly released features to ensure they work effectively in real operational settings. Strengthen customer communication around product updates, new features, and enhancements. Support digital product operations and internal improvement initiatives. Establish and improve workflows for proactively collecting user feedback. Document processes and product knowledge to ensure shared understanding across teams. Manage and maintain data pipelines; analyze business and regulatory-related datasets. Learn and apply maritime emissions regulations to ensure our digital processes and data structures meet compliance needs. Support teams and customers in ad hoc tasks, identifying opportunities for automation and efficiency. Act as a point of contact toward the internal IT organization for specifying and coordinating digital projects.</t>
         </is>
       </c>
       <c r="P109" s="6" t="inlineStr">
         <is>
-          <t>Ability to write and run SQL queries. Ability to read and understand Python code (C# familiarity is a plus). Experience analyzing data using APIs and a programming language, preferably Python. Familiarity with Git-based version control tools (Azure DevOps, GitHub). Understanding of Agile/Scrum or si</t>
+          <t>Ability to write and run SQL queries. Ability to read and understand Python code (C# familiarity is a plus). Experience analyzing data using APIs and a programming language, preferably Python. Familiarity with Git-based version control tools (Azure DevOps, GitHub). Understanding of Agile/Scrum or similar digital project methodologies. Interest in specialized emissions software, databases, or registry platforms.</t>
         </is>
       </c>
       <c r="Q109" s="6" t="inlineStr">
         <is>
-          <t>[carbon_markets] The job description mentions experience with maritime emissions regulations, carbon markets, and environmental financial products, which are all relevant to the carbon markets profile.</t>
+          <t>The job description mentions experience with maritime emissions regulations, carbon markets, and environmental financial products, which are all relevant to the carbon markets profile.</t>
         </is>
       </c>
       <c r="R109" s="2" t="inlineStr">
@@ -10281,7 +10306,7 @@
       </c>
       <c r="O110" s="6" t="inlineStr">
         <is>
-          <t>You’ll be at the forefront of our sales function, guiding customers through their home energy transition. You’ll convert inbound inquiries, proactively follow up on leads, and design technical solutions that meet customer needs while exceeding expectations. You’ll also play a key role in maintaining high compliance standards and identifying new business opportunities. Key Responsibilities: Lead Engagement, Follow-Up &amp; Conversion, Customer Support, Solution Design, Compliance &amp; Standards, Busines</t>
+          <t>You’ll be at the forefront of our sales function, guiding customers through their home energy transition. You’ll convert inbound inquiries, proactively follow up on leads, and design technical solutions that meet customer needs while exceeding expectations. You’ll also play a key role in maintaining high compliance standards and identifying new business opportunities. Key Responsibilities: Lead Engagement, Follow-Up &amp; Conversion, Customer Support, Solution Design, Compliance &amp; Standards, Business Development, CRM &amp; Reporting, Industry Presence, Team Collaboration</t>
         </is>
       </c>
       <c r="P110" s="6" t="inlineStr">
@@ -10291,7 +10316,7 @@
       </c>
       <c r="Q110" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions renewable energy solutions, heat pumps, solar panels, and carbon-neutral home energy solutions, which are all related to clean energy and environmental sustainability.</t>
+          <t>The job description mentions renewable energy solutions, heat pumps, solar panels, and carbon-neutral home energy solutions, which are all related to clean energy and environmental sustainability.</t>
         </is>
       </c>
       <c r="R110" s="2" t="inlineStr">
@@ -10384,7 +10409,7 @@
       </c>
       <c r="Q111" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions sustainable development, climate change, and environmental health, which are related to ESG topics. Although the role is not explicitly focused on ESG, the context suggests that it may involve working on projects that contribute to sustainable development a</t>
+          <t>The job description mentions sustainable development, climate change, and environmental health, which are related to ESG topics. Although the role is not explicitly focused on ESG, the context suggests that it may involve working on projects that contribute to sustainable development and environmental health.</t>
         </is>
       </c>
       <c r="R111" s="2" t="inlineStr">
@@ -10477,7 +10502,7 @@
       </c>
       <c r="Q112" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions working with teams focused on sustainable development, climate change, and environmental issues, which aligns with the general ESG profile.</t>
+          <t>The job description mentions working with teams focused on sustainable development, climate change, and environmental issues, which aligns with the general ESG profile.</t>
         </is>
       </c>
       <c r="R112" s="2" t="inlineStr">
@@ -10556,17 +10581,17 @@
       </c>
       <c r="O113" s="6" t="inlineStr">
         <is>
-          <t>Identify focus countries/locations, strategic partners, outward delegation itineraries, event formats; plan B2B/B2G meetings and prepare talking points &amp; press notes. Coordinate with Invest India, Chambers, Missions; build investor lists, outreach plans, and track conversion. Draft invitation, program scripts, and proceedings; prepare participation summaries. Prepare project/sector/infrastructure profiles, brochures/flyers, web &amp; social content; support monthly newsletters. Facilitate meetings w</t>
+          <t>Identify focus countries/locations, strategic partners, outward delegation itineraries, event formats; plan B2B/B2G meetings and prepare talking points &amp; press notes. Coordinate with Invest India, Chambers, Missions; build investor lists, outreach plans, and track conversion. Draft invitation, program scripts, and proceedings; prepare participation summaries. Prepare project/sector/infrastructure profiles, brochures/flyers, web &amp; social content; support monthly newsletters. Facilitate meetings with inward delegations; ensure documentation of minutes, outcomes, and actions for all delegations.</t>
         </is>
       </c>
       <c r="P113" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mandatory skill sets: Investor targeting &amp; engagement; event/roadshow planning; strong writing for talking points, invites, briefs, and press notes; comfort with collaboration tools; data-driven outreach tracking. Preferred skill sets: Quality &amp; timeliness of event concept notes; roadshow execution </t>
+          <t>Mandatory skill sets: Investor targeting &amp; engagement; event/roadshow planning; strong writing for talking points, invites, briefs, and press notes; comfort with collaboration tools; data-driven outreach tracking. Preferred skill sets: Quality &amp; timeliness of event concept notes; roadshow execution &amp; meeting conversions; quality of collaterals; completeness of proceedings reports; responsiveness to client instructions. Required Skills: Data Analysis</t>
         </is>
       </c>
       <c r="Q113" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions working with clients on transformation in Government with a focus on Sustainability, Climate Change, and Environment, indicating a role related to ESG strategy and corporate sustainability.</t>
+          <t>The job description mentions working with clients on transformation in Government with a focus on Sustainability, Climate Change, and Environment, indicating a role related to ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R113" s="2" t="inlineStr"/>
@@ -10645,7 +10670,7 @@
       </c>
       <c r="O114" s="6" t="inlineStr">
         <is>
-          <t>Research Leadership: Taking forward RAND Europe’s successful research track record in technology policy research, developing and leading a varied portfolio of research projects and expanding into new areas of work. Providing thought leadership on technology policy issues. Mentoring research staff and facilitating development of others' project management and methodological skills. Taking a leading role in ensuring that RAND Europe’s research has a positive impact within policy communities. Busin</t>
+          <t>Research Leadership: Taking forward RAND Europe’s successful research track record in technology policy research, developing and leading a varied portfolio of research projects and expanding into new areas of work. Providing thought leadership on technology policy issues. Mentoring research staff and facilitating development of others' project management and methodological skills. Taking a leading role in ensuring that RAND Europe’s research has a positive impact within policy communities. Business development: Contributing to the work of SET, through contributing to or supporting the delivery of research group target revenues and sales by securing funding for research and supporting others in doing so. Co-ordinating, managing and supporting a portfolio of business development initiatives including leading and supporting bid and proposal activity, often as multi-partner proposals. Consolidating and initiating networks and contacts with funders and collaborators in the biosecurity and wider biotechnology policy sector. Group and other responsibilities: Working with other team members and the Research Group Director to develop SET’s research and strategy. As a senior member of the team, setting a collegiate tone and contributing to the development and profile of the wider organisation. Leading on innovative ways to raise RAND Europe’s profile and communicate research findings to maximise impact.</t>
         </is>
       </c>
       <c r="P114" s="6" t="inlineStr">
@@ -10655,7 +10680,7 @@
       </c>
       <c r="Q114" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions biotechnology, biosecurity, and technology policy, which are related to environmental science and sustainability. Although the job is not directly focused on renewable energy or conservation, it is adjacent to the clean energy field and involves r</t>
+          <t>The job description mentions biotechnology, biosecurity, and technology policy, which are related to environmental science and sustainability. Although the job is not directly focused on renewable energy or conservation, it is adjacent to the clean energy field and involves research and policy development related to emerging technologies.</t>
         </is>
       </c>
       <c r="R114" s="2" t="inlineStr">
@@ -10742,7 +10767,7 @@
       </c>
       <c r="O115" s="6" t="inlineStr">
         <is>
-          <t>Během auditu trávíme spoustu času u klientů, kde pečlivě procházíme čísla a informace, které o sobě zveřejňují. Ověřujeme jejich pravdivost, aby byli v očích svých obchodních partnerů, akcionářů, věřitelů i veřejnosti důvěryhodní. Ze začátku budeš pracovat spolu se zkušenými kolegy, kteří ti všechno vysvětlí a k ruce dostaneš i counselora, který tě bude provádět nejen auditem, ale pomůže ti i s kariérním růstem. Postupem času poznáš firemní procesy a ovládneš české účetnictví i mezinárodní audit</t>
+          <t>Během auditu trávíme spoustu času u klientů, kde pečlivě procházíme čísla a informace, které o sobě zveřejňují. Ověřujeme jejich pravdivost, aby byli v očích svých obchodních partnerů, akcionářů, věřitelů i veřejnosti důvěryhodní. Ze začátku budeš pracovat spolu se zkušenými kolegy, kteří ti všechno vysvětlí a k ruce dostaneš i counselora, který tě bude provádět nejen auditem, ale pomůže ti i s kariérním růstem. Postupem času poznáš firemní procesy a ovládneš české účetnictví i mezinárodní auditorské a účetní standardy. Potkáš se se zástupci firem napříč odvětvími a naučíš se s nimi komunikovat. Časem se setkáš i s řediteli a členy boardů.</t>
         </is>
       </c>
       <c r="P115" s="6" t="inlineStr">
@@ -10752,7 +10777,7 @@
       </c>
       <c r="Q115" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions experience with ESG (Environmental, Social, and Governance) and sustainability services, specifically Climate Change and Sustainability Services (CCaSS), which indicates a connection to ESG strategy and corporate sustainability.</t>
+          <t>The job description mentions experience with ESG (Environmental, Social, and Governance) and sustainability services, specifically Climate Change and Sustainability Services (CCaSS), which indicates a connection to ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R115" s="2" t="inlineStr">
@@ -10835,7 +10860,7 @@
       </c>
       <c r="O116" s="6" t="inlineStr">
         <is>
-          <t>Během auditu trávíme spoustu času u klientů, kde pečlivě procházíme čísla a informace, které o sobě zveřejňují. Ověřujeme jejich pravdivost, aby byli v očích svých obchodních partnerů, akcionářů, věřitelů i veřejnosti důvěryhodní. Postupem času poznáš firemní procesy a ovládneš české účetnictví i mezinárodní auditorské a účetní standardy. Potkáš se se zástupci firem napříč odvětvími a naučíš se s nimi komunikovat. Časem se setkáš i s řediteli a členy boardů. Díky auditu nahlédneš do různých obla</t>
+          <t>Během auditu trávíme spoustu času u klientů, kde pečlivě procházíme čísla a informace, které o sobě zveřejňují. Ověřujeme jejich pravdivost, aby byli v očích svých obchodních partnerů, akcionářů, věřitelů i veřejnosti důvěryhodní. Postupem času poznáš firemní procesy a ovládneš české účetnictví i mezinárodní auditorské a účetní standardy. Potkáš se se zástupci firem napříč odvětvími a naučíš se s nimi komunikovat. Časem se setkáš i s řediteli a členy boardů. Díky auditu nahlédneš do různých oblastí firmy – od financí, účetnictví, daní až po oceňování a IT procesy.</t>
         </is>
       </c>
       <c r="P116" s="6" t="inlineStr">
@@ -10845,7 +10870,7 @@
       </c>
       <c r="Q116" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions 'zprávy o udržitelnosti' (sustainability reports) and 'ESG odborníků' (ESG experts), indicating a connection to environmental, social, and governance topics.</t>
+          <t>The job description mentions 'zprávy o udržitelnosti' (sustainability reports) and 'ESG odborníků' (ESG experts), indicating a connection to environmental, social, and governance topics.</t>
         </is>
       </c>
       <c r="R116" s="2" t="inlineStr">
@@ -10924,7 +10949,7 @@
       </c>
       <c r="O117" s="6" t="inlineStr">
         <is>
-          <t>The work duties include conducting research within the project Human Rights for a Politically and Culturally Sustainable World, with a specific focus on the digital and green transition. Through theoretical and/or empirical studies, you will examine new standard threats to human rights, aiming to develop a model for what human rights need to be able to address in a new era. The work involves some travel – to conferences as well as potential field, study or archive trips – although the majority o</t>
+          <t>The work duties include conducting research within the project Human Rights for a Politically and Culturally Sustainable World, with a specific focus on the digital and green transition. Through theoretical and/or empirical studies, you will examine new standard threats to human rights, aiming to develop a model for what human rights need to be able to address in a new era. The work involves some travel – to conferences as well as potential field, study or archive trips – although the majority of the project will be carried out at the workplace. The position also includes some pedagogical training. In addition to research, the position includes teaching, supervision, and other teaching-related tasks amounting to 20% of the working time.</t>
         </is>
       </c>
       <c r="P117" s="6" t="inlineStr">
@@ -10934,7 +10959,7 @@
       </c>
       <c r="Q117" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions human rights, digitisation, and the green transition, which are all related to environmental, social, and governance topics. The focus on human rights as a concept and practice to address risks linked to societal transformations and an uncertain future also</t>
+          <t>The job description mentions human rights, digitisation, and the green transition, which are all related to environmental, social, and governance topics. The focus on human rights as a concept and practice to address risks linked to societal transformations and an uncertain future also indicates relevance to ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R117" s="2" t="inlineStr"/>
@@ -11023,7 +11048,7 @@
       </c>
       <c r="Q118" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions ESG, sustainability, and translating sustainability data into financial impact, which are key aspects of sustainable finance.</t>
+          <t>The job description mentions ESG, sustainability, and translating sustainability data into financial impact, which are key aspects of sustainable finance.</t>
         </is>
       </c>
       <c r="R118" s="2" t="inlineStr">
@@ -11116,7 +11141,7 @@
       </c>
       <c r="Q119" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'Sustainable Finance' as one of the possible rotation areas, and also mentions 'supporting the transition to a climate-resilient future by structuring loans so they are linked to achieving environmental, social and corporate governance (ESG) outcome</t>
+          <t>The job description mentions 'Sustainable Finance' as one of the possible rotation areas, and also mentions 'supporting the transition to a climate-resilient future by structuring loans so they are linked to achieving environmental, social and corporate governance (ESG) outcomes', indicating a focus on sustainable finance and ESG.</t>
         </is>
       </c>
       <c r="R119" s="2" t="inlineStr">
@@ -11199,17 +11224,17 @@
       </c>
       <c r="O120" s="6" t="inlineStr">
         <is>
-          <t>The Lead - Finance &amp; Accounts-SM is responsible for managing the financial and accounting operations of smart metering projects within AESL, overseeing activities such as bookkeeping, accounts payable, accounts receivable, and financial reporting. The role ensures the accurate and timely execution of financial processes while serving as the Controller of Accounts and Tax for the business. It drives operational efficiency, ensures compliance with financial regulations, and provides critical finan</t>
+          <t>The Lead - Finance &amp; Accounts-SM is responsible for managing the financial and accounting operations of smart metering projects within AESL, overseeing activities such as bookkeeping, accounts payable, accounts receivable, and financial reporting. The role ensures the accurate and timely execution of financial processes while serving as the Controller of Accounts and Tax for the business. It drives operational efficiency, ensures compliance with financial regulations, and provides critical financial insights to support decision-making, cost optimization, and sustainable business growth in smart metering operations.</t>
         </is>
       </c>
       <c r="P120" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP FICO, MM, FM Module, BI/BPC Tools, Advance Excel, SAP BG Module, Accounts knowledge, Control Over SAP FICO, MM, FM Module &amp; basic Knowledge SAP BI &amp; BPC Tools, Commercial acumen, Knowledge on Different VAT act, Income Tax Act, and update on Same, Strong interpersonal skills, Coordination skill, </t>
+          <t>SAP FICO, MM, FM Module, BI/BPC Tools, Advance Excel, SAP BG Module, Accounts knowledge, Control Over SAP FICO, MM, FM Module &amp; basic Knowledge SAP BI &amp; BPC Tools, Commercial acumen, Knowledge on Different VAT act, Income Tax Act, and update on Same, Strong interpersonal skills, Coordination skill, Good Team player, Communication Skill, Leadership qualities</t>
         </is>
       </c>
       <c r="Q120" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions smart metering projects, energy infrastructure, and power transmission, which are related to renewable energy and environmental science, making it a clean energy adjacent profile.</t>
+          <t>The job description mentions smart metering projects, energy infrastructure, and power transmission, which are related to renewable energy and environmental science, making it a clean energy adjacent profile.</t>
         </is>
       </c>
       <c r="R120" s="2" t="inlineStr">
@@ -11280,17 +11305,17 @@
       </c>
       <c r="O121" s="6" t="inlineStr">
         <is>
-          <t>The primary role is to make immediate, direct contributions to enhancing our clients’ competitive position and performance in ways that are distinctive, innovative, and sustainable. The SAP EHSM professional will be responsible for tasks related to liaise with customer, understand business processes, apply analytical skills, act as a trusted advisor in the business and technology consulting of SAP S/4HANA Product Compliance and classical Product Safety solution, also experience in SAP EHSM – Inc</t>
+          <t>The primary role is to make immediate, direct contributions to enhancing our clients’ competitive position and performance in ways that are distinctive, innovative, and sustainable. The SAP EHSM professional will be responsible for tasks related to liaise with customer, understand business processes, apply analytical skills, act as a trusted advisor in the business and technology consulting of SAP S/4HANA Product Compliance and classical Product Safety solution, also experience in SAP EHSM – Incident Management, Risk Assessment, Environment Management, Audit Management, Management of Change and Master data management.</t>
         </is>
       </c>
       <c r="P121" s="6" t="inlineStr">
         <is>
-          <t>SAP S/4HANA EHSM, Good communication skill to collaborate with business process owners, project team and other stakeholders / vendors, Good proficiency in Industrial Health &amp; Safety practices and business knowledge like OSHA regulations and ability to understand global regulatory safety standards to</t>
+          <t>SAP S/4HANA EHSM, Good communication skill to collaborate with business process owners, project team and other stakeholders / vendors, Good proficiency in Industrial Health &amp; Safety practices and business knowledge like OSHA regulations and ability to understand global regulatory safety standards to interact with the customer and business process owners, Proficiency in SAP Sustainability modules like Sustainability Footprint Management, Sustainability Control Tower, SAP Green Token are an added advantage</t>
         </is>
       </c>
       <c r="Q121" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[general_esg] The job description mentions experience in SAP EHSM, Sustainability Footprint Management, Sustainability Control Tower, and SAP Green Token, which are related to environmental sustainability and ESG. The role also involves working with clients to enhance their competitive position and </t>
+          <t>The job description mentions experience in SAP EHSM, Sustainability Footprint Management, Sustainability Control Tower, and SAP Green Token, which are related to environmental sustainability and ESG. The role also involves working with clients to enhance their competitive position and performance in a sustainable way, which aligns with the general ESG profile.</t>
         </is>
       </c>
       <c r="R121" s="2" t="inlineStr"/>
@@ -11357,17 +11382,17 @@
       </c>
       <c r="O122" s="6" t="inlineStr">
         <is>
-          <t>Individuals responsible for In-business Risk Management oversee risk identification, assessment, measurement, monitoring, and reporting. They design and implement risk mitigation actions and focus on managing one or more risks in support of business activities. Key Responsibilities: Design and lead projects to execute control enhancements over processes. Document processes developed, actions taken and track matters to ensure resolution. Collaborate with ICRM Sanctions regularly to ensure correct</t>
+          <t>Individuals responsible for In-business Risk Management oversee risk identification, assessment, measurement, monitoring, and reporting. They design and implement risk mitigation actions and focus on managing one or more risks in support of business activities. Key Responsibilities: Design and lead projects to execute control enhancements over processes. Document processes developed, actions taken and track matters to ensure resolution. Collaborate with ICRM Sanctions regularly to ensure correct interpretation and application of sanctions compliance and policy requirements. Liaise with Compliance Assurance and Internal Audit to facilitate resolution of any issues (or corrective actions plans) identified. Maintain oversight through review of metrics, monitoring of activity, and tracking of corrective action plans. Prepare presentations to update senior management and various governance committees on developments, emerging risks, control issues, and enhancements. Ensure the maintenance of a robust Manager’s Control Assessment (MCA) in compliance with the Citi’s Risk Policy. Assess high-risk clients with significant sanctions exposure, including the write up/drafting of internal sanctions risk memos for senior management engagement. Design and develop process plans, notes or guidelines documents. Support any Internal Audit or ICRM Sanctions inquiries and ensure that all audit requests are timely and appropriately provided.</t>
         </is>
       </c>
       <c r="P122" s="6" t="inlineStr">
         <is>
-          <t>Essential: Strong proficiency with Microsoft Suite, excellent organizational and communication skills. Desirable: Project management capabilities, strategic and/or analytical thinking skills. Most Relevant Skills: Analytical Thinking, Business Acumen, Constructive Debate, Escalation Management, Issu</t>
+          <t>Essential: Strong proficiency with Microsoft Suite, excellent organizational and communication skills. Desirable: Project management capabilities, strategic and/or analytical thinking skills. Most Relevant Skills: Analytical Thinking, Business Acumen, Constructive Debate, Escalation Management, Issue Management, Policy and Procedure, Policy and Regulation, Risk Controls and Monitors, Risk Identification and Assessment, Stakeholder Management.</t>
         </is>
       </c>
       <c r="Q122" s="6" t="inlineStr">
         <is>
-          <t>[carbon_markets] The job description mentions experience with maritime emissions regulations, carbon markets, and environmental financial products, which are all relevant to the carbon markets profile.</t>
+          <t>The job description does not mention any specific ESG/sustainability topics, climate risk, or sustainable finance. The role is focused on risk management, compliance, and sanctions, which does not fit into any of the specified profiles.</t>
         </is>
       </c>
       <c r="R122" s="2" t="inlineStr"/>
@@ -11439,12 +11464,12 @@
       </c>
       <c r="P123" s="6" t="inlineStr">
         <is>
-          <t>Strong hands-on experience with: ETL / ELT Cloud platforms (AWS, Snowflake , Open source), Databricks, Open Source, SAP Analytics (BW, HANA, S/4) Data Warehousing and, Strong grasp of: Data modeling and semantic layers, Analytics performance and scalability, Integration patterns across heterogeneous</t>
+          <t>Strong hands-on experience with: ETL / ELT Cloud platforms (AWS, Snowflake , Open source), Databricks, Open Source, SAP Analytics (BW, HANA, S/4) Data Warehousing and, Strong grasp of: Data modeling and semantic layers, Analytics performance and scalability, Integration patterns across heterogeneous source systems, Experience with BI platforms (Power BI, Looker, Tableau, Qlik, etc.)</t>
         </is>
       </c>
       <c r="Q123" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions 'intelligent climate and energy solutions' and ' Carrier Global Corporation' which is a company that provides solutions for climate and energy, indicating a connection to renewable energy and environmental science.</t>
+          <t>The job description mentions 'intelligent climate and energy solutions' and ' Carrier Global Corporation' which is a company that provides solutions for climate and energy, indicating a connection to renewable energy and environmental science.</t>
         </is>
       </c>
       <c r="R123" s="2" t="inlineStr"/>
@@ -11511,17 +11536,17 @@
       </c>
       <c r="O124" s="6" t="inlineStr">
         <is>
-          <t>Develop and refine the test strategy and test planning for embedded systems. Collaborate with software testers and developers to expand and improve test automation and testing strategies. Execute test cases, analyze results, and clearly document findings. Design and execute advanced system tests (both manual and automated). Develop test environments and tools for hardware-near testing. Troubleshoot and analyze complex system failures. Ensure testability during the design phase through requiremen</t>
+          <t>Develop and refine the test strategy and test planning for embedded systems. Collaborate with software testers and developers to expand and improve test automation and testing strategies. Execute test cases, analyze results, and clearly document findings. Design and execute advanced system tests (both manual and automated). Develop test environments and tools for hardware-near testing. Troubleshoot and analyze complex system failures. Ensure testability during the design phase through requirements review and technical guidance. Lead and support junior testers. Collaborate with development, product management, and quality teams to ensure quality throughout the development lifecycle. Report test results, risks, and improvement suggestions to stakeholders.</t>
         </is>
       </c>
       <c r="P124" s="6" t="inlineStr">
         <is>
-          <t>RTOS, microcontrollers, embedded Linux, communication protocols (e.g., Modbus, I2C), test automation using tools such as Python, Robot Framework, or similar, hardware-near development, troubleshooting, CI/CD, version control (e.g., Git, Jenkins, Azure DevOps), SCRUM, test plan design, test case exec</t>
+          <t>RTOS, microcontrollers, embedded Linux, communication protocols (e.g., Modbus, I2C), test automation using tools such as Python, Robot Framework, or similar, hardware-near development, troubleshooting, CI/CD, version control (e.g., Git, Jenkins, Azure DevOps), SCRUM, test plan design, test case execution, strong team player, collaborative mindset, problem-solving ability, strategic and analytical skills, committed to quality and technical excellence, excellent verbal and written communication skills.</t>
         </is>
       </c>
       <c r="Q124" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions 'sustainable climate solutions' and 'energy-efficient solutions for industrial environments', which indicates a focus on environmental sustainability and renewable energy. Although it's not a direct match with renewable energy, the company's produ</t>
+          <t>The job description mentions 'sustainable climate solutions' and 'energy-efficient solutions for industrial environments', which indicates a focus on environmental sustainability and renewable energy. Although it's not a direct match with renewable energy, the company's products and mission are closely related to the clean energy sector.</t>
         </is>
       </c>
       <c r="R124" s="2" t="inlineStr"/>
@@ -11610,7 +11635,7 @@
       </c>
       <c r="Q125" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions ESG, sustainability, and supply chain concepts, indicating a focus on environmental, social, and governance topics. The role involves working with ESG data, conducting QA reviews, and supporting the improvement of internal processes, which aligns with the g</t>
+          <t>The job description mentions ESG, sustainability, and supply chain concepts, indicating a focus on environmental, social, and governance topics. The role involves working with ESG data, conducting QA reviews, and supporting the improvement of internal processes, which aligns with the general ESG profile.</t>
         </is>
       </c>
       <c r="R125" s="2" t="inlineStr">
@@ -11703,7 +11728,7 @@
       </c>
       <c r="Q126" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions supporting the transition to a climate-resilient future, structuring loans linked to achieving environmental, social and corporate governance (ESG) outcomes, and a rotation in Sustainable Finance.</t>
+          <t>The job description mentions supporting the transition to a climate-resilient future, structuring loans linked to achieving environmental, social and corporate governance (ESG) outcomes, and a rotation in Sustainable Finance.</t>
         </is>
       </c>
       <c r="R126" s="2" t="inlineStr">
@@ -11786,7 +11811,7 @@
       </c>
       <c r="O127" s="6" t="inlineStr">
         <is>
-          <t>This is a versatile, high-impact role for someone who wants to make a real difference at an early-stage climate-tech company. As Business Development Manager, you will work across two of BBB's most important growth areas: securing funding through grants and supporting commercial sales activity to agricultural, utilities, and industrial organisations. You will identify and write applications, help shape proposals, coordinate inputs, and manage submissions, while also supporting the commercial tea</t>
+          <t>This is a versatile, high-impact role for someone who wants to make a real difference at an early-stage climate-tech company. As Business Development Manager, you will work across two of BBB's most important growth areas: securing funding through grants and supporting commercial sales activity to agricultural, utilities, and industrial organisations. You will identify and write applications, help shape proposals, coordinate inputs, and manage submissions, while also supporting the commercial team with sales outreach, customer enquiries, lead follow-up, CRM management, and event representation.</t>
         </is>
       </c>
       <c r="P127" s="6" t="inlineStr">
@@ -11796,7 +11821,7 @@
       </c>
       <c r="Q127" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[clean_energy_adjacent] The job description mentions biochar, carbon removal, regenerative agriculture, and climate-tech, which are all related to renewable energy and environmental science. The company's mission is to improve soil health and remove carbon from the atmosphere, which aligns with the </t>
+          <t>The job description mentions biochar, carbon removal, regenerative agriculture, and climate-tech, which are all related to renewable energy and environmental science. The company's mission is to improve soil health and remove carbon from the atmosphere, which aligns with the clean energy adjacent profile.</t>
         </is>
       </c>
       <c r="R127" s="2" t="inlineStr">
@@ -11885,7 +11910,7 @@
       </c>
       <c r="Q128" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions utility-scale solar projects in Southern Africa, renewable energy transactions, and impact investment funds, which are all related to clean energy and environmental sustainability.</t>
+          <t>The job description mentions utility-scale solar projects in Southern Africa, renewable energy transactions, and impact investment funds, which are all related to clean energy and environmental sustainability.</t>
         </is>
       </c>
       <c r="R128" s="2" t="inlineStr">
@@ -11956,7 +11981,7 @@
       </c>
       <c r="O129" s="6" t="inlineStr">
         <is>
-          <t>The Regional Service Delivery Manager - Business Services supports the Assistant Chief Officer Business Services and the Regional Leadership Team with the assessment of operational capability and capacity needs within the region, delivery of support services to members at a Regional level, including the development of a strategically aligned annual operational plan and budget for the Region that includes operational workforce and asset (facility, fleet and equipment) planning, infrastructure pla</t>
+          <t>The Regional Service Delivery Manager - Business Services supports the Assistant Chief Officer Business Services and the Regional Leadership Team with the assessment of operational capability and capacity needs within the region, delivery of support services to members at a Regional level, including the development of a strategically aligned annual operational plan and budget for the Region that includes operational workforce and asset (facility, fleet and equipment) planning, infrastructure planning and delivery, information management and records management, resource allocation support and monitoring processes. The role also supports the ACO Business Services with ensuring the region has in place both Business Continuity and Service Continuity plans and the coordination of risk and issues management with VICSES Business Partners at the regional level. The role provides leadership to business support staff, collaborates closely with internal and external stakeholders, and represents VICSES in regional forums. It drives continuous improvement, supports change initiatives, and ensures that service delivery functions enable volunteers and operational staff to focus on emergency response outcomes.</t>
         </is>
       </c>
       <c r="P129" s="2" t="inlineStr">
@@ -11964,9 +11989,9 @@
           <t>Requires experience in business operations, strategic planning, budget management, risk management, and team leadership.</t>
         </is>
       </c>
-      <c r="Q129" s="2" t="inlineStr">
-        <is>
-          <t>VICSES is a volunteer-based emergency service that focuses on building community resilience through preparedness and response to emergencies.</t>
+      <c r="Q129" s="6" t="inlineStr">
+        <is>
+          <t>The job description does not mention any ESG/sustainability topics, climate risk, sustainable finance, carbon markets, EU Taxonomy, or other related keywords. The role is focused on emergency service delivery and management, which does not fit any of the specified profiles.</t>
         </is>
       </c>
       <c r="R129" s="2" t="inlineStr"/>
@@ -12033,7 +12058,7 @@
       </c>
       <c r="O130" s="6" t="inlineStr">
         <is>
-          <t>You will own the end-to-end product and commercialisation agenda and bring it to life through action, influence and delivery. This includes: Scanning the market relentlessly to identify smart, connected and solution-based water opportunities across residential, commercial and institutional segments. Deeply understanding customers, uncovering real pain points through research, interviews and partner engagement, and validating where value truly lies. Designing compelling commercial models, includi</t>
+          <t>You will own the end-to-end product and commercialisation agenda and bring it to life through action, influence and delivery. This includes: Scanning the market relentlessly to identify smart, connected and solution-based water opportunities across residential, commercial and institutional segments. Deeply understanding customers, uncovering real pain points through research, interviews and partner engagement, and validating where value truly lies. Designing compelling commercial models, including pricing, installation, service, maintenance and subscription or recurring revenue streams. Shaping and optimising the portfolio, making clear calls on what to scale, improve, pivot or exit. Building and owning a multi-year roadmap that balances near-term revenue with long-term platform and ecosystem bets. Leading go-to-market strategy and execution, personally driving value propositions, positioning, solution narratives and sales enablement. Defining operating models that ensure solutions can be sold, installed, supported and maintained at scale. Applying a constructive lens to ways of working, bringing clarity, structure and commercial discipline to complex, ambiguous problems. Acting as a dynamic connector, building strong relationships across Innovation, Technology, Finance, Supply Chain and Sales.</t>
         </is>
       </c>
       <c r="P130" s="6" t="inlineStr">
@@ -12043,7 +12068,7 @@
       </c>
       <c r="Q130" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions 'sustainable water solutions', 'smart and connected water solutions', and 'water opportunities', indicating a focus on environmental sustainability and water management, which aligns with the clean energy adjacent profile.</t>
+          <t>The job description mentions 'sustainable water solutions', 'smart and connected water solutions', and 'water opportunities', indicating a focus on environmental sustainability and water management, which aligns with the clean energy adjacent profile.</t>
         </is>
       </c>
       <c r="R130" s="2" t="inlineStr"/>
@@ -12110,7 +12135,7 @@
       </c>
       <c r="O131" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Als Project- en Procesmanager binnen Royal Smit en Zoon ben je verantwoordelijk voor het initiëren, ontwikkelen en realiseren van investeringsprojecten en contract manufacturing-activiteiten. Je zorgt voor een veilige, efficiënte en toekomstbestendige productiecapaciteit, technische integriteit van assets en naleving van QESH- en procesveiligheidsnormen. Je ondersteunt hierbij de productielocaties in Weesp en Amersfoort en levert een belangrijke bijdrage aan de strategische ontwikkeling van het </t>
+          <t>Als Project- en Procesmanager binnen Royal Smit en Zoon ben je verantwoordelijk voor het initiëren, ontwikkelen en realiseren van investeringsprojecten en contract manufacturing-activiteiten. Je zorgt voor een veilige, efficiënte en toekomstbestendige productiecapaciteit, technische integriteit van assets en naleving van QESH- en procesveiligheidsnormen. Je ondersteunt hierbij de productielocaties in Weesp en Amersfoort en levert een belangrijke bijdrage aan de strategische ontwikkeling van het productie- en assetportfolio van Royal Smit &amp; Zoon.</t>
         </is>
       </c>
       <c r="P131" s="6" t="inlineStr">
@@ -12120,7 +12145,7 @@
       </c>
       <c r="Q131" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions 'duurzame grondstoffen' (sustainable raw materials) and 'de waardeketen van de leerindustrie verduurzamen' (sustaining the leather industry's value chain), indicating a focus on environmental sustainability, and 'procesveiligheid' (process safety)</t>
+          <t>The job description mentions 'duurzame grondstoffen' (sustainable raw materials) and 'de waardeketen van de leerindustrie verduurzamen' (sustaining the leather industry's value chain), indicating a focus on environmental sustainability, and 'procesveiligheid' (process safety) and 'technische integriteit' (technical integrity), which are relevant to the clean energy adjacent profile.</t>
         </is>
       </c>
       <c r="R131" s="2" t="inlineStr"/>
@@ -12187,7 +12212,7 @@
       </c>
       <c r="O132" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">This role is central to advancing NORCAP’s commitment to climate action, peace, democracy, and human rights through strategic leadership, policy influence, and effective programme delivery. You will lead one of NORCAP’s most forward‑looking portfolios—where strategic leadership, programme quality, and policy influence come together. You will guide a strong team, shape partnerships, and steer a portfolio that has the mandate to rethink how aid can better address climate‑related risks, strengthen </t>
+          <t>This role is central to advancing NORCAP’s commitment to climate action, peace, democracy, and human rights through strategic leadership, policy influence, and effective programme delivery. You will lead one of NORCAP’s most forward‑looking portfolios—where strategic leadership, programme quality, and policy influence come together. You will guide a strong team, shape partnerships, and steer a portfolio that has the mandate to rethink how aid can better address climate‑related risks, strengthen peaceful societies, and uphold democratic space.</t>
         </is>
       </c>
       <c r="P132" s="6" t="inlineStr">
@@ -12197,7 +12222,7 @@
       </c>
       <c r="Q132" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions 'climate action', 'climate change', and 'climate‑related risks', indicating a strong focus on climate risk management and mitigation.</t>
+          <t>The job description mentions 'climate action', 'climate change', and 'climate‑related risks', indicating a strong focus on climate risk management and mitigation.</t>
         </is>
       </c>
       <c r="R132" s="2" t="inlineStr"/>
@@ -12264,7 +12289,7 @@
       </c>
       <c r="O133" s="6" t="inlineStr">
         <is>
-          <t>Algorithm Development &amp; Signal Processing: Lead the design, implementation, and optimization of ECG signal‑processing algorithms. Develop robust algorithms suitable for embedded systems. Analyze diverse ECG datasets to ensure algorithm reliability. Conduct algorithm performance benchmarking and validation. Software Engineering &amp; Design Transfer: Implement algorithms in production-quality code and support Design Transfer. Cross-functional &amp; Technical Collaboration: Collaborate with internal and e</t>
+          <t>Algorithm Development &amp; Signal Processing: Lead the design, implementation, and optimization of ECG signal‑processing algorithms. Develop robust algorithms suitable for embedded systems. Analyze diverse ECG datasets to ensure algorithm reliability. Conduct algorithm performance benchmarking and validation. Software Engineering &amp; Design Transfer: Implement algorithms in production-quality code and support Design Transfer. Cross-functional &amp; Technical Collaboration: Collaborate with internal and external partners. Quality, Compliance &amp; Documentation: Develop and maintain detailed documentation and ensure compliance with regulatory standards. Support, Debugging &amp; Continuous Improvement: Support troubleshooting and drive continuous improvement initiatives.</t>
         </is>
       </c>
       <c r="P133" s="6" t="inlineStr">
@@ -12274,7 +12299,7 @@
       </c>
       <c r="Q133" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions ESG, sustainability, and translating sustainability data into financial impact, which are key aspects of sustainable finance.</t>
+          <t>The job description does not explicitly mention ESG, sustainability, climate risk, or other related topics. While the company mentions 'combat climate change' in its description, this is not directly related to the job responsibilities or requirements.</t>
         </is>
       </c>
       <c r="R133" s="2" t="inlineStr"/>
@@ -12353,17 +12378,17 @@
       </c>
       <c r="O134" s="6" t="inlineStr">
         <is>
-          <t>The carbon removal market is at an inflection point. Buyers are becoming more sophisticated, the supply side is maturing, and the conversations shaping this market - about quality, integrity, and scale - are happening right now. Carbonfuture sits at the center of those conversations, and we need someone who can make sure our voice is heard. This is a hands-on writing role. You'll own Carbonfuture's editorial output, from content to sharp thought leadership and press outreach. You'll help our exp</t>
+          <t>The carbon removal market is at an inflection point. Buyers are becoming more sophisticated, the supply side is maturing, and the conversations shaping this market - about quality, integrity, and scale - are happening right now. Carbonfuture sits at the center of those conversations, and we need someone who can make sure our voice is heard. This is a hands-on writing role. You'll own Carbonfuture's editorial output, from content to sharp thought leadership and press outreach. You'll help our experts show up well at events and in interviews. And you'll develop the formats that keep Carbonfuture at the center of the conversation.</t>
         </is>
       </c>
       <c r="P134" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exceptional written English — you write with the fluency and precision of a native speaker, across formats and audiences. Strong editorial judgement: you know and love to tinker with what makes a story work, and what makes it fall flat. Ability to translate complex, technical topics into compelling </t>
+          <t>Exceptional written English — you write with the fluency and precision of a native speaker, across formats and audiences. Strong editorial judgement: you know and love to tinker with what makes a story work, and what makes it fall flat. Ability to translate complex, technical topics into compelling narratives for non-expert audiences. Comfortable working cross-functionally — extracting insight from busy subject-matter experts and turning it into content without slowing anyone down. Self-directed and organized, able to manage multiple content streams in parallel</t>
         </is>
       </c>
       <c r="Q134" s="6" t="inlineStr">
         <is>
-          <t>[carbon_markets] The job description mentions carbon removal, carbon markets, and durable carbon removal, which are all related to carbon markets. The company, Carbonfuture, provides tools and services for carbon removal, which further supports this classification.</t>
+          <t>The job description mentions carbon removal, carbon markets, and durable carbon removal, which are all related to carbon markets. The company, Carbonfuture, provides tools and services for carbon removal, which further supports this classification.</t>
         </is>
       </c>
       <c r="R134" s="2" t="inlineStr">
@@ -12456,7 +12481,7 @@
       </c>
       <c r="Q135" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'sustainable finance' as one of the DCM products, indicating a focus on environmental, social, or governance topics.</t>
+          <t>The job description mentions 'sustainable finance' as one of the DCM products, indicating a focus on environmental, social, or governance topics.</t>
         </is>
       </c>
       <c r="R135" s="2" t="inlineStr">
@@ -12527,7 +12552,7 @@
       </c>
       <c r="O136" s="6" t="inlineStr">
         <is>
-          <t>You provide spatial and statistical support in the assembly and pre-processing of a wide variety of maternal health indicators from household survey data, such as Demographic and Health Surveys. You offer spatial and statistical support in the assembly and pre-processing of health indicators based on environment, climate, population and infrastructure data from open data portals. You conduct geospatial modelling and analyses to examine the variation of maternal health indicators across space and</t>
+          <t>You provide spatial and statistical support in the assembly and pre-processing of a wide variety of maternal health indicators from household survey data, such as Demographic and Health Surveys. You offer spatial and statistical support in the assembly and pre-processing of health indicators based on environment, climate, population and infrastructure data from open data portals. You conduct geospatial modelling and analyses to examine the variation of maternal health indicators across space and time. You interpret spatial and temporal patterns in maternal health indicators. You apply related statistical and advanced spatial analyses to determine and understand maternal health vulnerability in urban areas.</t>
         </is>
       </c>
       <c r="P136" s="6" t="inlineStr">
@@ -12537,7 +12562,7 @@
       </c>
       <c r="Q136" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job involves geospatial analysis of maternal health indicators, which is related to environmental science and public health, and the company is involved in public health research and service delivery, which is adjacent to the clean energy and environmental science field.</t>
+          <t>The job involves geospatial analysis of maternal health indicators, which is related to environmental science and public health, and the company is involved in public health research and service delivery, which is adjacent to the clean energy and environmental science field.</t>
         </is>
       </c>
       <c r="R136" s="2" t="inlineStr"/>
@@ -12616,7 +12641,7 @@
       </c>
       <c r="O137" s="6" t="inlineStr">
         <is>
-          <t>The role will be responsible for supporting the assessment, design and implementation of the Global ESG reporting control framework and will be required to collaborate cross functionally. The role will specifically support the alignment of the ESG control framework with the Global Finance control framework. This will include the integration with the Novartis 3LOD model, which will require collaboration with the Financial Controls and Compliance team. Major accountabilities include: monitoring th</t>
+          <t>The role will be responsible for supporting the assessment, design and implementation of the Global ESG reporting control framework and will be required to collaborate cross functionally. The role will specifically support the alignment of the ESG control framework with the Global Finance control framework. This will include the integration with the Novartis 3LOD model, which will require collaboration with the Financial Controls and Compliance team. Major accountabilities include: monitoring the internal control framework over ESG reporting, supporting the uplift of the ESG reporting control framework, maintaining the accuracy of the ESG reporting RACM and RACI, supporting areas of priority and focus, driving process deep-dives to identify process-control gaps, overseeing definition and implementation of solutions to enhance internal controls assurance, supporting assurance readiness, roadmap to reasonable assurance, supporting process/systems control improvement, automation, and standardization, monitoring process changes, and continuously assessing the impact of process changes on control environment, risk and defining mitigating actions to ensure reliable processes and systems with in-built controls.</t>
         </is>
       </c>
       <c r="P137" s="6" t="inlineStr">
@@ -12626,7 +12651,7 @@
       </c>
       <c r="Q137" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions ESG (Environmental Social Governance) risk and controls, ESG reporting, and ESG control framework, which are all related to environmental, social, and governance topics, indicating a strong fit with the general ESG profile.</t>
+          <t>The job description mentions ESG (Environmental Social Governance) risk and controls, ESG reporting, and ESG control framework, which are all related to environmental, social, and governance topics, indicating a strong fit with the general ESG profile.</t>
         </is>
       </c>
       <c r="R137" s="2" t="inlineStr">
@@ -12717,9 +12742,9 @@
           <t>Analytical skills, Effective verbal and written communication skills, Experience with process improvements, Experience with cross-functional and cross-regional process initiatives, Familiarity with EY and/or global delivery models</t>
         </is>
       </c>
-      <c r="Q138" s="2" t="inlineStr">
-        <is>
-          <t>The position is within the audit service line at EY GDS Assurance, contributing to climate change, ESG, sustainability, and finance practices.</t>
+      <c r="Q138" s="6" t="inlineStr">
+        <is>
+          <t>The job description does not mention any specific ESG/sustainability topics, climate risk, sustainable finance, carbon markets, EU Taxonomy, or clean energy. The focus is on process improvements, audit delivery, and assurance services, which are not directly related to environmental, social, or governance topics.</t>
         </is>
       </c>
       <c r="R138" s="2" t="inlineStr">
@@ -12802,7 +12827,7 @@
       </c>
       <c r="O139" s="6" t="inlineStr">
         <is>
-          <t>Lead end-to-end change management activities across programs of work, supporting digital and business transformation initiatives, partnering with subject matter experts to plan, coordinate and deliver successful change outcomes. Design and deliver targeted training solutions including training needs analysis, planning, and development of engaging learning activities aligned with adult learning principles and delivered in partnership with the Learning &amp; Development team. Manage change and communi</t>
+          <t>Lead end-to-end change management activities across programs of work, supporting digital and business transformation initiatives, partnering with subject matter experts to plan, coordinate and deliver successful change outcomes. Design and deliver targeted training solutions including training needs analysis, planning, and development of engaging learning activities aligned with adult learning principles and delivered in partnership with the Learning &amp; Development team. Manage change and communications delivery by implementing structured change and communication plans for technology-enabled initiatives, while proactively identifying and addressing risks or issues that may impact outcomes. Provide expert change advice and solutions to stakeholders, ensuring digital initiatives align with the City’s strategic priorities. Empower leaders to lead change effectively by coaching them to plan key conversations and deliver engaging information sessions, presentations, and change communications. Create impactful reports, briefings and presentations to engage stakeholders and support successful change adoption. Monitor risks and track key indicators, identifying and escalating issues early to keep change initiatives on track.</t>
         </is>
       </c>
       <c r="P139" s="6" t="inlineStr">
@@ -12812,7 +12837,7 @@
       </c>
       <c r="Q139" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions 'intelligent climate and energy solutions' and ' Carrier Global Corporation' which is a company that provides solutions for climate and energy, indicating a connection to renewable energy and environmental science.</t>
+          <t>The job description does not mention any specific ESG/sustainability topics, and the mention of 'sustainability' in the company description is in the context of general business operations, not environmental or social sustainability.</t>
         </is>
       </c>
       <c r="R139" s="2" t="inlineStr">
@@ -12895,7 +12920,7 @@
       </c>
       <c r="O140" s="6" t="inlineStr">
         <is>
-          <t>Test Strategy &amp; Execution: Define and execute system validation and integration test plans for Analog Devices' SoCs running Zephyr RTOS and embedded Linux. Build test cases covering functional correctness, corner cases, performance, power mode transitions, and boot sequence validation across virtual prototyping, emulation, and post-silicon environments. Establish test coverage metrics, pass/fail criteria, and quality gates for release milestones. CI/CD &amp; Test Infrastructure: Architect and mainta</t>
+          <t>Test Strategy &amp; Execution: Define and execute system validation and integration test plans for Analog Devices' SoCs running Zephyr RTOS and embedded Linux. Build test cases covering functional correctness, corner cases, performance, power mode transitions, and boot sequence validation across virtual prototyping, emulation, and post-silicon environments. Establish test coverage metrics, pass/fail criteria, and quality gates for release milestones. CI/CD &amp; Test Infrastructure: Architect and maintain CI/CD pipelines using GitHub Actions for automated build, test, and regression workflows across Zephyr and Linux targets. Define the test framework strategy (e.g., Zephyr Twister, custom frameworks, or hybrid approaches) and integrate static analysis, code coverage, and test reporting into CI/CD workflows. Debugging &amp; Root-Cause Analysis: Lead cross-domain debugging spanning hardware, firmware, RTOS, BSP, using debug tools, trace utilities, and logs. Collaborate with firmware, driver, and bare-metal test teams to resolve issues and refine test methodologies. Team Leadership: Mentor engineers on test methodologies and debugging best practices. Document findings and present status and risks to stakeholders.</t>
         </is>
       </c>
       <c r="P140" s="6" t="inlineStr">
@@ -12905,7 +12930,7 @@
       </c>
       <c r="Q140" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions 'sustainable climate solutions' and 'energy-efficient solutions for industrial environments', which indicates a focus on environmental sustainability and renewable energy. Although it's not a direct match with renewable energy, the company's produ</t>
+          <t>The job description does not mention any specific ESG/sustainability topics, climate change mitigation, or environmental sustainability. Although the company description mentions 'combat climate change', it is not directly related to the job responsibilities, requirements, or skills.</t>
         </is>
       </c>
       <c r="R140" s="2" t="inlineStr">
@@ -12993,12 +13018,12 @@
       </c>
       <c r="P141" s="6" t="inlineStr">
         <is>
-          <t>Experience and expertise in one or more of the six categories, including Monitoring, Evaluation and Learning, Agriculture, Food/nutrition and Water Security, Climate Change and Disaster Risk Reduction, Communications and Creatives, Program and Investment Design, and Gender, Disability, Equity and So</t>
+          <t>Experience and expertise in one or more of the six categories, including Monitoring, Evaluation and Learning, Agriculture, Food/nutrition and Water Security, Climate Change and Disaster Risk Reduction, Communications and Creatives, Program and Investment Design, and Gender, Disability, Equity and Social Inclusion.</t>
         </is>
       </c>
       <c r="Q141" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate change, disaster risk reduction, and climate resilience, which are all relevant to the climate risk profile.</t>
+          <t>The job description mentions climate change, disaster risk reduction, and climate resilience, which are all relevant to the climate risk profile.</t>
         </is>
       </c>
       <c r="R141" s="2" t="inlineStr">
@@ -13069,7 +13094,7 @@
       </c>
       <c r="O142" s="6" t="inlineStr">
         <is>
-          <t>Lead and/or contribute to international ESIA processes for large-scale infrastructure, energy, transport, industrial, and environmental projects. Conduct or support Environmental and Social Due Diligence (ESDD)/ Environmental, Health and Safety Due Diligence (EHS DD) assignments for IFIs, lenders, and private investors. Conduct or support Environmental Due Diligence (EDD)/ Environmental, Health and Safety Due Diligence (EHS DD) assignments in relation to mergers and acquisitions (M&amp;A). Coordinat</t>
+          <t>Lead and/or contribute to international ESIA processes for large-scale infrastructure, energy, transport, industrial, and environmental projects. Conduct or support Environmental and Social Due Diligence (ESDD)/ Environmental, Health and Safety Due Diligence (EHS DD) assignments for IFIs, lenders, and private investors. Conduct or support Environmental Due Diligence (EDD)/ Environmental, Health and Safety Due Diligence (EHS DD) assignments in relation to mergers and acquisitions (M&amp;A). Coordinate environmental and social workstreams in multidisciplinary project teams. Engage with clients, IFIs, authorities, local stakeholders and subcontractors in various countries. Prepare high quality technical documentation, including ESIA reports, EDD reports, management plans, and monitoring frameworks.</t>
         </is>
       </c>
       <c r="P142" s="6" t="inlineStr">
@@ -13079,7 +13104,7 @@
       </c>
       <c r="Q142" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions working on sustainability-driven assignments, international environmental and social impact assessments, and environmental and social due diligence, which are all related to ESG strategy and corporate sustainability.</t>
+          <t>The job description mentions working on sustainability-driven assignments, international environmental and social impact assessments, and environmental and social due diligence, which are all related to ESG strategy and corporate sustainability.</t>
         </is>
       </c>
       <c r="R142" s="2" t="inlineStr"/>
@@ -13146,7 +13171,7 @@
       </c>
       <c r="O143" s="6" t="inlineStr">
         <is>
-          <t>What are you going to do? Als (Junior) Consultant Green Investments word je onderdeel van het INVEST-team: een hecht en enthousiast team dat dagelijks werkt aan Europese of nationale impactvolle projecten. Je staat in direct contact met onze klanten en helpt hen bij het realiseren van duurzame investeringen. Dat doe je door kansen te signaleren, mee te denken over de beste aanpak en subsidies en regelingen te vertalen naar concrete projecten. Je brengt al een basiskennis mee van hernieuwbare ene</t>
+          <t>What are you going to do? Als (Junior) Consultant Green Investments word je onderdeel van het INVEST-team: een hecht en enthousiast team dat dagelijks werkt aan Europese of nationale impactvolle projecten. Je staat in direct contact met onze klanten en helpt hen bij het realiseren van duurzame investeringen. Dat doe je door kansen te signaleren, mee te denken over de beste aanpak en subsidies en regelingen te vertalen naar concrete projecten. Je brengt al een basiskennis mee van hernieuwbare energiesystemen, waardoor je snel kunt meedenken met klanten. Binnen het INVEST-team ontwikkel je je verder en groei je stap voor stap uit tot een volwaardige adviseur voor klanten in de industrie en energiesector, met directe impact op duurzame investeringen. Je analyseert duurzame investeringsplannen van klanten en identificeert de meest kansrijke subsidiemogelijkheden; Je verdiept je in en begrijpt de projecten van de klant inhoudelijk en vertaalt technische projectinformatie naar een heldere financiële en subsidie-technische onderbouwing; Je ontwikkelt sterke investeringsbusinesscases (CAPEX/OPEX, cashflows, terugverdientijd, risico’s); Je rol is praktisch en resultaatgericht: je werkt toe naar concrete subsidieaanvragen, méér dan alleen naar analyses of beleidsadviezen. Je levert een actieve bijdrage aan de groei van het INVEST-team door betrokkenheid bij business development en de verdere professionalisering van onze dienstverlening; Je werkt samen met collega’s om klanten optimaal te bedienen met op maat gemaakte investeringsstrategieën.</t>
         </is>
       </c>
       <c r="P143" s="6" t="inlineStr">
@@ -13156,7 +13181,7 @@
       </c>
       <c r="Q143" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions 'duurzame investeringen' (sustainable investments), 'hernieuwbare energiesystemen' (renewable energy systems), and 'energietransitie' (energy transition), which are all related to renewable energy and environmental science, fitting the clean_energ</t>
+          <t>The job description mentions 'duurzame investeringen' (sustainable investments), 'hernieuwbare energiesystemen' (renewable energy systems), and 'energietransitie' (energy transition), which are all related to renewable energy and environmental science, fitting the clean_energy_adjacent profile.</t>
         </is>
       </c>
       <c r="R143" s="2" t="inlineStr"/>
@@ -13225,7 +13250,7 @@
       <c r="P144" s="2" t="inlineStr"/>
       <c r="Q144" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] Job title contains 'Climate Action', indicating a strong focus on climate-related issues.</t>
+          <t>Job title contains 'Climate Action', indicating a strong focus on climate-related issues.</t>
         </is>
       </c>
       <c r="R144" s="2" t="inlineStr"/>
@@ -13302,7 +13327,7 @@
       </c>
       <c r="Q145" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] Job title contains 'Climate Risk Analysis' indicating a strong focus on climate risk</t>
+          <t>Job title contains 'Climate Risk Analysis' indicating a strong focus on climate risk</t>
         </is>
       </c>
       <c r="R145" s="2" t="inlineStr"/>
@@ -13381,7 +13406,7 @@
       </c>
       <c r="O146" s="6" t="inlineStr">
         <is>
-          <t>We are seeking a dynamic and experienced environmental project manager to lead and support island, marine and vulnerable species management, including conservation and intervention actions, within the Great Barrier Reef World Heritage Area. This is a dynamic position with a wide range of responsibilities including project planning and reporting, risk assessment, project evaluation, procurement, communication product development, stakeholder and Traditional Owner engagement, and some marine-based</t>
+          <t>We are seeking a dynamic and experienced environmental project manager to lead and support island, marine and vulnerable species management, including conservation and intervention actions, within the Great Barrier Reef World Heritage Area. This is a dynamic position with a wide range of responsibilities including project planning and reporting, risk assessment, project evaluation, procurement, communication product development, stakeholder and Traditional Owner engagement, and some marine-based fieldwork.</t>
         </is>
       </c>
       <c r="P146" s="6" t="inlineStr">
@@ -13391,7 +13416,7 @@
       </c>
       <c r="Q146" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions reef conservation, marine and vulnerable species management, and environmental project management, which are related to renewable energy, environmental science, and conservation, making it a good fit for the clean_energy_adjacent profile.</t>
+          <t>The job description mentions reef conservation, marine and vulnerable species management, and environmental project management, which are related to renewable energy, environmental science, and conservation, making it a good fit for the clean_energy_adjacent profile.</t>
         </is>
       </c>
       <c r="R146" s="2" t="inlineStr">
@@ -13474,7 +13499,7 @@
       </c>
       <c r="O147" s="6" t="inlineStr">
         <is>
-          <t>In this role, you will use your commodities trading knowledge and analytical skills to provide expert advice on front line trading risks for the Gas, Power and Carbon desks. You will support and facilitate the continued improvement of processes, controls and operational risk awareness and culture across our businesses. As a subject matter expert you will partner with the trading desks and leverage your technical expertise to develop a comprehensive knowledge of all processes to proactively manag</t>
+          <t>In this role, you will use your commodities trading knowledge and analytical skills to provide expert advice on front line trading risks for the Gas, Power and Carbon desks. You will support and facilitate the continued improvement of processes, controls and operational risk awareness and culture across our businesses. As a subject matter expert you will partner with the trading desks and leverage your technical expertise to develop a comprehensive knowledge of all processes to proactively manage the operational risks. You will provide advice on a broad range of risk matters, assess new product and business initiatives, investigate incidents and test effectiveness of controls.</t>
         </is>
       </c>
       <c r="P147" s="6" t="inlineStr">
@@ -13484,7 +13509,7 @@
       </c>
       <c r="Q147" s="6" t="inlineStr">
         <is>
-          <t>[carbon_markets] The job description mentions experience in Carbon markets as a plus, and the role involves providing expert advice on front line trading risks for the Gas, Power and Carbon desks, indicating a strong connection to carbon markets and emissions trading.</t>
+          <t>The job description mentions experience in Carbon markets as a plus, and the role involves providing expert advice on front line trading risks for the Gas, Power and Carbon desks, indicating a strong connection to carbon markets and emissions trading.</t>
         </is>
       </c>
       <c r="R147" s="2" t="inlineStr">
@@ -13567,7 +13592,7 @@
       </c>
       <c r="O148" s="6" t="inlineStr">
         <is>
-          <t>Managing, maintaining, and expanding the client portfolio, with a focus on new business and high potential markets. Developing our trading activities for short and long-term strategies in line with the company’s objectives. Conduct market research where you will research and analyse market trends, technological advancements, potential clients, and their industry trends, to help inform business decisions. Creating analyses and presentations to update your clients and stakeholders with market tren</t>
+          <t>Managing, maintaining, and expanding the client portfolio, with a focus on new business and high potential markets. Developing our trading activities for short and long-term strategies in line with the company’s objectives. Conduct market research where you will research and analyse market trends, technological advancements, potential clients, and their industry trends, to help inform business decisions. Creating analyses and presentations to update your clients and stakeholders with market trends, new upcoming projects, and other relevant information. Ensure brand awareness and building your network through participation in business events, fairs, and other occasions. Collaborate, learn, enjoy, and work together with other teams together to achieve the best possible for AFS Energy.</t>
         </is>
       </c>
       <c r="P148" s="6" t="inlineStr">
@@ -13577,7 +13602,7 @@
       </c>
       <c r="Q148" s="6" t="inlineStr">
         <is>
-          <t>[carbon_markets] The job description mentions 'Carbon Markets including trading dynamics related to the buy and sell side of transactions, negotiation, and other macroeconomic factors' and 'Environmental commodities', indicating a strong focus on carbon markets and environmental sustainability.</t>
+          <t>The job description mentions 'Carbon Markets including trading dynamics related to the buy and sell side of transactions, negotiation, and other macroeconomic factors' and 'Environmental commodities', indicating a strong focus on carbon markets and environmental sustainability.</t>
         </is>
       </c>
       <c r="R148" s="2" t="inlineStr">
@@ -13660,12 +13685,14 @@
       </c>
       <c r="O149" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">As a Senior Associate / Legal Director, you will: 
+          <t>As a Senior Associate / Legal Director, you will: 
    * Lead the drafting and negotiation of complex project, construction and finance documentation
    * Take primary responsibility for managing transactions, including supervising junior lawyers and coordinating multi-jurisdictional teams
    * Provide strategic advice to clients on risk allocation, structuring and execution of projects
    * Play a key role in client relationship management, acting as a trusted advisor on ongoing and new matters
-</t>
+   * Drive business development initiatives, including identifying opportunities, preparing pitches and contributing to sector-focused thought leadership
+   * Mentor and develop junior team members, fostering a collaborative and high-performing team culture
+   * Work closely with partners on practice development and contribute to the broader strategic growth of the team</t>
         </is>
       </c>
       <c r="P149" s="6" t="inlineStr">
@@ -13675,7 +13702,7 @@
       </c>
       <c r="Q149" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions experience in renewable energy, low-carbon infrastructure, carbon markets, and natural capital, which are all relevant to the clean energy and environmental sectors.</t>
+          <t>The job description mentions experience in renewable energy, low-carbon infrastructure, carbon markets, and natural capital, which are all relevant to the clean energy and environmental sectors.</t>
         </is>
       </c>
       <c r="R149" s="2" t="inlineStr">
@@ -13764,7 +13791,7 @@
       </c>
       <c r="Q150" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions renewable energy development, solar, wind, and hybrid systems, which are directly related to clean energy. The company's focus on transitioning toward clean and intelligent energy systems also supports this classification.</t>
+          <t>The job description mentions renewable energy development, solar, wind, and hybrid systems, which are directly related to clean energy. The company's focus on transitioning toward clean and intelligent energy systems also supports this classification.</t>
         </is>
       </c>
       <c r="R150" s="2" t="inlineStr">
@@ -13843,7 +13870,7 @@
       </c>
       <c r="O151" s="6" t="inlineStr">
         <is>
-          <t>Manage AIDMIs social media accounts, including Instagram, Twitter, LinkedIn, Facebook, and WhatsApp Chat Bot Integration and Management. Develop and implement social media strategies that align with AIDMIs goals and Create engaging and educational social media content, including graphics, videos, and Monitor social media trends and good practices, and incorporate new techniques and tools to remain at the forefront. Collaborate, co-create and implement at least three social media campaigns that s</t>
+          <t>Manage AIDMIs social media accounts, including Instagram, Twitter, LinkedIn, Facebook, and WhatsApp Chat Bot Integration and Management. Develop and implement social media strategies that align with AIDMIs goals and Create engaging and educational social media content, including graphics, videos, and Monitor social media trends and good practices, and incorporate new techniques and tools to remain at the forefront. Collaborate, co-create and implement at least three social media campaigns that support Develop and maintain the AIDMI website, including troubleshooting and bug fixing. Develop and implement new web-based projects such as quizzes, Google Surveys, etc., Write clean and efficient code that is easy to maintain. Ensure website and web-based projects are user-friendly, accessible, and visually appealing with high impact and visible results. Test website and web-based projects to ensure they meet the quality and performance standards of organisations such as ODI. Keep up to date with web development and social media trends and technologies, and incorporate new techniques and tools as soon as they are available. Collecting, maintaining, and analysing data for record and development processes.</t>
         </is>
       </c>
       <c r="P151" s="6" t="inlineStr">
@@ -13853,7 +13880,7 @@
       </c>
       <c r="Q151" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job title mentions 'Disaster Risk and Climate Resilience', indicating a focus on climate-related risks, and the company name 'All India Disaster Mitigation Institute' also suggests a connection to disaster risk and climate resilience.</t>
+          <t>The job title mentions 'Disaster Risk and Climate Resilience', indicating a focus on climate-related risks, and the company name 'All India Disaster Mitigation Institute' also suggests a connection to disaster risk and climate resilience.</t>
         </is>
       </c>
       <c r="R151" s="2" t="inlineStr"/>
@@ -13932,7 +13959,7 @@
       </c>
       <c r="O152" s="6" t="inlineStr">
         <is>
-          <t>Proven work experience as an Operations Manager or similar role in the Solar Energy sector. Experience with inventory management, database systems, or similar software is beneficial. Relevant training and/or certifications as an Operations Associate. O&amp;M Manager is responsible for scheduling cleaning, breakdown, and preventive maintenance activities. All reports must be sent to the client with comments within 4 hours of completing the activity. O&amp;M Manager must prepare MIS reports, verify vendor</t>
+          <t>Proven work experience as an Operations Manager or similar role in the Solar Energy sector. Experience with inventory management, database systems, or similar software is beneficial. Relevant training and/or certifications as an Operations Associate. O&amp;M Manager is responsible for scheduling cleaning, breakdown, and preventive maintenance activities. All reports must be sent to the client with comments within 4 hours of completing the activity. O&amp;M Manager must prepare MIS reports, verify vendor bills, and coordinate with the accounts team for payments. O&amp;M Manager shall coordinate with the purchase department regarding warranty claims. O&amp;M Executive will report to the O&amp;M Manager. Excellent communication and listening skills. Ability to work effectively under pressure. Strong computer proficiency.</t>
         </is>
       </c>
       <c r="P152" s="6" t="inlineStr">
@@ -13942,7 +13969,7 @@
       </c>
       <c r="Q152" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions solar energy, renewable energy, and utility-scale solar energy projects, which are all related to clean energy and environmental sustainability.</t>
+          <t>The job description mentions solar energy, renewable energy, and utility-scale solar energy projects, which are all related to clean energy and environmental sustainability.</t>
         </is>
       </c>
       <c r="R152" s="2" t="inlineStr">
@@ -14039,7 +14066,7 @@
       </c>
       <c r="Q153" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description is for a Deputy Manager-Wind Engineering role, which involves working with wind energy projects, and the company ReNew is a renewable energy company, indicating a strong connection to clean energy and environmental sustainability</t>
+          <t>The job description is for a Deputy Manager-Wind Engineering role, which involves working with wind energy projects, and the company ReNew is a renewable energy company, indicating a strong connection to clean energy and environmental sustainability</t>
         </is>
       </c>
       <c r="R153" s="2" t="inlineStr">
@@ -14122,7 +14149,7 @@
       </c>
       <c r="O154" s="6" t="inlineStr">
         <is>
-          <t>Operation and maintenance of HT, LT Electrical System. Mechanical HVAC, Pump House, ETP, STP&amp; Shift team handling -Utility. Roles to Perform preventative maintenance on electrical &amp; mechanical systems and components by the team. Troubleshoot problems and make timely repairs. Plan, execute, and coordinate within the department. Tools requirement, spare management, and team management. Shift schedule, corrective actions, special activities planning. Calibration and testing of Electrical, Mechanica</t>
+          <t>Operation and maintenance of HT, LT Electrical System. Mechanical HVAC, Pump House, ETP, STP&amp; Shift team handling -Utility. Roles to Perform preventative maintenance on electrical &amp; mechanical systems and components by the team. Troubleshoot problems and make timely repairs. Plan, execute, and coordinate within the department. Tools requirement, spare management, and team management. Shift schedule, corrective actions, special activities planning. Calibration and testing of Electrical, Mechanical Equipment. Coordinate and plan with other dept. as their requirements. Maintain safety and adhere to all recommendations.</t>
         </is>
       </c>
       <c r="P154" s="6" t="inlineStr">
@@ -14132,7 +14159,7 @@
       </c>
       <c r="Q154" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions renewable energy, solar energy projects, and utility-scale wind energy projects, which are all related to clean energy. The company, ReNew, is also described as one of the largest renewable energy companies globally.</t>
+          <t>The job description mentions renewable energy, solar energy projects, and utility-scale wind energy projects, which are all related to clean energy. The company, ReNew, is also described as one of the largest renewable energy companies globally.</t>
         </is>
       </c>
       <c r="R154" s="2" t="inlineStr">
@@ -14215,7 +14242,7 @@
       </c>
       <c r="O155" s="6" t="inlineStr">
         <is>
-          <t>As Finance Lead – WEET, you will act as the key commercial and financial partner to Project Managers and operational leaders. Reporting to the CFO, this role is responsible for driving financial performance, strengthening project governance, and improving working capital outcomes across the service line. You will provide end-to-end project finance leadership across the full project lifecycle – from bid support and project set-up, through delivery and revenue recognition, to project close. Lead f</t>
+          <t>As Finance Lead – WEET, you will act as the key commercial and financial partner to Project Managers and operational leaders. Reporting to the CFO, this role is responsible for driving financial performance, strengthening project governance, and improving working capital outcomes across the service line. You will provide end-to-end project finance leadership across the full project lifecycle – from bid support and project set-up, through delivery and revenue recognition, to project close. Lead financial performance across the WEET portfolio, fostering accountability and a high-performing culture. Partner with Project Managers on project setup, forecasting, ETC, revenue recognition (PoC), invoicing and cash flow management. Deliver accurate monthly revenue recognition in collaboration with operational teams. Conduct risk reviews on projects with overruns, delays or margin erosion and recommend corrective actions. Drive working capital performance, including weekly cash flow forecasting and reporting to leadership. Own the budgeting and forecasting cycle, including resourcing analysis, backlog and pipeline projections through to P&amp;L and operational cash flow. Provide commercial input into bids and pricing models, balancing risk and return in collaboration with legal and operational stakeholders. Support ERP rollout activities including data cleansing, process mapping, UAT testing, training and adoption monitoring. Standardise financial and operational processes, aligning master data and reporting structures across the group. Act as the SME for ERP project accounting, coaching and educating Project Managers on governance and financial controls. Liaise with APAC Shared Services (tax, accounting, payables, receivables, payroll and FP&amp;A) to ensure accurate and compliant financial operations.</t>
         </is>
       </c>
       <c r="P155" s="6" t="inlineStr">
@@ -14225,7 +14252,7 @@
       </c>
       <c r="Q155" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[clean_energy_adjacent] The job title 'Finance Lead - Water, Environment &amp; Energy Transition' and the company's focus on sustainable solutions and infrastructure indicate a connection to environmental topics, specifically water, environment, and energy transition, which aligns with the clean energy </t>
+          <t>The job title 'Finance Lead - Water, Environment &amp; Energy Transition' and the company's focus on sustainable solutions and infrastructure indicate a connection to environmental topics, specifically water, environment, and energy transition, which aligns with the clean energy adjacent profile.</t>
         </is>
       </c>
       <c r="R155" s="2" t="inlineStr">
@@ -14308,17 +14335,17 @@
       </c>
       <c r="O156" s="6" t="inlineStr">
         <is>
-          <t>Assist the global strategic research team in providing quantitative analytics, and qualitative research to support our strategic research views on long term themes, and related communication material. Keep up-to-date on current investment trends and themes; help to identify and develop Mercer’s investment themes and opportunities. Drive the production side of our processes, for instance maintaining our theme summary material or quarterly thematic updates, project managing some of our material to</t>
+          <t>Assist the global strategic research team in providing quantitative analytics, and qualitative research to support our strategic research views on long term themes, and related communication material. Keep up-to-date on current investment trends and themes; help to identify and develop Mercer’s investment themes and opportunities. Drive the production side of our processes, for instance maintaining our theme summary material or quarterly thematic updates, project managing some of our material to final delivery. Build and maintain strong relationships with external parties such as specialist fund managers to explore investment ideas, develop research agendas. Work closely with other specialist teams, in particular our manager research boutiques, alternatives teams, sustainable investment team, delegated solutions and investment consulting colleagues to refine our team’s material, and to support intellectual capital development in respect of their specialist areas. Provide ad-hoc support to consultants in preparing thematic material for internal and external research meetings.</t>
         </is>
       </c>
       <c r="P156" s="6" t="inlineStr">
         <is>
-          <t>Strong researching and critical-thinking skills; ability to interpret and use qualitative and quantitative data to reach conclusions and explain them in terms that others can understand. Proven experience of research Investment knowledge: market awareness, asset class knowledge, asset allocation kno</t>
+          <t>Strong researching and critical-thinking skills; ability to interpret and use qualitative and quantitative data to reach conclusions and explain them in terms that others can understand. Proven experience of research Investment knowledge: market awareness, asset class knowledge, asset allocation knowledge, responsible investment, investment/risk tools (including MercerInsight and Datastream/Databank); eagerness to learn and keep up to date with the investment industry and market conditions. High proficiency in Excel. Creativity – a keenness to develop new processes and techniques, and an eye for design. Bloomberg and Factset trained (strongly preferred but not essential). Willingness to study IMC/CFA.</t>
         </is>
       </c>
       <c r="Q156" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'responsible investment' and 'sustainable investment team', indicating a focus on ESG investing and sustainable finance.</t>
+          <t>The job description mentions 'responsible investment' and 'sustainable investment team', indicating a focus on ESG investing and sustainable finance.</t>
         </is>
       </c>
       <c r="R156" s="2" t="inlineStr">
@@ -14401,17 +14428,17 @@
       </c>
       <c r="O157" s="6" t="inlineStr">
         <is>
-          <t>The position is within the Energy &amp; Infrastructure Vertical at ASSOCHAM, playing a pivotal role in advancing division’s advocacy and industry engagement agenda. The incumbent will lead high-impact policy advocacy and drive sector-focused initiatives spanning Energy, Power, Renewable Energy, Green Hydrogen, Transmission, Highways &amp; Tunnelling, and Civil Aviation. This role will act as a catalyst for transformative government initiatives, working closely with policymakers, industry leaders, and ke</t>
+          <t>The position is within the Energy &amp; Infrastructure Vertical at ASSOCHAM, playing a pivotal role in advancing division’s advocacy and industry engagement agenda. The incumbent will lead high-impact policy advocacy and drive sector-focused initiatives spanning Energy, Power, Renewable Energy, Green Hydrogen, Transmission, Highways &amp; Tunnelling, and Civil Aviation. This role will act as a catalyst for transformative government initiatives, working closely with policymakers, industry leaders, and key stakeholders to address critical sectoral challenges and unlock opportunities for sustainable and inclusive growth. In addition, the role carries a strong mandate for expanding industry membership, deepening stakeholder engagement, and driving revenue growth through innovative programs, conferences, partnerships, and strategic projects.</t>
         </is>
       </c>
       <c r="P157" s="6" t="inlineStr">
         <is>
-          <t>Policy &amp; Regulatory Understanding, Sectoral Knowledge, Research &amp; Analytical Skills, Government &amp; Institutional Liaison, Project &amp; Event Management, Membership &amp; Revenue Development, Communication &amp; Documentation, Stakeholder Management, Strategic Thinking, Communication &amp; Influence, Networking &amp; Re</t>
+          <t>Policy &amp; Regulatory Understanding, Sectoral Knowledge, Research &amp; Analytical Skills, Government &amp; Institutional Liaison, Project &amp; Event Management, Membership &amp; Revenue Development, Communication &amp; Documentation, Stakeholder Management, Strategic Thinking, Communication &amp; Influence, Networking &amp; Relationship Building, Commercial Orientation, Execution &amp; Ownership, Proficiency in MS Office Suite</t>
         </is>
       </c>
       <c r="Q157" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions renewable energy, green hydrogen, energy transition, and other related topics, which are relevant to the clean energy and environmental science fields.</t>
+          <t>The job description mentions renewable energy, green hydrogen, energy transition, and other related topics, which are relevant to the clean energy and environmental science fields.</t>
         </is>
       </c>
       <c r="R157" s="2" t="inlineStr">
@@ -14494,7 +14521,7 @@
       </c>
       <c r="O158" s="6" t="inlineStr">
         <is>
-          <t>Candidate shall be posted in general shift &amp; will have to make himself available as and when required in any critical condition to attain the site project work. He will be responsible to electrical work in project execution and completion till the commissioning. Working knowledge in Hindi, English language is essential. Computer literate with knowledge of MS Word, Excel, Power point, auto-cad. Installation, testing and commissioning of electrical equipment, cables as per standards and customer r</t>
+          <t>Candidate shall be posted in general shift &amp; will have to make himself available as and when required in any critical condition to attain the site project work. He will be responsible to electrical work in project execution and completion till the commissioning. Working knowledge in Hindi, English language is essential. Computer literate with knowledge of MS Word, Excel, Power point, auto-cad. Installation, testing and commissioning of electrical equipment, cables as per standards and customer requirements by preparing electrical systems specification, technical drawings. Establishing construction, manufacturing, or installation standards or specifications by performing a wide range of detailed calculations. Ensuring compliance with specifications, codes, or customer requirement by directing or coordinating installation, manufacturing, construction, maintenance, documentation, support, or testing activities. Writing reports and compiling data regarding existing and potential electrical engineering projects and studies. Supervising the ongoing project and providing training to O&amp;M team members. Estimating material, labor, or construction costs for budget preparation.</t>
         </is>
       </c>
       <c r="P158" s="6" t="inlineStr">
@@ -14504,7 +14531,7 @@
       </c>
       <c r="Q158" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions renewable energy, solar energy projects, and clean energy, which are all related to the clean energy adjacent profile. The company's mission to provide clean, safe, affordable, and sustainable energy also supports this classification.</t>
+          <t>The job description mentions renewable energy, solar energy projects, and clean energy, which are all related to the clean energy adjacent profile. The company's mission to provide clean, safe, affordable, and sustainable energy also supports this classification.</t>
         </is>
       </c>
       <c r="R158" s="2" t="inlineStr">
@@ -14591,7 +14618,7 @@
       </c>
       <c r="O159" s="6" t="inlineStr">
         <is>
-          <t>Lead and manage the full end-to-end lifecycle delivery of medium to highly complex regulatory change projects from initiation through implementation and closure. Define and manage the business case, project objectives, scope, resources and expected benefits for assigned initiatives. Act as the primary delivery owner ensuring alignment across stakeholders and teams across geographies. Develop and maintain high-quality project plans including risk mitigation strategies and structured work packages</t>
+          <t>Lead and manage the full end-to-end lifecycle delivery of medium to highly complex regulatory change projects from initiation through implementation and closure. Define and manage the business case, project objectives, scope, resources and expected benefits for assigned initiatives. Act as the primary delivery owner ensuring alignment across stakeholders and teams across geographies. Develop and maintain high-quality project plans including risk mitigation strategies and structured work packages. Evaluate delivery approaches, track performance and adjust plans to ensure alignment with scope, schedule, budget and project outcomes. Provide forecasts of future change and BAU resource requirements required to support project delivery.</t>
         </is>
       </c>
       <c r="P159" s="6" t="inlineStr">
@@ -14601,7 +14628,7 @@
       </c>
       <c r="Q159" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'sustainable investing' and 'SFDR' which are related to sustainable finance and ESG investing. The role involves leading regulatory change initiatives within the asset management domain, which also aligns with sustainable finance.</t>
+          <t>The job description mentions 'sustainable investing' and 'SFDR' which are related to sustainable finance and ESG investing. The role involves leading regulatory change initiatives within the asset management domain, which also aligns with sustainable finance.</t>
         </is>
       </c>
       <c r="R159" s="2" t="inlineStr">
@@ -14680,17 +14707,17 @@
       </c>
       <c r="O160" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lead Fundipedia implementation and enhancement projects to optimize fund data management. Define and enforce fund data governance frameworks, including pricing governance and quality controls. Own the fund master data strategy, ensuring accuracy, timeliness, and completeness across internal and external platforms. Drive automation, standardization, and scalability of data operations using Fundipedia and other tools. Act as escalation point for fund data discrepancies, reconciliation exceptions, </t>
+          <t>Lead Fundipedia implementation and enhancement projects to optimize fund data management. Define and enforce fund data governance frameworks, including pricing governance and quality controls. Own the fund master data strategy, ensuring accuracy, timeliness, and completeness across internal and external platforms. Drive automation, standardization, and scalability of data operations using Fundipedia and other tools. Act as escalation point for fund data discrepancies, reconciliation exceptions, and complex data-related queries. Collaborate with cross-functional teams including investments, compliance, distribution, client servicing, regulatory, vendor, and global teams. Represent Investment Operations in transformation programs and data governance forums. Monitor and report KPIs, delivering insights to improve fund data quality, operational efficiency, and service excellence. Mentor and guide team members on Fundipedia usage, data best practices, and continuous improvement. Implement assurance checks to ensure data meets investment, client reporting, and regulatory standards. Conduct data analysis to support business decisions and reporting needs. Oversee sustainability data integration and reporting across investment platforms. Ensure compliance with regulatory requirements and internal controls. Lead and manage the Data Services team, fostering innovation and continuous improvement.</t>
         </is>
       </c>
       <c r="P160" s="6" t="inlineStr">
         <is>
-          <t>Deep expertise in fund structures, share classes, and investment products. Hands-on experience with Fundipedia or similar EDM platforms. Strong understanding of regulatory frameworks (e.g., UCITS, MiFID II, SFDR). Proficiency in data tools (Excel, SQL, Power BI, Python, VBA). Excellent leadership, s</t>
+          <t>Deep expertise in fund structures, share classes, and investment products. Hands-on experience with Fundipedia or similar EDM platforms. Strong understanding of regulatory frameworks (e.g., UCITS, MiFID II, SFDR). Proficiency in data tools (Excel, SQL, Power BI, Python, VBA). Excellent leadership, stakeholder management, and communication skills. Analytical mindset with ability to interpret complex fund data. Proven ability to lead teams and manage cross-functional initiatives.</t>
         </is>
       </c>
       <c r="Q160" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions SFDR, which is a key regulation in sustainable finance, and also mentions overseeing sustainability data integration and reporting across investment platforms, indicating a focus on ESG considerations in investment operations.</t>
+          <t>The job description mentions SFDR, which is a key regulation in sustainable finance, and also mentions overseeing sustainability data integration and reporting across investment platforms, indicating a focus on ESG considerations in investment operations.</t>
         </is>
       </c>
       <c r="R160" s="2" t="inlineStr"/>
@@ -14765,17 +14792,17 @@
       </c>
       <c r="O161" s="6" t="inlineStr">
         <is>
-          <t>Work within a team responsible for Investment Restriction Compliance Management violation oversight, onboarding, and query resolution. Oversee daily reviews of overnight violation monitoring; escalate and track issues through to resolution. Partner with Investment Desks, Product, and Client Executives across asset classes on investment guideline matters and pre-trade violation overrides. Maintain broker and ready-to-trade coding in Aladdin and assist Trading Desks with related queries and escala</t>
+          <t>Work within a team responsible for Investment Restriction Compliance Management violation oversight, onboarding, and query resolution. Oversee daily reviews of overnight violation monitoring; escalate and track issues through to resolution. Partner with Investment Desks, Product, and Client Executives across asset classes on investment guideline matters and pre-trade violation overrides. Maintain broker and ready-to-trade coding in Aladdin and assist Trading Desks with related queries and escalations. Deliver and review mandate investment guideline onboarding and change activities, supporting control implementation on the Aladdin platform. Process and capture commitments sourced from IMAs, regulations, or internal teams. Collaborate with internal teams and vendors to ensure best practices and a consistent control environment. Respond to audit, regulator, and client queries, ensuring timely and accurate delivery of responses. Identify process gaps, troubleshoot issues, and communicate risks while proposing effective solutions. Participate in projects and working groups related to new markets, instruments, or mandates, assessing impacts on restrictions monitoring. Coach and mentor junior team members, ensuring training materials and procedures remain current.</t>
         </is>
       </c>
       <c r="P161" s="6" t="inlineStr">
         <is>
-          <t>Strong experience in Investment Restriction Monitoring and compliance processes within Asset Management. Hands-on experience with Aladdin (or equivalent portfolio management systems). Solid understanding of investment guidelines, regulatory compliance, and mandate restriction management. Proficiency</t>
+          <t>Strong experience in Investment Restriction Monitoring and compliance processes within Asset Management. Hands-on experience with Aladdin (or equivalent portfolio management systems). Solid understanding of investment guidelines, regulatory compliance, and mandate restriction management. Proficiency in Microsoft Excel; working knowledge of Word, PowerPoint, and SQL. Excellent communication and stakeholder management skills, with proven ability to collaborate across teams. Strong attention to detail and accuracy in reviewing documentation and compliance checks. Demonstrated ability to work under pressure and meet strict deadlines in a fast-paced environment. Proven leadership and mentoring skills, with the ability to support junior colleagues. Knowledge of investment restriction regulations such as UCITS, SFDR, and SDR. Prior involvement in change initiatives or process improvement projects. Experience working with regulatory audits or client visits. Exposure to risk assessment, policy setting, and control frameworks. Familiarity with broader investment products and asset classes. Understanding of data management and automation opportunities in control processes.</t>
         </is>
       </c>
       <c r="Q161" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions SFDR, which is a key regulation in sustainable finance, and also mentions investment restriction monitoring and compliance processes, which are relevant to ESG investing and sustainable finance.</t>
+          <t>The job description mentions SFDR, which is a key regulation in sustainable finance, and also mentions investment restriction monitoring and compliance processes, which are relevant to ESG investing and sustainable finance.</t>
         </is>
       </c>
       <c r="R161" s="2" t="inlineStr"/>
@@ -14850,17 +14877,17 @@
       </c>
       <c r="O162" s="6" t="inlineStr">
         <is>
-          <t>To lead the Fund Master function within Investment Data Services, ensuring high-quality, complete, and compliant fund data management using Fundipedia. This role is pivotal in driving data governance, reconciliation, and strategic data initiatives across investment operations. Lead Fundipedia implementation and enhancement projects to optimize fund data management. Define and enforce fund data governance frameworks, including pricing governance and quality controls. Own the fund master data stra</t>
+          <t>To lead the Fund Master function within Investment Data Services, ensuring high-quality, complete, and compliant fund data management using Fundipedia. This role is pivotal in driving data governance, reconciliation, and strategic data initiatives across investment operations. Lead Fundipedia implementation and enhancement projects to optimize fund data management. Define and enforce fund data governance frameworks, including pricing governance and quality controls. Own the fund master data strategy, ensuring accuracy, timeliness, and completeness across internal and external platforms. Drive automation, standardization, and scalability of data operations using Fundipedia and other tools. Act as escalation point for fund data discrepancies, reconciliation exceptions, and complex data-related queries. Collaborate with cross-functional teams including investments, compliance, distribution, client servicing, regulatory, vendor, and global teams. Represent Investment Operations in transformation programs and data governance forums. Monitor and report KPIs, delivering insights to improve fund data quality, operational efficiency, and service excellence. Mentor and guide team members on Fundipedia usage, data best practices, and continuous improvement. Implement assurance checks to ensure data meets investment, client reporting, and regulatory standards. Conduct data analysis to support business decisions and reporting needs. Oversee sustainability data integration and reporting across investment platforms. Ensure compliance with regulatory requirements and internal controls. Lead and manage the Data Services team, fostering innovation and continuous improvement.</t>
         </is>
       </c>
       <c r="P162" s="6" t="inlineStr">
         <is>
-          <t>Deep expertise in fund structures, share classes, and investment products. Hands-on experience with Fundipedia or similar EDM platforms. Strong understanding of regulatory frameworks (e.g., UCITS, MiFID II, SFDR). Proficiency in data tools (Excel, SQL, Power BI, Python, VBA). Excellent leadership, s</t>
+          <t>Deep expertise in fund structures, share classes, and investment products. Hands-on experience with Fundipedia or similar EDM platforms. Strong understanding of regulatory frameworks (e.g., UCITS, MiFID II, SFDR). Proficiency in data tools (Excel, SQL, Power BI, Python, VBA). Excellent leadership, stakeholder management, and communication skills. Analytical mindset with ability to interpret complex fund data. Proven ability to lead teams and manage cross-functional initiatives.</t>
         </is>
       </c>
       <c r="Q162" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions SFDR, which is a key regulation in sustainable finance, and also mentions overseeing sustainability data integration and reporting across investment platforms, indicating a focus on ESG considerations in investment operations.</t>
+          <t>The job description mentions SFDR, which is a key regulation in sustainable finance, and also mentions overseeing sustainability data integration and reporting across investment platforms, indicating a focus on ESG considerations in investment operations.</t>
         </is>
       </c>
       <c r="R162" s="2" t="inlineStr"/>
@@ -14927,7 +14954,7 @@
       </c>
       <c r="O163" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deliver assurance services to multinational clients across a variety of sectors. Support Project Managers in the independent verification of GHG/ESG information, sustainability‑linked financial instruments, and product‑level claims. Contribute to high‑quality assessments that uphold ERM CVS’s reputation as a trusted global verification body. Build strong capability in sustainability assurance standards, environmental data methodologies, and emerging regulatory frameworks across APAC. Strengthen </t>
+          <t>Deliver assurance services to multinational clients across a variety of sectors. Support Project Managers in the independent verification of GHG/ESG information, sustainability‑linked financial instruments, and product‑level claims. Contribute to high‑quality assessments that uphold ERM CVS’s reputation as a trusted global verification body. Build strong capability in sustainability assurance standards, environmental data methodologies, and emerging regulatory frameworks across APAC. Strengthen client relationships through clear communication, reliable delivery, and a commitment to quality. Support Project Managers in delivering independent assurance of GHG/ESG information, including sustainability reporting, sustainability‑linked financial instruments, product claims, and carbon market requirements. Execute assurance procedures under the supervision of senior colleagues, including: Media and desktop research, Analytical review of ESG and GHG data, Evidence collection and evaluation, Site visits, Disclosure assessments. Maintain complete and accurate documentation in accordance with assurance standards and internal quality systems. Assist senior colleagues during head office and operational site visits, contributing to fieldwork and client discussions. Work collaboratively across multiple projects to ensure timely, high‑quality deliverables.</t>
         </is>
       </c>
       <c r="P163" s="6" t="inlineStr">
@@ -14937,7 +14964,7 @@
       </c>
       <c r="Q163" s="6" t="inlineStr">
         <is>
-          <t>[general_esg] The job description mentions ESG, sustainability reporting, GHG disclosures, and climate action, which are all relevant to the general ESG profile. The role involves delivering assurance services to multinational clients, supporting project managers in independent verification of GHG/E</t>
+          <t>The job description mentions ESG, sustainability reporting, GHG disclosures, and climate action, which are all relevant to the general ESG profile. The role involves delivering assurance services to multinational clients, supporting project managers in independent verification of GHG/ESG information, and contributing to high-quality assessments that uphold ERM CVS’s reputation as a trusted global verification body.</t>
         </is>
       </c>
       <c r="R163" s="2" t="inlineStr"/>
@@ -15081,7 +15108,7 @@
       </c>
       <c r="O165" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lead the delivery of sustainability and decarbonisation initiatives across operations and projects, including development of Project Sustainability Scorecards, KPIs and reporting dashboards. Manage GHG emissions accounting and emissions data validation in accordance with NGER and internal governance requirements. Provide specialist sustainability support for bids, tenders and operational decision-making, imbedding sustainability rating schemes (e.g. ISC), decarbonisation KPIs and ESG principles </t>
+          <t>Lead the delivery of sustainability and decarbonisation initiatives across operations and projects, including development of Project Sustainability Scorecards, KPIs and reporting dashboards. Manage GHG emissions accounting and emissions data validation in accordance with NGER and internal governance requirements. Provide specialist sustainability support for bids, tenders and operational decision-making, imbedding sustainability rating schemes (e.g. ISC), decarbonisation KPIs and ESG principles into delivery. Drive sustainable procurement and Scope 3 emissions considerations, collaborating with procurement and supply chain teams. Support continuous improvement by monitoring emerging sustainability legislation, market trends, and client expectations.</t>
         </is>
       </c>
       <c r="P165" s="6" t="inlineStr">
@@ -15091,7 +15118,7 @@
       </c>
       <c r="Q165" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] The job description mentions climate-related initiatives, GHG emissions accounting, carbon modelling, and decarbonisation, which are all relevant to climate risk. The role also involves managing emissions data validation, sustainability reporting, and performance metrics, which are cr</t>
+          <t>The job description mentions climate-related initiatives, GHG emissions accounting, carbon modelling, and decarbonisation, which are all relevant to climate risk. The role also involves managing emissions data validation, sustainability reporting, and performance metrics, which are critical components of climate risk management.</t>
         </is>
       </c>
       <c r="R165" s="2" t="inlineStr"/>
@@ -15158,17 +15185,17 @@
       </c>
       <c r="O166" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">We are seeking dynamic, creative, and resourceful candidates for our Bengaluru, India location to work on challenging petrophysical problems in collaboration with a multidisciplinary team of formation evaluation specialists and operations geologists based in Houston, USA. You will conduct applied project work using well logs, core data, and well test data, leveraging a variety of software platforms for petrophysical data processing and interpretation. Define project objectives, work scopes, and </t>
+          <t>We are seeking dynamic, creative, and resourceful candidates for our Bengaluru, India location to work on challenging petrophysical problems in collaboration with a multidisciplinary team of formation evaluation specialists and operations geologists based in Houston, USA. You will conduct applied project work using well logs, core data, and well test data, leveraging a variety of software platforms for petrophysical data processing and interpretation. Define project objectives, work scopes, and deliverables in collaboration with ExxonMobil’s Formation Evaluation group in Houston and relevant Business Units. Contribute to all stages of petrophysical project work, including data preparation, preprocessing, filtering/augmentation, environmental corrections, calibration and interpretation. Provide real time operational support during drilling and completion activities, ensuring accurate and timely petrophysical interpretations to guide operational decisions. Conduct model based petrophysical analyses to evaluate reservoir properties and fluid distributions across the field lifecycle. Proactively develop new and innovative approaches to enhance the efficiency of multi well workflows. Collaborate with geologists, geophysicists, engineers, and other disciplines—as well as Business Units—to ensure accurate and integrated petrophysical interpretations across conventional, unconventional, and CCS reservoirs. Perform log QA/QC, rock physics modeling, fluid substitution to support seismic studies as needed. Work with computational scientists, engineers, and geoscientists to test, deliver, and support petrophysical software tools, models, algorithms, and workflows across multiple projects globally.</t>
         </is>
       </c>
       <c r="P166" s="6" t="inlineStr">
         <is>
-          <t>Excellent communication and teamwork skills, with the ability to collaborate effectively with multidisciplinary global teams and take ownership of deliverables. Hands on experience across various stages of the field lifecycle in conventional and unconventional reservoirs with operational support, ex</t>
+          <t>Excellent communication and teamwork skills, with the ability to collaborate effectively with multidisciplinary global teams and take ownership of deliverables. Hands on experience across various stages of the field lifecycle in conventional and unconventional reservoirs with operational support, experience in cased hole log interpretation, knowledge of advanced logging measurements and data acquisition is desirable. Strong analytical and problem solving skills with the ability to interpret complex datasets. Experience with one or more integrated petrophysical analysis software suites. Coding skills and knowledge of statistical methods, machine learning, or numerical modeling are an added advantage. Proficiency in English.</t>
         </is>
       </c>
       <c r="Q166" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions experience in renewable energy, low-carbon infrastructure, carbon markets, and natural capital, which are all relevant to the clean energy and environmental sectors.</t>
+          <t>The job description does not mention any ESG/sustainability topics, climate risk, sustainable finance, carbon markets, EU Taxonomy, or other related keywords. The company's vision to lead in energy innovations that advance modern living and a net-zero future is mentioned, but it is not directly related to the job responsibilities or requirements.</t>
         </is>
       </c>
       <c r="R166" s="2" t="inlineStr"/>
@@ -15490,17 +15517,17 @@
       </c>
       <c r="O170" s="6" t="inlineStr">
         <is>
-          <t>1) Product management - Continue to build XcelGreen with the technical know how of ESG SaaS, AI Agents and ESG Regulations understanding, continue the journey from 0-1. 2) ESG Consulting - Managing ESG consulting projects, developing sustainability strategies, delivering training sessions, and fostering strong client relationships. 3) Start-up Evangelist - Grow the start-up with lean resources and budget. We are looking for 2-3 people unicorn model with AI tools &amp; resources available. The ESG Co</t>
+          <t>1) Product management - Continue to build XcelGreen with the technical know how of ESG SaaS, AI Agents and ESG Regulations understanding, continue the journey from 0-1. 2) ESG Consulting - Managing ESG consulting projects, developing sustainability strategies, delivering training sessions, and fostering strong client relationships. 3) Start-up Evangelist - Grow the start-up with lean resources and budget. We are looking for 2-3 people unicorn model with AI tools &amp; resources available. The ESG Consulting Lead will also lead cross-functional teams and stay updated on industry trends and standards to provide best-in-class recommendations.</t>
         </is>
       </c>
       <c r="P170" s="6" t="inlineStr">
         <is>
-          <t>ESG SaaS, AI Agents, ESG Regulations, AI tools, Strong Analytical Skills, Excellent Communication skills, Proficiency in Training programs and workshops, Ability to lead and collaborate with cross-functional teams, Knowledge of ESG frameworks, global reporting standards, and regional compliance regu</t>
+          <t>ESG SaaS, AI Agents, ESG Regulations, AI tools, Strong Analytical Skills, Excellent Communication skills, Proficiency in Training programs and workshops, Ability to lead and collaborate with cross-functional teams, Knowledge of ESG frameworks, global reporting standards, and regional compliance regulations</t>
         </is>
       </c>
       <c r="Q170" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[general_esg] The job description mentions ESG strategy, ESG consulting, sustainability strategies, and ESG frameworks, which are all relevant to the general ESG profile. The role also involves working with ESG data, tracking carbon performance, and evaluating regulatory requirements, which further </t>
+          <t>The job description mentions ESG strategy, ESG consulting, sustainability strategies, and ESG frameworks, which are all relevant to the general ESG profile. The role also involves working with ESG data, tracking carbon performance, and evaluating regulatory requirements, which further supports this classification.</t>
         </is>
       </c>
       <c r="R170" s="2" t="inlineStr">
@@ -15587,7 +15614,7 @@
       </c>
       <c r="O171" s="6" t="inlineStr">
         <is>
-          <t>There are a variety of tasks and responsibilities you might be assigned however some common tasks that many of our graduate engineers perform include: * Assisting senior engineers with projects: You may be asked to help with research, testing, or other tasks related to ongoing projects. * Learning Wood processes and procedures: It's important to understand how Wood operates and the specific procedures and protocols you'll be expected to follow. * Collaborating with cross-functional teams: Engine</t>
+          <t>There are a variety of tasks and responsibilities you might be assigned however some common tasks that many of our graduate engineers perform include: * Assisting senior engineers with projects: You may be asked to help with research, testing, or other tasks related to ongoing projects. * Learning Wood processes and procedures: It's important to understand how Wood operates and the specific procedures and protocols you'll be expected to follow. * Collaborating with cross-functional teams: Engineering projects often involve multiple disciplines and teams, so you may need to work with colleagues from other areas of Wood. * Debugging and troubleshooting: If a product or system isn't working as intended, you may be called upon to help identify and resolve the problem. * Preparing reports and presentations: You may need to communicate your findings and progress to your team, manager, or other stakeholders. * Continuously improving your skills and knowledge: The engineering field is constantly evolving, so it's important to stay up to date with new developments and best practices.</t>
         </is>
       </c>
       <c r="P171" s="6" t="inlineStr">
@@ -15597,7 +15624,7 @@
       </c>
       <c r="Q171" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions 'renewables and emerging energy sectors' and 'decarbonisation, hydrogen, carbon capture and storage, renewables advisory', which are related to clean energy and environmental sustainability.</t>
+          <t>The job description mentions 'renewables and emerging energy sectors' and 'decarbonisation, hydrogen, carbon capture and storage, renewables advisory', which are related to clean energy and environmental sustainability.</t>
         </is>
       </c>
       <c r="R171" s="2" t="inlineStr">
@@ -15684,7 +15711,7 @@
       </c>
       <c r="O172" s="6" t="inlineStr">
         <is>
-          <t>The role is responsible for the development, innovation, and ongoing improvement of algorithms to optimize the trading of energy assets into the Australian National Electricity Market (NEM), with a particular focus on battery energy storage systems (BESS) and renewable assets. The role involves acting as a technical lead in an "agentic coding" environment, leveraging cutting-edge AI coding assistants to rapidly build, test, and deploy sophisticated mathematical forecasters, optimizers, and autom</t>
+          <t>The role is responsible for the development, innovation, and ongoing improvement of algorithms to optimize the trading of energy assets into the Australian National Electricity Market (NEM), with a particular focus on battery energy storage systems (BESS) and renewable assets. The role involves acting as a technical lead in an "agentic coding" environment, leveraging cutting-edge AI coding assistants to rapidly build, test, and deploy sophisticated mathematical forecasters, optimizers, and automated bidders. Client communication and marketing are critical aspects of this role, including acting as an evangelist for the technology and communicating algorithm and asset performance through various channels.</t>
         </is>
       </c>
       <c r="P172" s="6" t="inlineStr">
@@ -15694,7 +15721,7 @@
       </c>
       <c r="Q172" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions renewable energy, battery energy storage systems (BESS), and energy trading, which are all related to clean energy. The company also mentions climate goals and renewable energy integration, indicating a focus on environmental sustainability.</t>
+          <t>The job description mentions renewable energy, battery energy storage systems (BESS), and energy trading, which are all related to clean energy. The company also mentions climate goals and renewable energy integration, indicating a focus on environmental sustainability.</t>
         </is>
       </c>
       <c r="R172" s="2" t="inlineStr">
@@ -15878,7 +15905,7 @@
       </c>
       <c r="O174" s="6" t="inlineStr">
         <is>
-          <t>Own the technical design and evolution of Lendable’s data and analytics platform, collaborate closely with Lendable’s Senior Director of Analytics and Lendable’s CEO to define Lendable’s long-term data strategy and roadmap, drive AI adoption across Lendable, iterate and quickly prototype solutions for technology challenges, oversee Lendable’s strategy for identifying and quickly integrating new data sources, ensure that Lendable’s data is rational, well-structured, labeled, standardized, and ult</t>
+          <t>Own the technical design and evolution of Lendable’s data and analytics platform, collaborate closely with Lendable’s Senior Director of Analytics and Lendable’s CEO to define Lendable’s long-term data strategy and roadmap, drive AI adoption across Lendable, iterate and quickly prototype solutions for technology challenges, oversee Lendable’s strategy for identifying and quickly integrating new data sources, ensure that Lendable’s data is rational, well-structured, labeled, standardized, and ultimately understandable, establish the systems, controls, and accountability structures that guarantee the accuracy, speed, and trustworthiness of all data used across Lendable, manage a team and oversee the processes and systems to ensure that Lendable’s integrations with borrower systems are accurate, resilient, and continuously verified.</t>
         </is>
       </c>
       <c r="P174" s="6" t="inlineStr">
@@ -15888,7 +15915,7 @@
       </c>
       <c r="Q174" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions 'responsible investment' and 'sustainable investment team', indicating a focus on ESG investing and sustainable finance.</t>
+          <t>The job description does not explicitly mention ESG, sustainability, or environmental topics, and the focus is on data strategy, architecture, and governance in a financial services context.</t>
         </is>
       </c>
       <c r="R174" s="2" t="inlineStr">
@@ -15969,7 +15996,7 @@
       </c>
       <c r="Q175" s="6" t="inlineStr">
         <is>
-          <t>[climate_risk] Job title contains 'Climate', indicating a strong focus on climate-related work</t>
+          <t>Job title contains 'Climate', indicating a strong focus on climate-related work</t>
         </is>
       </c>
       <c r="R175" s="2" t="inlineStr"/>
@@ -16053,7 +16080,9 @@
 * Facilitating transactions in line with both client and Amsterdam Renewable Markets' standards. 
 * Striving to meet and exceed annual sales targets, ensuring sustained growth. 
 * Engaging in trading activities involving renewable power certificates, carbon offsets, among others. 
-* Daily interactions with team clients, expertly m</t>
+* Daily interactions with team clients, expertly managing existing portfolios while simultaneously expanding the client base. 
+* Continuously monitoring environmental commodities market shifts and proactively aiding Amsterdam Renewable Markets' growth. 
+* Innovating commodity deal structures that satisfy both client and company objectives.</t>
         </is>
       </c>
       <c r="P176" s="6" t="inlineStr">
@@ -16063,7 +16092,7 @@
       </c>
       <c r="Q176" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions environmental commodities, renewable energy markets, carbon offsets, and reducing carbon footprints, which are all related to clean energy and environmental sustainability.</t>
+          <t>The job description mentions environmental commodities, renewable energy markets, carbon offsets, and reducing carbon footprints, which are all related to clean energy and environmental sustainability.</t>
         </is>
       </c>
       <c r="R176" s="2" t="inlineStr">
@@ -16146,7 +16175,7 @@
       </c>
       <c r="O177" s="6" t="inlineStr">
         <is>
-          <t>You will support the New Market Certification team with general project work and tasks, including revision of PCFs, preparing presentation and reports, general research tasks, research of emission factors and development of Excel-based PCF calculations. You will support research activities for different areas related to sustainability certifications and PCFs, including topics such as, biogenic materials and renewable energy. You will support the team in preparing presentations and slides for tra</t>
+          <t>You will support the New Market Certification team with general project work and tasks, including revision of PCFs, preparing presentation and reports, general research tasks, research of emission factors and development of Excel-based PCF calculations. You will support research activities for different areas related to sustainability certifications and PCFs, including topics such as, biogenic materials and renewable energy. You will support the team in preparing presentations and slides for trainings or customer communications. You will support the team in communication with different internal and external stakeholders.</t>
         </is>
       </c>
       <c r="P177" s="6" t="inlineStr">
@@ -16156,7 +16185,7 @@
       </c>
       <c r="Q177" s="6" t="inlineStr">
         <is>
-          <t>[carbon_markets] The job description mentions carbon footprint certification, product carbon footprints, life cycle assessment, and sustainability certification, which are all related to carbon markets and emissions trading.</t>
+          <t>The job description mentions carbon footprint certification, product carbon footprints, life cycle assessment, and sustainability certification, which are all related to carbon markets and emissions trading.</t>
         </is>
       </c>
       <c r="R177" s="2" t="inlineStr">
@@ -16243,7 +16272,7 @@
       </c>
       <c r="O178" s="6" t="inlineStr">
         <is>
-          <t>Be willing to be a pioneer and have an interest in ESG &amp; Corporate Governance. Curiosity and passion for researching and highlighting recent trends in sustainability (environmental and social issues), business ethics, regulations and sustainable development goals. Use analytical tools and intellect to question, challenge and evaluate current practices in the evolving area of ESG. Highlight key sustainability / ESG issues that are material to an industry / company. Prepare sector research reports</t>
+          <t>Be willing to be a pioneer and have an interest in ESG &amp; Corporate Governance. Curiosity and passion for researching and highlighting recent trends in sustainability (environmental and social issues), business ethics, regulations and sustainable development goals. Use analytical tools and intellect to question, challenge and evaluate current practices in the evolving area of ESG. Highlight key sustainability / ESG issues that are material to an industry / company. Prepare sector research reports and rank companies based on their sustainability disclosures, performance and qualitative factors. Travel to meet with the company management to understand the company s overall sustainability strategy and progress. Able to vote for proxy voting for all the resolutions for portfolio companies. Prepare database of Proxy Voting, Stewardship Code, SFDR</t>
         </is>
       </c>
       <c r="P178" s="6" t="inlineStr">
@@ -16253,7 +16282,7 @@
       </c>
       <c r="Q178" s="6" t="inlineStr">
         <is>
-          <t>[sustainable_finance] The job description mentions ESG research, sustainability disclosures, performance, and qualitative factors, which are key aspects of sustainable finance. Additionally, the mention of SFDR (Sustainable Finance Disclosure Regulation) further supports this classification.</t>
+          <t>The job description mentions ESG research, sustainability disclosures, performance, and qualitative factors, which are key aspects of sustainable finance. Additionally, the mention of SFDR (Sustainable Finance Disclosure Regulation) further supports this classification.</t>
         </is>
       </c>
       <c r="R178" s="2" t="inlineStr">
@@ -16336,17 +16365,17 @@
       </c>
       <c r="O179" s="6" t="inlineStr">
         <is>
-          <t>Within our Energy Advisory capability, we advise clients on the challenges and opportunities regarding decarbonisation/net zero issues specifically in relation to requirements for delivering the global energy transition. This includes decentralised low carbon generation, innovation in technologies and energy sources, as well as policy and regulatory support. The successful applicant shall also have strong knowledge of the broader water industry in terms of growth and challenges to decarbonisatio</t>
+          <t>Within our Energy Advisory capability, we advise clients on the challenges and opportunities regarding decarbonisation/net zero issues specifically in relation to requirements for delivering the global energy transition. This includes decentralised low carbon generation, innovation in technologies and energy sources, as well as policy and regulatory support. The successful applicant shall also have strong knowledge of the broader water industry in terms of growth and challenges to decarbonisation, with knowledge on how to support our clients in developing decarbonisation strategies and business case assessment applying energy resources and demands, with a drive to also build-up the water network in the Energy Advisory team. Key Responsibilities Include: Lead technical delivery and being accountable for key tasks and quality data outputs through project reviewer role, Engaging with a range of stakeholders at all levels, Maintaining knowledge of energy/carbon policy developments, energy markets and wider energy/sustainability issues, Key inputs with respect to energy in the development or review of engineering design through-out project life-cycle, Energy technology options or energy efficiency appraisals and life cycle cost analysis, Energy management, energy efficiency, asset reviews and audit surveys, energy demand modelling and preparing low carbon energy solutions that are either led by reconfiguring existing operations at sites or developing new strategies, Mentoring and training colleagues in aspects of the water and energy sectors.</t>
         </is>
       </c>
       <c r="P179" s="6" t="inlineStr">
         <is>
-          <t>Strong verbal and written communication skills, excellent quantitative and problem-solving skills, ability to lead bid preparation, deliver to tight timescales, be technically accurate and to manage a number of schemes simultaneously, Strong project management skills, Knowledge of current and antici</t>
+          <t>Strong verbal and written communication skills, excellent quantitative and problem-solving skills, ability to lead bid preparation, deliver to tight timescales, be technically accurate and to manage a number of schemes simultaneously, Strong project management skills, Knowledge of current and anticipated environmental, carbon and energy policy and legislation, Ability to develop standard engineering deliverables such as heat and mass balances</t>
         </is>
       </c>
       <c r="Q179" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] The job description mentions decarbonisation, net zero, low carbon generation, energy efficiency, and energy transition, which are all relevant to the clean energy adjacent profile. Additionally, the job requires experience working on water sector energy projects and knowledg</t>
+          <t>The job description mentions decarbonisation, net zero, low carbon generation, energy efficiency, and energy transition, which are all relevant to the clean energy adjacent profile. Additionally, the job requires experience working on water sector energy projects and knowledge of the broader water industry in terms of growth and challenges to decarbonisation.</t>
         </is>
       </c>
       <c r="R179" s="2" t="inlineStr">
@@ -16427,7 +16456,7 @@
       </c>
       <c r="Q180" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] Job title contains 'Renewables', indicating a connection to renewable energy</t>
+          <t>Job title contains 'Renewables', indicating a connection to renewable energy</t>
         </is>
       </c>
       <c r="R180" s="2" t="inlineStr"/>
@@ -16504,7 +16533,7 @@
       </c>
       <c r="Q181" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] Job title contains 'Circular Bioeconomy', indicating a focus on environmental science and circular economy, which aligns with the clean energy adjacent profile.</t>
+          <t>Job title contains 'Circular Bioeconomy', indicating a focus on environmental science and circular economy, which aligns with the clean energy adjacent profile.</t>
         </is>
       </c>
       <c r="R181" s="2" t="inlineStr"/>
@@ -16581,7 +16610,7 @@
       </c>
       <c r="Q182" s="6" t="inlineStr">
         <is>
-          <t>[clean_energy_adjacent] Job title contains 'Wind', indicating a focus on renewable energy</t>
+          <t>Job title contains 'Wind', indicating a focus on renewable energy</t>
         </is>
       </c>
       <c r="R182" s="2" t="inlineStr"/>

</xml_diff>